<commit_message>
Packages Advisor/Sprinter/Priority, pricing note, titles
</commit_message>
<xml_diff>
--- a/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
+++ b/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
@@ -3683,17 +3683,17 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Clients who stopped guessing</t>
+          <t>Tangible results</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>კლიენტები, რომლებმაც ვარაუდი სისტემით ჩაანაცვლეს</t>
+          <t>ხელშესახები შედეგები</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Клиенты, которые перестали гадать</t>
+          <t>Ощутимые результаты</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="H77" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -4079,17 +4079,17 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>20 minutes closes every question</t>
+          <t>20 minutes to save 30+ hours</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>20 წუთი ყველა კითხვას პასუხს გაგცემს</t>
+          <t>20 წუთი, 30+ საათის დასაზოგად</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>20 минут закрывают любой вопрос</t>
+          <t>20 минут, чтобы сэкономить 30+ часов</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -5730,7 +5730,7 @@
           <t>Цены</t>
         </is>
       </c>
-      <c r="G126" s="3" t="inlineStr"/>
+      <c r="G126" s="3" t="n"/>
       <c r="H126" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -5768,7 +5768,7 @@
           <t>Три модели сотрудничества</t>
         </is>
       </c>
-      <c r="G127" s="3" t="inlineStr"/>
+      <c r="G127" s="3" t="n"/>
       <c r="H127" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -5806,7 +5806,7 @@
           <t>В зависимости от того, сколько нашего ресурса вам нужно, мы предлагаем три модели сотрудничества. Выберите самую удобную.</t>
         </is>
       </c>
-      <c r="G128" s="3" t="inlineStr"/>
+      <c r="G128" s="3" t="n"/>
       <c r="H128" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -5831,23 +5831,23 @@
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>Already have a system?</t>
+          <t>We share our tools and experience</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>უკვე გაქვს სისტემა?</t>
+          <t>გიზიარებთ ინსტრუმენტებს და გამოცდილებას</t>
         </is>
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>Уже есть система?</t>
-        </is>
-      </c>
-      <c r="G129" s="3" t="inlineStr"/>
+          <t>Делимся инструментами и опытом</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="n"/>
       <c r="H129" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -5869,23 +5869,23 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>STARTER</t>
+          <t>ADVISOR</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>STARTER</t>
+          <t>ADVISOR</t>
         </is>
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>STARTER</t>
-        </is>
-      </c>
-      <c r="G130" s="3" t="inlineStr"/>
+          <t>ADVISOR</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="n"/>
       <c r="H130" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -5920,7 +5920,7 @@
           <t>1-2 конкретных решения из нашего каталога, внедрённых в вашу систему. Быстро, точно, без переделки.</t>
         </is>
       </c>
-      <c r="G131" s="3" t="inlineStr"/>
+      <c r="G131" s="3" t="n"/>
       <c r="H131" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -5945,23 +5945,23 @@
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>€990-1,490</t>
+          <t>€990+</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>€990-1,490</t>
+          <t>€990+</t>
         </is>
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>€990-1,490</t>
-        </is>
-      </c>
-      <c r="G132" s="3" t="inlineStr"/>
+          <t>€990+</t>
+        </is>
+      </c>
+      <c r="G132" s="3" t="n"/>
       <c r="H132" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
           <t>+ НДС · разово</t>
         </is>
       </c>
-      <c r="G133" s="3" t="inlineStr"/>
+      <c r="G133" s="3" t="n"/>
       <c r="H133" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6021,23 +6021,23 @@
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>3-5 working days</t>
+          <t>3+ working days</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
-          <t>3-5 სამუშაო დღე</t>
+          <t>3+ სამუშაო დღე</t>
         </is>
       </c>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>3-5 рабочих дней</t>
-        </is>
-      </c>
-      <c r="G134" s="3" t="inlineStr"/>
+          <t>3+ рабочих дня</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="n"/>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6072,7 @@
           <t>1-2 решения из каталога</t>
         </is>
       </c>
-      <c r="G135" s="3" t="inlineStr"/>
+      <c r="G135" s="3" t="n"/>
       <c r="H135" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6110,7 +6110,7 @@
           <t>Интеграция в существующую систему</t>
         </is>
       </c>
-      <c r="G136" s="3" t="inlineStr"/>
+      <c r="G136" s="3" t="n"/>
       <c r="H136" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6148,7 +6148,7 @@
           <t>30-минутное обучение команды</t>
         </is>
       </c>
-      <c r="G137" s="3" t="inlineStr"/>
+      <c r="G137" s="3" t="n"/>
       <c r="H137" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6173,23 +6173,23 @@
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>14-day post-launch support</t>
+          <t>Consulting sessions</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>14-დღიანი დანერგვის შემდგომი მხარდაჭერა</t>
+          <t>საკონსულტაციო შეხვედრები</t>
         </is>
       </c>
       <c r="F138" s="3" t="inlineStr">
         <is>
-          <t>14-дневная поддержка после запуска</t>
-        </is>
-      </c>
-      <c r="G138" s="3" t="inlineStr"/>
+          <t>Консультационные встречи</t>
+        </is>
+      </c>
+      <c r="G138" s="3" t="n"/>
       <c r="H138" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6211,23 +6211,23 @@
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>Request Starter</t>
+          <t>Request Advisor</t>
         </is>
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე Starter</t>
+          <t>მოითხოვე Advisor</t>
         </is>
       </c>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>Запросить Starter</t>
-        </is>
-      </c>
-      <c r="G139" s="3" t="inlineStr"/>
+          <t>Запросить Advisor</t>
+        </is>
+      </c>
+      <c r="G139" s="3" t="n"/>
       <c r="H139" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6262,7 +6262,7 @@
           <t>⭐ Самый популярный</t>
         </is>
       </c>
-      <c r="G140" s="3" t="inlineStr"/>
+      <c r="G140" s="3" t="n"/>
       <c r="H140" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6287,23 +6287,23 @@
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>Build it right, from scratch</t>
+          <t>We help you implement step by step</t>
         </is>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>ააშენე სწორად, თავიდან</t>
+          <t>გეხმარებით ეტაპობრივად დანერგვაში</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>Построить правильно, с нуля</t>
-        </is>
-      </c>
-      <c r="G141" s="3" t="inlineStr"/>
+          <t>Помогаем внедрять поэтапно</t>
+        </is>
+      </c>
+      <c r="G141" s="3" t="n"/>
       <c r="H141" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6325,23 +6325,23 @@
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>SPRINT</t>
+          <t>SPRINTER</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>SPRINT</t>
+          <t>SPRINTER</t>
         </is>
       </c>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>SPRINT</t>
-        </is>
-      </c>
-      <c r="G142" s="3" t="inlineStr"/>
+          <t>SPRINTER</t>
+        </is>
+      </c>
+      <c r="G142" s="3" t="n"/>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6376,7 +6376,7 @@
           <t>Построение полной системы или решение главной боли. За 2 недели, команда обучена, всё ваше.</t>
         </is>
       </c>
-      <c r="G143" s="3" t="inlineStr"/>
+      <c r="G143" s="3" t="n"/>
       <c r="H143" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6414,7 +6414,7 @@
           <t>€2,990</t>
         </is>
       </c>
-      <c r="G144" s="3" t="inlineStr"/>
+      <c r="G144" s="3" t="n"/>
       <c r="H144" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6452,7 +6452,7 @@
           <t>+ НДС · разово</t>
         </is>
       </c>
-      <c r="G145" s="3" t="inlineStr"/>
+      <c r="G145" s="3" t="n"/>
       <c r="H145" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6490,7 +6490,7 @@
           <t>10-15 рабочих дней</t>
         </is>
       </c>
-      <c r="G146" s="3" t="inlineStr"/>
+      <c r="G146" s="3" t="n"/>
       <c r="H146" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6528,7 +6528,7 @@
           <t>Полный спринт Data Foundation или Sharpest Pain</t>
         </is>
       </c>
-      <c r="G147" s="3" t="inlineStr"/>
+      <c r="G147" s="3" t="n"/>
       <c r="H147" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6566,7 +6566,7 @@
           <t>До 6 решений из каталога</t>
         </is>
       </c>
-      <c r="G148" s="3" t="inlineStr"/>
+      <c r="G148" s="3" t="n"/>
       <c r="H148" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6604,7 +6604,7 @@
           <t>Автоматизация + 1 интеграция</t>
         </is>
       </c>
-      <c r="G149" s="3" t="inlineStr"/>
+      <c r="G149" s="3" t="n"/>
       <c r="H149" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6642,7 +6642,7 @@
           <t>Миграция данных (1 источник)</t>
         </is>
       </c>
-      <c r="G150" s="3" t="inlineStr"/>
+      <c r="G150" s="3" t="n"/>
       <c r="H150" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6680,7 +6680,7 @@
           <t>1-часовое обучение команды</t>
         </is>
       </c>
-      <c r="G151" s="3" t="inlineStr"/>
+      <c r="G151" s="3" t="n"/>
       <c r="H151" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6700,28 +6700,28 @@
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>pricing.2.feature.6</t>
+          <t>pricing.2.cta</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>30-day post-launch tuning</t>
+          <t>Request Sprinter</t>
         </is>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>30-დღიანი დანერგვის შემდგომი დახვეწა</t>
+          <t>მოითხოვე Sprinter</t>
         </is>
       </c>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>30-дневная настройка после запуска</t>
-        </is>
-      </c>
-      <c r="G152" s="3" t="inlineStr"/>
+          <t>Запросить Sprinter</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="n"/>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6738,28 +6738,28 @@
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>pricing.2.cta</t>
+          <t>pricing.3.tag</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
         <is>
-          <t>Request Sprint</t>
+          <t>We keep your growth moving, continuously</t>
         </is>
       </c>
       <c r="E153" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე Sprint</t>
+          <t>მუდმივად ვზრუნავთ განვითარებაზე</t>
         </is>
       </c>
       <c r="F153" s="3" t="inlineStr">
         <is>
-          <t>Запросить Sprint</t>
-        </is>
-      </c>
-      <c r="G153" s="3" t="inlineStr"/>
+          <t>Постоянно заботимся о развитии</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="n"/>
       <c r="H153" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6776,28 +6776,28 @@
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.tag</t>
+          <t>pricing.3.name</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Need a digital team on tap?</t>
+          <t>PRIORITY</t>
         </is>
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
-          <t>ციფრული გუნდი მუდმივად გჭირდება?</t>
+          <t>PRIORITY</t>
         </is>
       </c>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>Нужна цифровая команда на связи?</t>
-        </is>
-      </c>
-      <c r="G154" s="3" t="inlineStr"/>
+          <t>PRIORITY</t>
+        </is>
+      </c>
+      <c r="G154" s="3" t="n"/>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6814,25 +6814,25 @@
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.name</t>
+          <t>pricing.3.pitch</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
         <is>
-          <t>PARTNERSHIP</t>
+          <t>Multi-sprint build + ongoing managed services. Priority queue, direct line to our CEO + Tech Lead.</t>
         </is>
       </c>
       <c r="E155" s="3" t="inlineStr">
         <is>
-          <t>PARTNERSHIP</t>
+          <t>მრავალ-სპრინტიანი აწყობა + მუდმივი managed services. პრიორიტეტული რიგი, პირდაპირი კავშირი CEO-სთან და Tech Lead-სთან.</t>
         </is>
       </c>
       <c r="F155" s="3" t="inlineStr">
         <is>
-          <t>PARTNERSHIP</t>
-        </is>
-      </c>
-      <c r="G155" s="3" t="inlineStr"/>
+          <t>Многоспринтовое построение + постоянные managed services. Приоритетная очередь, прямая связь с CEO и Tech Lead.</t>
+        </is>
+      </c>
+      <c r="G155" s="3" t="n"/>
       <c r="H155" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6852,25 +6852,25 @@
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.pitch</t>
+          <t>pricing.3.price</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Multi-sprint build + ongoing managed services. Priority queue, direct line to our CEO + Tech Lead.</t>
+          <t>€7,990 + €790/mo</t>
         </is>
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
-          <t>მრავალ-სპრინტიანი აწყობა + მუდმივი managed services. პრიორიტეტული რიგი, პირდაპირი კავშირი CEO-სთან და Tech Lead-სთან.</t>
+          <t>€7,990 + €790/თვე</t>
         </is>
       </c>
       <c r="F156" s="3" t="inlineStr">
         <is>
-          <t>Многоспринтовое построение + постоянные managed services. Приоритетная очередь, прямая связь с CEO и Tech Lead.</t>
-        </is>
-      </c>
-      <c r="G156" s="3" t="inlineStr"/>
+          <t>€7,990 + €790/мес</t>
+        </is>
+      </c>
+      <c r="G156" s="3" t="n"/>
       <c r="H156" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6890,25 +6890,25 @@
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.price</t>
+          <t>pricing.3.priceUnit</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
         <is>
-          <t>€7,990 + €790/mo</t>
+          <t>+ VAT · 6-month minimum</t>
         </is>
       </c>
       <c r="E157" s="3" t="inlineStr">
         <is>
-          <t>€7,990 + €790/თვე</t>
+          <t>+ დღგ · 6 თვე მინ.</t>
         </is>
       </c>
       <c r="F157" s="3" t="inlineStr">
         <is>
-          <t>€7,990 + €790/мес</t>
-        </is>
-      </c>
-      <c r="G157" s="3" t="inlineStr"/>
+          <t>+ НДС · минимум 6 месяцев</t>
+        </is>
+      </c>
+      <c r="G157" s="3" t="n"/>
       <c r="H157" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6928,25 +6928,25 @@
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.priceUnit</t>
+          <t>pricing.3.timeline</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>+ VAT · 6-month minimum</t>
+          <t>90-day engagement</t>
         </is>
       </c>
       <c r="E158" s="3" t="inlineStr">
         <is>
-          <t>+ დღგ · 6 თვე მინ.</t>
+          <t>90-დღიანი ჩართულობა</t>
         </is>
       </c>
       <c r="F158" s="3" t="inlineStr">
         <is>
-          <t>+ НДС · минимум 6 месяцев</t>
-        </is>
-      </c>
-      <c r="G158" s="3" t="inlineStr"/>
+          <t>90-дневное взаимодействие</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="n"/>
       <c r="H158" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -6966,28 +6966,28 @@
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.timeline</t>
+          <t>pricing.3.feature.1</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
         <is>
-          <t>90-day engagement</t>
+          <t>Everything included in Sprinter</t>
         </is>
       </c>
       <c r="E159" s="3" t="inlineStr">
         <is>
-          <t>90-დღიანი ჩართულობა</t>
+          <t>ყველაფერი, რასაც Sprinter მოიცავს</t>
         </is>
       </c>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>90-дневное взаимодействие</t>
-        </is>
-      </c>
-      <c r="G159" s="3" t="inlineStr"/>
+          <t>Всё, что входит в Sprinter</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="n"/>
       <c r="H159" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -7004,25 +7004,25 @@
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.feature.1</t>
+          <t>pricing.3.feature.2</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Sprint 1 + Sprint 2 pre-planned</t>
+          <t>Priority dev queue</t>
         </is>
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
-          <t>Sprint 1 + Sprint 2 წინასწარ ჩაგეგმილი</t>
+          <t>პრიორიტეტული dev-ის რიგი</t>
         </is>
       </c>
       <c r="F160" s="3" t="inlineStr">
         <is>
-          <t>Спринт 1 + Спринт 2 запланированы</t>
-        </is>
-      </c>
-      <c r="G160" s="3" t="inlineStr"/>
+          <t>Приоритетная очередь разработки</t>
+        </is>
+      </c>
+      <c r="G160" s="3" t="n"/>
       <c r="H160" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7042,28 +7042,28 @@
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.feature.2</t>
+          <t>pricing.3.feature.3</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
         <is>
-          <t>Priority dev queue</t>
+          <t>A dedicated specialist from our team</t>
         </is>
       </c>
       <c r="E161" s="3" t="inlineStr">
         <is>
-          <t>პრიორიტეტული dev-ის რიგი</t>
+          <t>გამოყოფილი სპეციალისტი გუნდიდან</t>
         </is>
       </c>
       <c r="F161" s="3" t="inlineStr">
         <is>
-          <t>Приоритетная очередь разработки</t>
-        </is>
-      </c>
-      <c r="G161" s="3" t="inlineStr"/>
+          <t>Выделенный специалист из команды</t>
+        </is>
+      </c>
+      <c r="G161" s="3" t="n"/>
       <c r="H161" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -7080,25 +7080,25 @@
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.feature.3</t>
+          <t>pricing.3.feature.4</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Direct WhatsApp with CEO + Tech Lead</t>
+          <t>Managed services (ongoing optimization)</t>
         </is>
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
-          <t>პირდაპირი WhatsApp CEO-სთან + Tech Lead-სთან</t>
+          <t>Managed services (მუდმივი ოპტიმიზაცია)</t>
         </is>
       </c>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>Прямой WhatsApp с CEO + Tech Lead</t>
-        </is>
-      </c>
-      <c r="G162" s="3" t="inlineStr"/>
+          <t>Managed services (постоянная оптимизация)</t>
+        </is>
+      </c>
+      <c r="G162" s="3" t="n"/>
       <c r="H162" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7118,25 +7118,25 @@
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.feature.4</t>
+          <t>pricing.3.feature.5</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
         <is>
-          <t>Managed services (ongoing optimization)</t>
+          <t>Monthly strategy review (CEO level)</t>
         </is>
       </c>
       <c r="E163" s="3" t="inlineStr">
         <is>
-          <t>Managed services (მუდმივი ოპტიმიზაცია)</t>
+          <t>თვიური სტრატეგიული შეხვედრა (CEO)</t>
         </is>
       </c>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>Managed services (постоянная оптимизация)</t>
-        </is>
-      </c>
-      <c r="G163" s="3" t="inlineStr"/>
+          <t>Ежемесячная стратегическая встреча (CEO)</t>
+        </is>
+      </c>
+      <c r="G163" s="3" t="n"/>
       <c r="H163" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7156,28 +7156,28 @@
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.feature.5</t>
+          <t>pricing.3.cta</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Monthly strategy review (CEO level)</t>
+          <t>Request Priority</t>
         </is>
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>თვიური სტრატეგიული შეხვედრა (CEO)</t>
+          <t>მოითხოვე Priority</t>
         </is>
       </c>
       <c r="F164" s="3" t="inlineStr">
         <is>
-          <t>Ежемесячная стратегическая встреча (CEO)</t>
-        </is>
-      </c>
-      <c r="G164" s="3" t="inlineStr"/>
+          <t>Запросить Priority</t>
+        </is>
+      </c>
+      <c r="G164" s="3" t="n"/>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -7194,28 +7194,28 @@
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>pricing.3.cta</t>
+          <t>pricing.blueprint.title</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Request Partnership</t>
+          <t>Need more flexibility? Use our resource - by the hour</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე Partnership</t>
+          <t>მეტი მოქნილობა გჭირდება? გამოიყენე ჩვენი რესურსი - საათობრივად</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Запросить Partnership</t>
-        </is>
-      </c>
-      <c r="G165" s="3" t="inlineStr"/>
+          <t>Нужно больше гибкости? Используйте наш ресурс - почасово</t>
+        </is>
+      </c>
+      <c r="G165" s="3" t="n"/>
       <c r="H165" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -7232,25 +7232,25 @@
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>pricing.blueprint.title</t>
+          <t>pricing.blueprint.body</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
         <is>
-          <t>Need help with your existing system?</t>
+          <t>Order technical and expert support by the hour. Our team helps with implementation, know-how, and years of experience - exactly when you need it. €69/h + VAT, no minimum commitment.</t>
         </is>
       </c>
       <c r="E166" s="3" t="inlineStr">
         <is>
-          <t>გჭირდება მხარდაჭერა შენი არსებული სისტემისთვის?</t>
+          <t>შეუკვეთე ტექნიკური და საექსპერტო მხარდაჭერა საათობრივად. ჩვენი გუნდი დაგეხმარება ტექნიკური დანერგვით, ცოდნითა და წლების გამოცდილებით - ზუსტად მაშინ, როცა გჭირდება. €69/სთ + დღგ, არანაირი მინიმალური ვალდებულება.</t>
         </is>
       </c>
       <c r="F166" s="3" t="inlineStr">
         <is>
-          <t>Нужна поддержка существующей системы?</t>
-        </is>
-      </c>
-      <c r="G166" s="3" t="inlineStr"/>
+          <t>Закажите техническую и экспертную поддержку почасово. Наша команда поможет с технической реализацией, знаниями и многолетним опытом - именно тогда, когда это нужно. €69/ч + НДС, без минимальных обязательств.</t>
+        </is>
+      </c>
+      <c r="G166" s="3" t="n"/>
       <c r="H166" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7270,25 +7270,25 @@
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>pricing.blueprint.body</t>
+          <t>pricing.blueprint.cta</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
         <is>
-          <t>Order technical and expert support by the hour. Our team helps with implementation, know-how, and years of experience - exactly when you need it. €69/h + VAT, no minimum commitment.</t>
+          <t>Request support →</t>
         </is>
       </c>
       <c r="E167" s="3" t="inlineStr">
         <is>
-          <t>შეუკვეთე ტექნიკური და საექსპერტო მხარდაჭერა საათობრივად. ჩვენი გუნდი დაგეხმარება ტექნიკური დანერგვით, ცოდნითა და წლების გამოცდილებით - ზუსტად მაშინ, როცა გჭირდება. €69/სთ + დღგ, არანაირი მინიმალური ვალდებულება.</t>
+          <t>მოითხოვე მხარდაჭერა →</t>
         </is>
       </c>
       <c r="F167" s="3" t="inlineStr">
         <is>
-          <t>Закажите техническую и экспертную поддержку почасово. Наша команда поможет с технической реализацией, знаниями и многолетним опытом - именно тогда, когда это нужно. €69/ч + НДС, без минимальных обязательств.</t>
-        </is>
-      </c>
-      <c r="G167" s="3" t="inlineStr"/>
+          <t>Запросить поддержку →</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="n"/>
       <c r="H167" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7303,30 +7303,34 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>pricing.blueprint.cta</t>
+          <t>form.fullName</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
         <is>
-          <t>Request support →</t>
+          <t>Full Name</t>
         </is>
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე მხარდაჭერა →</t>
+          <t>სახელი და გვარი</t>
         </is>
       </c>
       <c r="F168" s="3" t="inlineStr">
         <is>
-          <t>Запросить поддержку →</t>
-        </is>
-      </c>
-      <c r="G168" s="3" t="inlineStr"/>
+          <t>Имя и фамилия</t>
+        </is>
+      </c>
+      <c r="G168" s="3" t="inlineStr">
+        <is>
+          <t>Single "Full Name" field. CRM: 1 word -&gt; Last Name; 2+ words -&gt; first = First Name, rest = Last Name</t>
+        </is>
+      </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7346,27 +7350,27 @@
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>form.fullName</t>
+          <t>form.consent</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
         <is>
-          <t>Full Name</t>
+          <t>By submitting this form, I consent to Unity LLC (unitty.io) processing my data for communication and direct marketing. I can withdraw consent or have my data corrected or deleted at any time by writing to digital@unitty.io.</t>
         </is>
       </c>
       <c r="E169" s="3" t="inlineStr">
         <is>
-          <t>სახელი და გვარი</t>
+          <t>ფორმის გაგზავნით ვეთანხმები შპს „იუნითის“ (unitty.io) მიერ ჩემი მონაცემების დამუშავებას კომუნიკაციისა და პირდაპირი მარკეტინგის მიზნით. თანხმობის გაუქმება ან მონაცემების გასწორება/წაშლა შესაძლებელია ნებისმიერ დროს: digital@unitty.io მიმართვით.</t>
         </is>
       </c>
       <c r="F169" s="3" t="inlineStr">
         <is>
-          <t>Имя и фамилия</t>
+          <t>Отправляя форму, я соглашаюсь на обработку моих данных ООО «Юнити» (unitty.io) в целях коммуникации и прямого маркетинга. Отозвать согласие или исправить/удалить данные можно в любое время, написав на digital@unitty.io.</t>
         </is>
       </c>
       <c r="G169" s="3" t="inlineStr">
         <is>
-          <t>Single "Full Name" field. CRM: 1 word -&gt; Last Name; 2+ words -&gt; first = First Name, rest = Last Name</t>
+          <t>Consent text under the lead form (personal data + direct marketing)</t>
         </is>
       </c>
       <c r="H169" s="3" t="inlineStr">
@@ -7383,32 +7387,32 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Nav</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>form.consent</t>
+          <t>nav.call</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>By submitting this form, I consent to Unity LLC (unitty.io) processing my data for communication and direct marketing. I can withdraw consent or have my data corrected or deleted at any time by writing to digital@unitty.io.</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="E170" s="3" t="inlineStr">
         <is>
-          <t>ფორმის გაგზავნით ვეთანხმები შპს „იუნითის“ (unitty.io) მიერ ჩემი მონაცემების დამუშავებას კომუნიკაციისა და პირდაპირი მარკეტინგის მიზნით. თანხმობის გაუქმება ან მონაცემების გასწორება/წაშლა შესაძლებელია ნებისმიერ დროს: digital@unitty.io მიმართვით.</t>
+          <t>დარეკვა</t>
         </is>
       </c>
       <c r="F170" s="3" t="inlineStr">
         <is>
-          <t>Отправляя форму, я соглашаюсь на обработку моих данных ООО «Юнити» (unitty.io) в целях коммуникации и прямого маркетинга. Отозвать согласие или исправить/удалить данные можно в любое время, написав на digital@unitty.io.</t>
+          <t>Позвонить</t>
         </is>
       </c>
       <c r="G170" s="3" t="inlineStr">
         <is>
-          <t>Consent text under the lead form (personal data + direct marketing)</t>
+          <t>Header call button (shown Mon-Fri 10:00-19:00 Tbilisi time)</t>
         </is>
       </c>
       <c r="H170" s="3" t="inlineStr">
@@ -7425,32 +7429,32 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>Nav</t>
+          <t>Pricing</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>nav.call</t>
+          <t>pricing.note</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>These packages describe the collaboration model and its minimum thresholds. The exact cost and details are agreed individually.</t>
         </is>
       </c>
       <c r="E171" s="3" t="inlineStr">
         <is>
-          <t>დარეკვა</t>
+          <t>ეს პაკეტები ასახავს თანამშრომლობის მოდელს და მინიმალურ ზღვრებს. უშუალოდ ღირებულების და დეტალების შეთანხმება ხდება ინდივიდუალურად.</t>
         </is>
       </c>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>Позвонить</t>
+          <t>Эти пакеты описывают модель сотрудничества и минимальные пороги. Точная стоимость и детали согласовываются индивидуально.</t>
         </is>
       </c>
       <c r="G171" s="3" t="inlineStr">
         <is>
-          <t>Header call button (shown Mon-Fri 10:00-19:00 Tbilisi time)</t>
+          <t>Note under the three packages</t>
         </is>
       </c>
       <c r="H171" s="3" t="inlineStr">
@@ -8666,7 +8670,7 @@
           <t>Выберите удобное время</t>
         </is>
       </c>
-      <c r="G200" s="3" t="inlineStr"/>
+      <c r="G200" s="3" t="n"/>
       <c r="H200" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -8704,7 +8708,7 @@
           <t>Подтверждение и ссылка на Google Meet придут на почту сразу.</t>
         </is>
       </c>
-      <c r="G201" s="3" t="inlineStr"/>
+      <c r="G201" s="3" t="n"/>
       <c r="H201" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -8742,7 +8746,7 @@
           <t>Календарь не загружается? Откройте в новой вкладке</t>
         </is>
       </c>
-      <c r="G202" s="3" t="inlineStr"/>
+      <c r="G202" s="3" t="n"/>
       <c r="H202" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -8850,7 +8854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -9399,6 +9403,44 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Landing</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Pricing</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>pricing.2.feature.6</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>30-day post-launch tuning</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>30-დღიანი დანერგვის შემდგომი დახვეწა</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>30-дневная настройка после запуска</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Hero subtitle + downloadable 10-tools PDF
</commit_message>
<xml_diff>
--- a/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
+++ b/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
@@ -827,17 +827,17 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>After 500+ successful deployments across multiple industries, we'll show you the exact 1-3 tools that solve your challenges - all in one call. Free if you book now.</t>
+          <t>With 500+ successful implementations behind us, in 20 minutes I'll walk you through the exact 1-3 tools that will handle your challenges. Free if you book now.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>სხვადასხვა ინდუსტრიაში 500+ წარმატებული დანერგვის გამოცდილებით, 20 წუთში გაგიჩვენებთ ზუსტად იმ 1-3 ხელსაწყოს, რომელიც შენ გამოწვევებს გაუმკლავდება. უფასოდ - თუ ახლავე დაჯავშნი.</t>
+          <t>500+ წარმატებული დანერგვის გამოცდილებით, 20 წუთში, მოგიყვები ზუსტად იმ 1-3 ინსტრუმენტის შესახებ, რომლებიც შენს გამოწვევებს გაუმკლავდება. უფასოდ - თუ ახლავე დაჯავშნი.</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>После более 500 успешных внедрений в разных отраслях мы за один звонок покажем вам ровно те 1-3 инструмента, которые решают ваши задачи. Бесплатно - если бронируете сейчас.</t>
+          <t>Опираясь на 500+ успешных внедрений, за 20 минут расскажу о тех 1-3 инструментах, которые справятся с вашими задачами. Бесплатно - если бронируете сейчас.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -7985,17 +7985,17 @@
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>PDF · 12 pages · personal picks</t>
+          <t>PDF · 3 pages · personal picks</t>
         </is>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>PDF · 12 გვერდი · პირადი რეკომენდაციები</t>
+          <t>PDF · 3 გვერდი · პირადი რეკომენდაციები</t>
         </is>
       </c>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>PDF · 12 страниц · личный выбор</t>
+          <t>PDF · 3 страницы · личные рекомендации</t>
         </is>
       </c>
       <c r="G184" s="3" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Meeting changes: header, hero, logos, pricing, bonus PDF, video controls
</commit_message>
<xml_diff>
--- a/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
+++ b/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
@@ -8,7 +8,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed keys" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Untitled'!$A$1:$H$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Untitled'!$A$1:$H$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z204"/>
+  <dimension ref="A1:Z201"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -743,17 +743,17 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>30+ hours</t>
+          <t>100+ hours</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>30+ საათიან</t>
+          <t>100+ საათიან</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>30+ часов</t>
+          <t>100+ часов</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -953,17 +953,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a Call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -1583,17 +1583,17 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Years · Market Expert</t>
+          <t>years of experience</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>წელი · ბაზრის ექსპერტი</t>
+          <t>წლიანი გამოცდილება</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>лет · Эксперт рынка</t>
+          <t>лет опыта</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -3683,17 +3683,17 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Tangible results</t>
+          <t>What our clients say</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>ხელშესახები შედეგები</t>
+          <t>რას ამბობენ კლიენტები</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>Ощутимые результаты</t>
+          <t>Что говорят клиенты</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -4079,17 +4079,17 @@
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>20 minutes to save 30+ hours</t>
+          <t>20 minutes to save 100+ hours</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>20 წუთი, 30+ საათის დასაზოგად</t>
+          <t>20 წუთი, 100+ საათის დასაზოგად</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>20 минут, чтобы сэкономить 30+ часов</t>
+          <t>20 минут, чтобы сэкономить 100+ часов</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -5717,23 +5717,23 @@
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>Collaboration</t>
         </is>
       </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
-          <t>ფასი</t>
+          <t>თანამშრომლობა</t>
         </is>
       </c>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>Цены</t>
+          <t>Сотрудничество</t>
         </is>
       </c>
       <c r="G126" s="3" t="n"/>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -5869,17 +5869,17 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>ADVISOR</t>
+          <t>CONSULTING</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>ADVISOR</t>
+          <t>კონსულტაცია</t>
         </is>
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>ADVISOR</t>
+          <t>КОНСУЛЬТАЦИЯ</t>
         </is>
       </c>
       <c r="G130" s="3" t="n"/>
@@ -6059,23 +6059,23 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>1-2 solutions from our catalog</t>
+          <t>1-2 specific solutions</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>1-2 გადაწყვეტა კატალოგიდან</t>
+          <t>1-2 კონკრეტული გადაწყვეტა</t>
         </is>
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>1-2 решения из каталога</t>
+          <t>1-2 конкретных решения</t>
         </is>
       </c>
       <c r="G135" s="3" t="n"/>
       <c r="H135" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6211,17 +6211,17 @@
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>Request Advisor</t>
+          <t>Request consulting</t>
         </is>
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე Advisor</t>
+          <t>მოითხოვე კონსულტაცია</t>
         </is>
       </c>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>Запросить Advisor</t>
+          <t>Запросить консультацию</t>
         </is>
       </c>
       <c r="G139" s="3" t="n"/>
@@ -6325,17 +6325,17 @@
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>SPRINTER</t>
+          <t>IMPLEMENTATION</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>SPRINTER</t>
+          <t>დანერგვა</t>
         </is>
       </c>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>SPRINTER</t>
+          <t>ВНЕДРЕНИЕ</t>
         </is>
       </c>
       <c r="G142" s="3" t="n"/>
@@ -6553,23 +6553,23 @@
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Up to 6 solutions from catalog</t>
+          <t>Up to 6 solutions</t>
         </is>
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>6-მდე გადაწყვეტა კატალოგიდან</t>
+          <t>6-მდე გადაწყვეტა</t>
         </is>
       </c>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>До 6 решений из каталога</t>
+          <t>До 6 решений</t>
         </is>
       </c>
       <c r="G148" s="3" t="n"/>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -6705,17 +6705,17 @@
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Request Sprinter</t>
+          <t>Request implementation</t>
         </is>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე Sprinter</t>
+          <t>მოითხოვე დანერგვა</t>
         </is>
       </c>
       <c r="F152" s="3" t="inlineStr">
         <is>
-          <t>Запросить Sprinter</t>
+          <t>Запросить внедрение</t>
         </is>
       </c>
       <c r="G152" s="3" t="n"/>
@@ -6781,17 +6781,17 @@
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>PRIORITY</t>
+          <t>PARTNERSHIP</t>
         </is>
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
-          <t>PRIORITY</t>
+          <t>პარტნიორობა</t>
         </is>
       </c>
       <c r="F154" s="3" t="inlineStr">
         <is>
-          <t>PRIORITY</t>
+          <t>ПАРТНЁРСТВО</t>
         </is>
       </c>
       <c r="G154" s="3" t="n"/>
@@ -6971,17 +6971,17 @@
       </c>
       <c r="D159" s="3" t="inlineStr">
         <is>
-          <t>Everything included in Sprinter</t>
+          <t>Everything included in Implementation</t>
         </is>
       </c>
       <c r="E159" s="3" t="inlineStr">
         <is>
-          <t>ყველაფერი, რასაც Sprinter მოიცავს</t>
+          <t>ყველაფერი, რასაც დანერგვა მოიცავს</t>
         </is>
       </c>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>Всё, что входит в Sprinter</t>
+          <t>Всё, что входит во Внедрение</t>
         </is>
       </c>
       <c r="G159" s="3" t="n"/>
@@ -7085,23 +7085,23 @@
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>Managed services (ongoing optimization)</t>
+          <t>Ongoing optimization</t>
         </is>
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
-          <t>Managed services (მუდმივი ოპტიმიზაცია)</t>
+          <t>მუდმივი ოპტიმიზაცია</t>
         </is>
       </c>
       <c r="F162" s="3" t="inlineStr">
         <is>
-          <t>Managed services (постоянная оптимизация)</t>
+          <t>Постоянная оптимизация</t>
         </is>
       </c>
       <c r="G162" s="3" t="n"/>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -7161,17 +7161,17 @@
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Request Priority</t>
+          <t>Request partnership</t>
         </is>
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე Priority</t>
+          <t>მოითხოვე პარტნიორობა</t>
         </is>
       </c>
       <c r="F164" s="3" t="inlineStr">
         <is>
-          <t>Запросить Priority</t>
+          <t>Запросить партнёрство</t>
         </is>
       </c>
       <c r="G164" s="3" t="n"/>
@@ -7439,17 +7439,17 @@
       </c>
       <c r="D171" s="3" t="inlineStr">
         <is>
-          <t>These packages describe the collaboration model and its minimum thresholds. The exact cost and details are agreed individually.</t>
+          <t>These packages describe our ways of working together. The cost is set individually and starts from 2,990 GEL (prices exclude VAT).</t>
         </is>
       </c>
       <c r="E171" s="3" t="inlineStr">
         <is>
-          <t>ეს პაკეტები ასახავს თანამშრომლობის მოდელს და მინიმალურ ზღვრებს. უშუალოდ ღირებულების და დეტალების შეთანხმება ხდება ინდივიდუალურად.</t>
+          <t>ეს პაკეტები ასახავს თანამშრომლობის მიდგომებს. ღირებულება ინდივიდუალურად განისაზღვრება და იწყება 2990 ლარიდან (ფასები არ მოიცავს დღგ-ს).</t>
         </is>
       </c>
       <c r="F171" s="3" t="inlineStr">
         <is>
-          <t>Эти пакеты описывают модель сотрудничества и минимальные пороги. Точная стоимость и детали согласовываются индивидуально.</t>
+          <t>Эти пакеты описывают подходы к сотрудничеству. Стоимость определяется индивидуально и начинается от 2990 лари (цены без НДС).</t>
         </is>
       </c>
       <c r="G171" s="3" t="inlineStr">
@@ -7459,175 +7459,159 @@
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>Thank-you</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>Confirm</t>
+          <t>Gain</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>ty.confirm.title</t>
+          <t>gain.title</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>Thank you {name}, your request has been received.</t>
+          <t>What you get from this call</t>
         </is>
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
-          <t>მადლობა {name}, თქვენი მოთხოვნა მიღებულია.</t>
+          <t>რას მიიღებ ამ ზარით</t>
         </is>
       </c>
       <c r="F172" s="3" t="inlineStr">
         <is>
-          <t>Спасибо, {name}, ваш запрос получен.</t>
-        </is>
-      </c>
-      <c r="G172" s="3" t="inlineStr">
-        <is>
-          <t>Thank-you headline. Keep {name} - it is replaced with the visitor's first name</t>
-        </is>
-      </c>
+          <t>Что вы получите от этого звонка</t>
+        </is>
+      </c>
+      <c r="G172" s="3" t="inlineStr"/>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>Thank-you</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>SelfBook</t>
+          <t>Gain</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>ty.selfbook.eyebrow</t>
+          <t>gain.1</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
         <is>
-          <t>Prefer to pick a time yourself?</t>
+          <t>You save a lot of time - and with it, money.</t>
         </is>
       </c>
       <c r="E173" s="3" t="inlineStr">
         <is>
-          <t>გირჩევნია დრო თავად შეარჩიო?</t>
+          <t>დაზოგავ უამრავ დროს, შესაბამისად ფულსაც.</t>
         </is>
       </c>
       <c r="F173" s="3" t="inlineStr">
         <is>
-          <t>Хотите выбрать время сами?</t>
-        </is>
-      </c>
-      <c r="G173" s="3" t="inlineStr">
-        <is>
-          <t>Lime eyebrow</t>
-        </is>
-      </c>
+          <t>Сэкономите массу времени, а значит и денег.</t>
+        </is>
+      </c>
+      <c r="G173" s="3" t="inlineStr"/>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>Thank-you</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>SelfBook</t>
+          <t>Gain</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>ty.selfbook.title</t>
+          <t>gain.2</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Skip the wait - book a 20-minute slot directly on my calendar</t>
+          <t>You'll know the concrete next steps to take.</t>
         </is>
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>ნუ დაელოდები ზარს - დაჯავშნე 20-წუთიანი სლოტი პირდაპირ ჩემს კალენდარში</t>
+          <t>გეცოდინება კონკრეტული გადასადგმელი ნაბიჯები.</t>
         </is>
       </c>
       <c r="F174" s="3" t="inlineStr">
         <is>
-          <t>Не ждите - забронируйте 20-минутный слот прямо в моём календаре</t>
-        </is>
-      </c>
-      <c r="G174" s="3" t="inlineStr">
-        <is>
-          <t>Self-book card title</t>
-        </is>
-      </c>
+          <t>Будете знать конкретные следующие шаги.</t>
+        </is>
+      </c>
+      <c r="G174" s="3" t="inlineStr"/>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>New</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>Thank-you</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>SelfBook</t>
+          <t>Gain</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>ty.selfbook.note</t>
+          <t>gain.3</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
-          <t>Pick a time that works for you. The confirmation and the Google Meet link will be sent to your email.</t>
+          <t>You'll set realistic expectations for results, timelines and budget.</t>
         </is>
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>შეარჩიე შენთვის მოსახერხებელი დრო. დადასტურება და Google Meet-ის ბმული გამოიგზავნება შენს ელ.ფოსტაზე.</t>
+          <t>შეიქმნი ადეკვატურ მოლოდინს შედეგზე, ვადებზე და ბიუჯეტზე.</t>
         </is>
       </c>
       <c r="F175" s="3" t="inlineStr">
         <is>
-          <t>Выберите удобное время. Подтверждение и ссылка на Google Meet придут на вашу почту.</t>
-        </is>
-      </c>
-      <c r="G175" s="3" t="inlineStr">
-        <is>
-          <t>Self-book card note</t>
-        </is>
-      </c>
+          <t>Сформируете реалистичные ожидания по результату, срокам и бюджету.</t>
+        </is>
+      </c>
+      <c r="G175" s="3" t="inlineStr"/>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -7639,37 +7623,37 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>SelfBook</t>
+          <t>Confirm</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>ty.selfbook.cta</t>
+          <t>ty.confirm.title</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Book a Call</t>
+          <t>Thank you {name}, your request has been received.</t>
         </is>
       </c>
       <c r="E176" s="3" t="inlineStr">
         <is>
-          <t>დაჯავშნე შეხვედრა</t>
+          <t>მადლობა {name}, თქვენი მოთხოვნა მიღებულია.</t>
         </is>
       </c>
       <c r="F176" s="3" t="inlineStr">
         <is>
-          <t>Забронировать звонок</t>
+          <t>Спасибо, {name}, ваш запрос получен.</t>
         </is>
       </c>
       <c r="G176" s="3" t="inlineStr">
         <is>
-          <t>Primary CTA button</t>
+          <t>Thank-you headline. Keep {name} - it is replaced with the visitor's first name</t>
         </is>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -7686,27 +7670,27 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>ty.selfbook.meta</t>
+          <t>ty.selfbook.eyebrow</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
         <is>
-          <t>⏱ 20 min · 🖥 Google Meet · Free</t>
+          <t>Prefer to pick a time yourself?</t>
         </is>
       </c>
       <c r="E177" s="3" t="inlineStr">
         <is>
-          <t>⏱ 20 წთ · 🖥 Google Meet · უფასო</t>
+          <t>გირჩევნია დრო თავად შეარჩიო?</t>
         </is>
       </c>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>⏱ 20 мин · 🖥 Google Meet · Бесплатно</t>
+          <t>Хотите выбрать время сами?</t>
         </is>
       </c>
       <c r="G177" s="3" t="inlineStr">
         <is>
-          <t>Meta line under CTA</t>
+          <t>Lime eyebrow</t>
         </is>
       </c>
       <c r="H177" s="3" t="inlineStr">
@@ -7723,32 +7707,32 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>SelfBook</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>ty.video.eyebrow</t>
+          <t>ty.selfbook.title</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Before we talk</t>
+          <t>Skip the wait - book a 20-minute slot directly on my calendar</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
-          <t>სანამ ვისაუბრებთ</t>
+          <t>ნუ დაელოდები ზარს - დაჯავშნე 20-წუთიანი სლოტი პირდაპირ ჩემს კალენდარში</t>
         </is>
       </c>
       <c r="F178" s="3" t="inlineStr">
         <is>
-          <t>Прежде чем поговорим</t>
+          <t>Не ждите - забронируйте 20-минутный слот прямо в моём календаре</t>
         </is>
       </c>
       <c r="G178" s="3" t="inlineStr">
         <is>
-          <t>Section eyebrow</t>
+          <t>Self-book card title</t>
         </is>
       </c>
       <c r="H178" s="3" t="inlineStr">
@@ -7765,37 +7749,37 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>SelfBook</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>ty.video.title</t>
+          <t>ty.selfbook.cta</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
         <is>
-          <t>A 60-second note from Giorgi</t>
+          <t>Book a Call</t>
         </is>
       </c>
       <c r="E179" s="3" t="inlineStr">
         <is>
-          <t>60-წამიანი მიმართვა გიორგისგან</t>
+          <t>დაჯავშნე შეხვედრა</t>
         </is>
       </c>
       <c r="F179" s="3" t="inlineStr">
         <is>
-          <t>60-секундное обращение от Георгия</t>
+          <t>Забронировать звонок</t>
         </is>
       </c>
       <c r="G179" s="3" t="inlineStr">
         <is>
-          <t>Section title</t>
+          <t>Primary CTA button</t>
         </is>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7807,32 +7791,32 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>SelfBook</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>ty.video.caption</t>
+          <t>ty.selfbook.meta</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Welcome from Giorgi</t>
+          <t>⏱ 20 min · 🖥 Google Meet · Free</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
-          <t>მოკლე ვიდეო გიორგისგან</t>
+          <t>⏱ 20 წთ · 🖥 Google Meet · უფასო</t>
         </is>
       </c>
       <c r="F180" s="3" t="inlineStr">
         <is>
-          <t>Приветствие от Георгия</t>
+          <t>⏱ 20 мин · 🖥 Google Meet · Бесплатно</t>
         </is>
       </c>
       <c r="G180" s="3" t="inlineStr">
         <is>
-          <t>Video poster caption</t>
+          <t>Meta line under CTA</t>
         </is>
       </c>
       <c r="H180" s="3" t="inlineStr">
@@ -7849,27 +7833,27 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>Gift</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>ty.gift.eyebrow</t>
+          <t>ty.video.eyebrow</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
         <is>
-          <t>A gift from me</t>
+          <t>Before we talk</t>
         </is>
       </c>
       <c r="E181" s="3" t="inlineStr">
         <is>
-          <t>საჩუქარი ჩემგან</t>
+          <t>სანამ ვისაუბრებთ</t>
         </is>
       </c>
       <c r="F181" s="3" t="inlineStr">
         <is>
-          <t>Подарок от меня</t>
+          <t>Прежде чем поговорим</t>
         </is>
       </c>
       <c r="G181" s="3" t="inlineStr">
@@ -7891,32 +7875,32 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>Gift</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>ty.gift.title</t>
+          <t>ty.video.title</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>10 tools we use every day to run faster</t>
+          <t>A 60-second note from Giorgi</t>
         </is>
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>10 ინსტრუმენტი, რომელსაც ყოველდღიურად ვიყენებთ ეფექტურობის გასაზრდელად</t>
+          <t>60-წამიანი მიმართვა გიორგისგან</t>
         </is>
       </c>
       <c r="F182" s="3" t="inlineStr">
         <is>
-          <t>10 инструментов, которыми мы пользуемся каждый день, чтобы работать быстрее</t>
+          <t>60-секундное обращение от Георгия</t>
         </is>
       </c>
       <c r="G182" s="3" t="inlineStr">
         <is>
-          <t>Gift section title</t>
+          <t>Section title</t>
         </is>
       </c>
       <c r="H182" s="3" t="inlineStr">
@@ -7933,37 +7917,37 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>Gift</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>ty.gift.sub</t>
+          <t>ty.video.caption</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
         <is>
-          <t>An opinionated PDF - the exact stack we rely on for research, writing, scheduling, note-taking, and keeping my own team sharp. Yours, free, no strings.</t>
+          <t>Welcome from Giorgi</t>
         </is>
       </c>
       <c r="E183" s="3" t="inlineStr">
         <is>
-          <t>პრაქტიკული PDF გზამკვლევი - ინსტრუმენტები, რომლებსაც ყოველდღე ვიყენებთ კვლევისთვის, ტექსტების დასაწერად, შეხვედრების დასაგეგმად და გუნდის ეფექტურობისთვის. სრულიად უფასოდ, ჩამოტვირთე.</t>
+          <t>მოკლე ვიდეო გიორგისგან</t>
         </is>
       </c>
       <c r="F183" s="3" t="inlineStr">
         <is>
-          <t>Личный PDF с подборкой - точный стек, которым мы пользуемся для исследований, писанины, планирования встреч, заметок и чтобы держать команду в тонусе. Ваше, бесплатно, без условий.</t>
+          <t>Приветствие от Георгия</t>
         </is>
       </c>
       <c r="G183" s="3" t="inlineStr">
         <is>
-          <t>Gift section subtitle</t>
+          <t>Video poster caption</t>
         </is>
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7975,37 +7959,37 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>Gift</t>
+          <t>Prep</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>ty.gift.tag</t>
+          <t>ty.prep.eyebrow</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>PDF · 3 pages · personal picks</t>
+          <t>Optional - if you want to go deeper</t>
         </is>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>PDF · 3 გვერდი · პირადი რეკომენდაციები</t>
+          <t>სურვილისამებრ - თუ გსურს უფრო სიღრმისეულად მომზადება</t>
         </is>
       </c>
       <c r="F184" s="3" t="inlineStr">
         <is>
-          <t>PDF · 3 страницы · личные рекомендации</t>
+          <t>По желанию - если хотите углубиться</t>
         </is>
       </c>
       <c r="G184" s="3" t="inlineStr">
         <is>
-          <t>Small tag above gift card title</t>
+          <t>Section eyebrow</t>
         </is>
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8017,37 +8001,37 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Gift</t>
+          <t>Prep</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>ty.gift.card.title</t>
+          <t>ty.prep.title</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
         <is>
-          <t>Unitty's Productivity Stack 2026</t>
+          <t>Five questions to think about beforehand</t>
         </is>
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
-          <t>Unitty-ის პროდუქტიულობის ნაკრები 2026</t>
+          <t>5 კითხვა, რომელზეც შეგიძლია წინასწარ დაფიქრდე</t>
         </is>
       </c>
       <c r="F185" s="3" t="inlineStr">
         <is>
-          <t>Стек продуктивности Unitty 2026</t>
+          <t>Пять вопросов, о которых подумать заранее</t>
         </is>
       </c>
       <c r="G185" s="3" t="inlineStr">
         <is>
-          <t>Gift card title</t>
+          <t>Section title</t>
         </is>
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8059,37 +8043,37 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>Gift</t>
+          <t>Prep</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>ty.gift.card.desc</t>
+          <t>ty.prep.sub</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
         <is>
-          <t>Each tool with what we use it for, why it beats the alternatives I tried, and the one setting most people miss. Takes 8 minutes to read, saves hours a week.</t>
+          <t>Not required. But if you want our 20 minutes to cut straight to the answer, these are the places I usually start.</t>
         </is>
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>თითოეული ხელსაწყოს დეტალური აღწერა: რისთვის ვიყენებთ, რით ჯობია ალტერნატივებს და რომელია ის მთავარი ფუნქცია, რაც უმეტესობას გამორჩება ხოლმე. წასაკითხად საჭიროა 8 წუთი - გიზოგავს კვირაში რამდენიმე საათს.</t>
+          <t>არ არის სავალდებულო. მაგრამ თუ გსურს, ჩვენი 20 წუთი პირდაპირ გადაწყვეტაზე ორიენტირებული იყოს, ეს ის კითხვებია, რითაც ყოველთვის ვიწყებ.</t>
         </is>
       </c>
       <c r="F186" s="3" t="inlineStr">
         <is>
-          <t>О каждом инструменте: для чего используем, почему он лучше альтернатив, которые пробовали, и та одна настройка, которую большинство упускает. Читается 8 минут, экономит часы в неделю.</t>
+          <t>Не обязательно. Но если хотите, чтобы наши 20 минут сразу вышли на ответ - вот откуда я обычно начинаю.</t>
         </is>
       </c>
       <c r="G186" s="3" t="inlineStr">
         <is>
-          <t>Gift card description</t>
+          <t>Section subtitle</t>
         </is>
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8101,32 +8085,32 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>Gift</t>
+          <t>Prep</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>ty.gift.card.cta</t>
+          <t>ty.prep.q1</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
         <is>
-          <t>Download the PDF</t>
+          <t>How does the work you want to improve happen today - who does it, in which tool, and where does it break?</t>
         </is>
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
-          <t>ჩამოტვირთე PDF</t>
+          <t>როგორ სრულდება ის პროცესი დღეს, რომლის გაუმჯობესებაც გსურს - ვინ აკეთებს, სად, და რა იწვევს შეფერხებას?</t>
         </is>
       </c>
       <c r="F187" s="3" t="inlineStr">
         <is>
-          <t>Скачать PDF</t>
+          <t>Как сейчас происходит работа, которую вы хотите улучшить - кто её делает, в каком инструменте и где всё ломается?</t>
         </is>
       </c>
       <c r="G187" s="3" t="inlineStr">
         <is>
-          <t>Gift card CTA button</t>
+          <t>Prep Q1</t>
         </is>
       </c>
       <c r="H187" s="3" t="inlineStr">
@@ -8148,27 +8132,27 @@
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>ty.prep.eyebrow</t>
+          <t>ty.prep.q2</t>
         </is>
       </c>
       <c r="D188" s="3" t="inlineStr">
         <is>
-          <t>Optional - if you want to go deeper</t>
+          <t>What have you already tried, and what specifically didn't work about it?</t>
         </is>
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>სურვილისამებრ - თუ გსურს უფრო სიღრმისეულად მომზადება</t>
+          <t>რა გზები სცადეთ უკვე და კონკრეტულად რატომ არ გაამართლა?</t>
         </is>
       </c>
       <c r="F188" s="3" t="inlineStr">
         <is>
-          <t>По желанию - если хотите углубиться</t>
+          <t>Что вы уже пробовали, и что конкретно не сработало?</t>
         </is>
       </c>
       <c r="G188" s="3" t="inlineStr">
         <is>
-          <t>Section eyebrow</t>
+          <t>Prep Q2</t>
         </is>
       </c>
       <c r="H188" s="3" t="inlineStr">
@@ -8190,27 +8174,27 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>ty.prep.title</t>
+          <t>ty.prep.q3</t>
         </is>
       </c>
       <c r="D189" s="3" t="inlineStr">
         <is>
-          <t>Five questions to think about beforehand</t>
+          <t>If this problem were solved three months from now, what would be different about your day?</t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>5 კითხვა, რომელზეც შეგიძლია წინასწარ დაფიქრდე</t>
+          <t>ეს პრობლემა 3 თვეში რომ სრულად მოგვარდეს, რა შეიცვლებოდა შენს ყოველდღიურ საქმიანობაში?</t>
         </is>
       </c>
       <c r="F189" s="3" t="inlineStr">
         <is>
-          <t>Пять вопросов, о которых подумать заранее</t>
+          <t>Если бы эта проблема была решена через три месяца, что в вашем дне стало бы другим?</t>
         </is>
       </c>
       <c r="G189" s="3" t="inlineStr">
         <is>
-          <t>Section title</t>
+          <t>Prep Q3</t>
         </is>
       </c>
       <c r="H189" s="3" t="inlineStr">
@@ -8232,27 +8216,27 @@
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>ty.prep.sub</t>
+          <t>ty.prep.q4</t>
         </is>
       </c>
       <c r="D190" s="3" t="inlineStr">
         <is>
-          <t>Not required. But if you want our 20 minutes to cut straight to the answer, these are the places I usually start.</t>
+          <t>Who in your team will own the new process - a specific person, or still deciding?</t>
         </is>
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>არ არის სავალდებულო. მაგრამ თუ გსურს, ჩვენი 20 წუთი პირდაპირ გადაწყვეტაზე ორიენტირებული იყოს, ეს ის კითხვებია, რითაც ყოველთვის ვიწყებ.</t>
+          <t>ვინ იქნება შენს გუნდში ახალი პროცესის პასუხისმგებელი პირი - კონკრეტული თანამშრომელი, თუ ჯერ გადასაწყვეტია?</t>
         </is>
       </c>
       <c r="F190" s="3" t="inlineStr">
         <is>
-          <t>Не обязательно. Но если хотите, чтобы наши 20 минут сразу вышли на ответ - вот откуда я обычно начинаю.</t>
+          <t>Кто в вашей команде будет владельцем нового процесса - конкретный человек или ещё решаете?</t>
         </is>
       </c>
       <c r="G190" s="3" t="inlineStr">
         <is>
-          <t>Section subtitle</t>
+          <t>Prep Q4</t>
         </is>
       </c>
       <c r="H190" s="3" t="inlineStr">
@@ -8274,32 +8258,32 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>ty.prep.q1</t>
+          <t>ty.prep.q5</t>
         </is>
       </c>
       <c r="D191" s="3" t="inlineStr">
         <is>
-          <t>How does the work you want to improve happen today - who does it, in which tool, and where does it break?</t>
+          <t>What's your rough budget range - not a commitment, just so we don't propose something that doesn't fit?</t>
         </is>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>როგორ სრულდება ის პროცესი დღეს, რომლის გაუმჯობესებაც გსურს - ვინ აკეთებს, სად, და რა იწვევს შეფერხებას?</t>
+          <t>რა არის შენი სავარაუდო საორიენტაციო ბიუჯეტი? (ეს არ არის ვალდებულება, უბრალოდ იმისთვის, რომ არ შემოგთავაზოთ ისეთი რამ, რაც შენს შესაძლებლობებს არ შეესაბამება).</t>
         </is>
       </c>
       <c r="F191" s="3" t="inlineStr">
         <is>
-          <t>Как сейчас происходит работа, которую вы хотите улучшить - кто её делает, в каком инструменте и где всё ломается?</t>
+          <t>Какой у вас примерный бюджетный диапазон - не обязательство, просто чтобы мы не предложили что-то, что не вписывается?</t>
         </is>
       </c>
       <c r="G191" s="3" t="inlineStr">
         <is>
-          <t>Prep Q1</t>
+          <t>Prep Q5</t>
         </is>
       </c>
       <c r="H191" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -8311,32 +8295,32 @@
       </c>
       <c r="B192" s="3" t="inlineStr">
         <is>
-          <t>Prep</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>ty.prep.q2</t>
+          <t>ty.social.eyebrow</t>
         </is>
       </c>
       <c r="D192" s="3" t="inlineStr">
         <is>
-          <t>What have you already tried, and what specifically didn't work about it?</t>
+          <t>Follow my work</t>
         </is>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
-          <t>რა გზები სცადეთ უკვე და კონკრეტულად რატომ არ გაამართლა?</t>
+          <t>თვალი ადევნე ჩემს საქმიანობას</t>
         </is>
       </c>
       <c r="F192" s="3" t="inlineStr">
         <is>
-          <t>Что вы уже пробовали, и что конкретно не сработало?</t>
+          <t>Следите за моей работой</t>
         </is>
       </c>
       <c r="G192" s="3" t="inlineStr">
         <is>
-          <t>Prep Q2</t>
+          <t>Section eyebrow</t>
         </is>
       </c>
       <c r="H192" s="3" t="inlineStr">
@@ -8353,32 +8337,32 @@
       </c>
       <c r="B193" s="3" t="inlineStr">
         <is>
-          <t>Prep</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>ty.prep.q3</t>
+          <t>ty.social.title</t>
         </is>
       </c>
       <c r="D193" s="3" t="inlineStr">
         <is>
-          <t>If this problem were solved three months from now, what would be different about your day?</t>
+          <t>Follow for daily videos on productivity tools worth your time</t>
         </is>
       </c>
       <c r="E193" s="3" t="inlineStr">
         <is>
-          <t>ეს პრობლემა 3 თვეში რომ სრულად მოგვარდეს, რა შეიცვლებოდა შენს ყოველდღიურ საქმიანობაში?</t>
+          <t>გამოიწერე ჩემი არხები ყოველდღიური სასარგებლო ვიდეოებისთვის იმ ციფრულ ხელსაწყოებზე, რომლებიც შენს დროს ნამდვილად იმსახურებს</t>
         </is>
       </c>
       <c r="F193" s="3" t="inlineStr">
         <is>
-          <t>Если бы эта проблема была решена через три месяца, что в вашем дне стало бы другим?</t>
+          <t>Подпишитесь, чтобы каждый день получать видео о продуктивных инструментах, которые стоят вашего времени</t>
         </is>
       </c>
       <c r="G193" s="3" t="inlineStr">
         <is>
-          <t>Prep Q3</t>
+          <t>Social section title</t>
         </is>
       </c>
       <c r="H193" s="3" t="inlineStr">
@@ -8395,37 +8379,37 @@
       </c>
       <c r="B194" s="3" t="inlineStr">
         <is>
-          <t>Prep</t>
+          <t>Social</t>
         </is>
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>ty.prep.q4</t>
+          <t>ty.social.sub</t>
         </is>
       </c>
       <c r="D194" s="3" t="inlineStr">
         <is>
-          <t>Who in your team will own the new process - a specific person, or still deciding?</t>
+          <t>Short breakdowns of the tools we actually use with clients - what works, what doesn't, and how to set it up without the sales pitch.</t>
         </is>
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
-          <t>ვინ იქნება შენს გუნდში ახალი პროცესის პასუხისმგებელი პირი - კონკრეტული თანამშრომელი, თუ ჯერ გადასაწყვეტია?</t>
+          <t>მოკლე პრაქტიკული მიმოხილვები ხელსაწყოებზე, რომლებსაც რეალურად ვიყენებთ კლიენტებთან — რა მუშაობს, რა არა და როგორ გამართო მარტივად, ზედმეტი სარეკლამო ხმაურის გარეშე.</t>
         </is>
       </c>
       <c r="F194" s="3" t="inlineStr">
         <is>
-          <t>Кто в вашей команде будет владельцем нового процесса - конкретный человек или ещё решаете?</t>
+          <t>Короткие разборы инструментов, которые мы реально используем с клиентами - что работает, что нет, и как настроить без продажного пафоса.</t>
         </is>
       </c>
       <c r="G194" s="3" t="inlineStr">
         <is>
-          <t>Prep Q4</t>
+          <t>Social section subtitle</t>
         </is>
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Updated</t>
         </is>
       </c>
     </row>
@@ -8437,37 +8421,37 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>Prep</t>
+          <t>Bookings</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>ty.prep.q5</t>
+          <t>ty.bookings.eyebrow</t>
         </is>
       </c>
       <c r="D195" s="3" t="inlineStr">
         <is>
-          <t>What's your rough budget range - not a commitment, just so we don't propose something that doesn't fit?</t>
+          <t>Pick a time now</t>
         </is>
       </c>
       <c r="E195" s="3" t="inlineStr">
         <is>
-          <t>რა არის შენი სავარაუდო საორიენტაციო ბიუჯეტი? (ეს არ არის ვალდებულება, უბრალოდ იმისთვის, რომ არ შემოგთავაზოთ ისეთი რამ, რაც შენს შესაძლებლობებს არ შეესაბამება).</t>
+          <t>აირჩიე დრო ახლავე</t>
         </is>
       </c>
       <c r="F195" s="3" t="inlineStr">
         <is>
-          <t>Какой у вас примерный бюджетный диапазон - не обязательство, просто чтобы мы не предложили что-то, что не вписывается?</t>
+          <t>Выберите время сейчас</t>
         </is>
       </c>
       <c r="G195" s="3" t="inlineStr">
         <is>
-          <t>Prep Q5</t>
+          <t>Booking calendar section</t>
         </is>
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -8479,37 +8463,33 @@
       </c>
       <c r="B196" s="3" t="inlineStr">
         <is>
-          <t>Social</t>
+          <t>Bookings</t>
         </is>
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>ty.social.eyebrow</t>
+          <t>ty.bookings.title</t>
         </is>
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>Follow my work</t>
+          <t>Choose a slot that works for you</t>
         </is>
       </c>
       <c r="E196" s="3" t="inlineStr">
         <is>
-          <t>თვალი ადევნე ჩემს საქმიანობას</t>
+          <t>აირჩიე შენთვის მოსახერხებელი დრო</t>
         </is>
       </c>
       <c r="F196" s="3" t="inlineStr">
         <is>
-          <t>Следите за моей работой</t>
-        </is>
-      </c>
-      <c r="G196" s="3" t="inlineStr">
-        <is>
-          <t>Section eyebrow</t>
-        </is>
-      </c>
+          <t>Выберите удобное время</t>
+        </is>
+      </c>
+      <c r="G196" s="3" t="n"/>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -8521,37 +8501,33 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>Social</t>
+          <t>Bookings</t>
         </is>
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>ty.social.title</t>
+          <t>ty.bookings.note</t>
         </is>
       </c>
       <c r="D197" s="3" t="inlineStr">
         <is>
-          <t>Follow for daily videos on productivity tools worth your time</t>
+          <t>Confirmation and the Google Meet link land in your inbox immediately.</t>
         </is>
       </c>
       <c r="E197" s="3" t="inlineStr">
         <is>
-          <t>გამოიწერე ჩემი არხები ყოველდღიური სასარგებლო ვიდეოებისთვის იმ ციფრულ ხელსაწყოებზე, რომლებიც შენს დროს ნამდვილად იმსახურებს</t>
+          <t>დადასტურება და Google Meet-ის ბმული მაშინვე მოგივა ელფოსტაზე.</t>
         </is>
       </c>
       <c r="F197" s="3" t="inlineStr">
         <is>
-          <t>Подпишитесь, чтобы каждый день получать видео о продуктивных инструментах, которые стоят вашего времени</t>
-        </is>
-      </c>
-      <c r="G197" s="3" t="inlineStr">
-        <is>
-          <t>Social section title</t>
-        </is>
-      </c>
+          <t>Подтверждение и ссылка на Google Meet придут на почту сразу.</t>
+        </is>
+      </c>
+      <c r="G197" s="3" t="n"/>
       <c r="H197" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -8563,37 +8539,33 @@
       </c>
       <c r="B198" s="3" t="inlineStr">
         <is>
-          <t>Social</t>
+          <t>Bookings</t>
         </is>
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>ty.social.sub</t>
+          <t>ty.bookings.fallback</t>
         </is>
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>Short breakdowns of the tools we actually use with clients - what works, what doesn't, and how to set it up without the sales pitch.</t>
+          <t>Calendar not loading? Open it in a new tab</t>
         </is>
       </c>
       <c r="E198" s="3" t="inlineStr">
         <is>
-          <t>მოკლე პრაქტიკული მიმოხილვები ხელსაწყოებზე, რომლებსაც რეალურად ვიყენებთ კლიენტებთან — რა მუშაობს, რა არა და როგორ გამართო მარტივად, ზედმეტი სარეკლამო ხმაურის გარეშე.</t>
+          <t>კალენდარი არ იტვირთება? გახსენი ახალ ფანჯარაში</t>
         </is>
       </c>
       <c r="F198" s="3" t="inlineStr">
         <is>
-          <t>Короткие разборы инструментов, которые мы реально используем с клиентами - что работает, что нет, и как настроить без продажного пафоса.</t>
-        </is>
-      </c>
-      <c r="G198" s="3" t="inlineStr">
-        <is>
-          <t>Social section subtitle</t>
-        </is>
-      </c>
+          <t>Календарь не загружается? Откройте в новой вкладке</t>
+        </is>
+      </c>
+      <c r="G198" s="3" t="n"/>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -8605,32 +8577,32 @@
       </c>
       <c r="B199" s="3" t="inlineStr">
         <is>
-          <t>Bookings</t>
+          <t>Confirm</t>
         </is>
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>ty.bookings.eyebrow</t>
+          <t>ty.confirm.title.noname</t>
         </is>
       </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
-          <t>Pick a time now</t>
+          <t>Thank you, your request has been received.</t>
         </is>
       </c>
       <c r="E199" s="3" t="inlineStr">
         <is>
-          <t>აირჩიე დრო ახლავე</t>
+          <t>მადლობა, თქვენი მოთხოვნა მიღებულია.</t>
         </is>
       </c>
       <c r="F199" s="3" t="inlineStr">
         <is>
-          <t>Выберите время сейчас</t>
+          <t>Спасибо, ваш запрос получен.</t>
         </is>
       </c>
       <c r="G199" s="3" t="inlineStr">
         <is>
-          <t>Booking calendar section</t>
+          <t>Thank-you headline when no name is known</t>
         </is>
       </c>
       <c r="H199" s="3" t="inlineStr">
@@ -8647,30 +8619,34 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>Bookings</t>
+          <t>Nav</t>
         </is>
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>ty.bookings.title</t>
+          <t>nav.call</t>
         </is>
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>Choose a slot that works for you</t>
+          <t>Call</t>
         </is>
       </c>
       <c r="E200" s="3" t="inlineStr">
         <is>
-          <t>აირჩიე შენთვის მოსახერხებელი დრო</t>
+          <t>დარეკვა</t>
         </is>
       </c>
       <c r="F200" s="3" t="inlineStr">
         <is>
-          <t>Выберите удобное время</t>
-        </is>
-      </c>
-      <c r="G200" s="3" t="n"/>
+          <t>Позвонить</t>
+        </is>
+      </c>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>Same text as on the landing - change both rows together</t>
+        </is>
+      </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -8685,160 +8661,38 @@
       </c>
       <c r="B201" s="3" t="inlineStr">
         <is>
-          <t>Bookings</t>
+          <t>Ty</t>
         </is>
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>ty.bookings.note</t>
+          <t>ty.bonus.cta</t>
         </is>
       </c>
       <c r="D201" s="3" t="inlineStr">
         <is>
-          <t>Confirmation and the Google Meet link land in your inbox immediately.</t>
+          <t>Download the bonus PDF</t>
         </is>
       </c>
       <c r="E201" s="3" t="inlineStr">
         <is>
-          <t>დადასტურება და Google Meet-ის ბმული მაშინვე მოგივა ელფოსტაზე.</t>
+          <t>ჩამოტვირთე PDF ბონუსად</t>
         </is>
       </c>
       <c r="F201" s="3" t="inlineStr">
         <is>
-          <t>Подтверждение и ссылка на Google Meet придут на почту сразу.</t>
-        </is>
-      </c>
-      <c r="G201" s="3" t="n"/>
+          <t>Скачать бонусный PDF</t>
+        </is>
+      </c>
+      <c r="G201" s="3" t="inlineStr"/>
       <c r="H201" s="3" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="3" t="inlineStr">
-        <is>
-          <t>Thank-you</t>
-        </is>
-      </c>
-      <c r="B202" s="3" t="inlineStr">
-        <is>
-          <t>Bookings</t>
-        </is>
-      </c>
-      <c r="C202" s="3" t="inlineStr">
-        <is>
-          <t>ty.bookings.fallback</t>
-        </is>
-      </c>
-      <c r="D202" s="3" t="inlineStr">
-        <is>
-          <t>Calendar not loading? Open it in a new tab</t>
-        </is>
-      </c>
-      <c r="E202" s="3" t="inlineStr">
-        <is>
-          <t>კალენდარი არ იტვირთება? გახსენი ახალ ფანჯარაში</t>
-        </is>
-      </c>
-      <c r="F202" s="3" t="inlineStr">
-        <is>
-          <t>Календарь не загружается? Откройте в новой вкладке</t>
-        </is>
-      </c>
-      <c r="G202" s="3" t="n"/>
-      <c r="H202" s="3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="3" t="inlineStr">
-        <is>
-          <t>Thank-you</t>
-        </is>
-      </c>
-      <c r="B203" s="3" t="inlineStr">
-        <is>
-          <t>Confirm</t>
-        </is>
-      </c>
-      <c r="C203" s="3" t="inlineStr">
-        <is>
-          <t>ty.confirm.title.noname</t>
-        </is>
-      </c>
-      <c r="D203" s="3" t="inlineStr">
-        <is>
-          <t>Thank you, your request has been received.</t>
-        </is>
-      </c>
-      <c r="E203" s="3" t="inlineStr">
-        <is>
-          <t>მადლობა, თქვენი მოთხოვნა მიღებულია.</t>
-        </is>
-      </c>
-      <c r="F203" s="3" t="inlineStr">
-        <is>
-          <t>Спасибо, ваш запрос получен.</t>
-        </is>
-      </c>
-      <c r="G203" s="3" t="inlineStr">
-        <is>
-          <t>Thank-you headline when no name is known</t>
-        </is>
-      </c>
-      <c r="H203" s="3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="3" t="inlineStr">
-        <is>
-          <t>Thank-you</t>
-        </is>
-      </c>
-      <c r="B204" s="3" t="inlineStr">
-        <is>
-          <t>Nav</t>
-        </is>
-      </c>
-      <c r="C204" s="3" t="inlineStr">
-        <is>
-          <t>nav.call</t>
-        </is>
-      </c>
-      <c r="D204" s="3" t="inlineStr">
-        <is>
-          <t>Call</t>
-        </is>
-      </c>
-      <c r="E204" s="3" t="inlineStr">
-        <is>
-          <t>დარეკვა</t>
-        </is>
-      </c>
-      <c r="F204" s="3" t="inlineStr">
-        <is>
-          <t>Позвонить</t>
-        </is>
-      </c>
-      <c r="G204" s="3" t="inlineStr">
-        <is>
-          <t>Same text as on the landing - change both rows together</t>
-        </is>
-      </c>
-      <c r="H204" s="3" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H204"/>
+  <autoFilter ref="A1:H201"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
@@ -8854,7 +8708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -9441,6 +9295,342 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>SelfBook</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>ty.selfbook.note</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Pick a time that works for you. The confirmation and the Google Meet link will be sent to your email.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>შეარჩიე შენთვის მოსახერხებელი დრო. დადასტურება და Google Meet-ის ბმული გამოიგზავნება შენს ელ.ფოსტაზე.</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Выберите удобное время. Подтверждение и ссылка на Google Meet придут на вашу почту.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Self-book card note</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>ty.gift.eyebrow</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>A gift from me</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>საჩუქარი ჩემგან</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Подарок от меня</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Section eyebrow</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>ty.gift.title</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>10 tools we use every day to run faster</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>10 ინსტრუმენტი, რომელსაც ყოველდღიურად ვიყენებთ ეფექტურობის გასაზრდელად</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>10 инструментов, которыми мы пользуемся каждый день, чтобы работать быстрее</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Gift section title</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>ty.gift.sub</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>An opinionated PDF - the exact stack we rely on for research, writing, scheduling, note-taking, and keeping my own team sharp. Yours, free, no strings.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>პრაქტიკული PDF გზამკვლევი - ინსტრუმენტები, რომლებსაც ყოველდღე ვიყენებთ კვლევისთვის, ტექსტების დასაწერად, შეხვედრების დასაგეგმად და გუნდის ეფექტურობისთვის. სრულიად უფასოდ, ჩამოტვირთე.</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Личный PDF с подборкой - точный стек, которым мы пользуемся для исследований, писанины, планирования встреч, заметок и чтобы держать команду в тонусе. Ваше, бесплатно, без условий.</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Gift section subtitle</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>ty.gift.tag</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>PDF · 3 pages · personal picks</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>PDF · 3 გვერდი · პირადი რეკომენდაციები</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>PDF · 3 страницы · личные рекомендации</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Small tag above gift card title</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>ty.gift.card.title</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Unitty's Productivity Stack 2026</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Unitty-ის პროდუქტიულობის ნაკრები 2026</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Стек продуктивности Unitty 2026</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Gift card title</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>ty.gift.card.desc</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Each tool with what we use it for, why it beats the alternatives I tried, and the one setting most people miss. Takes 8 minutes to read, saves hours a week.</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>თითოეული ხელსაწყოს დეტალური აღწერა: რისთვის ვიყენებთ, რით ჯობია ალტერნატივებს და რომელია ის მთავარი ფუნქცია, რაც უმეტესობას გამორჩება ხოლმე. წასაკითხად საჭიროა 8 წუთი - გიზოგავს კვირაში რამდენიმე საათს.</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>О каждом инструменте: для чего используем, почему он лучше альтернатив, которые пробовали, и та одна настройка, которую большинство упускает. Читается 8 минут, экономит часы в неделю.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Gift card description</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Gift</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>ty.gift.card.cta</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Download the PDF</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>ჩამოტვირთე PDF</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Скачать PDF</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Gift card CTA button</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Removed 2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
GitHub Desktop → Fetch → Pull → Commit („v33 CRM landing“)
</commit_message>
<xml_diff>
--- a/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
+++ b/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
@@ -14,11 +14,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Start'!$A$1:$H$165</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CRM'!$A$1:$H$205</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AI'!$A$1:$H$205</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CRM'!$A$1:$H$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AI'!$A$1:$H$208</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Banks'!$A$1:$H$165</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Solutions'!$A$1:$H$176</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Thank-you'!$A$1:$H$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Thank-you'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -386,7 +386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" style="6" min="1" max="1"/>
@@ -465,6 +465,24 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -927,17 +945,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე უფასო ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -4347,17 +4365,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a Call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -5997,7 +6015,7 @@
       <c r="G145" s="3" t="inlineStr"/>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6737,7 @@
       <c r="G164" s="3" t="inlineStr"/>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -6741,17 +6759,17 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Start with a free consultation</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>დაიწყე უფასო კონსულტაციით</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Начните с бесплатной консультации</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr"/>
@@ -6778,7 +6796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H205"/>
+  <dimension ref="A1:H237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -6929,17 +6947,17 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Choosing the right CRM is hard</t>
+          <t>Choose the right CRM</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>სწორი CRM-ის შერჩევა რთულია</t>
+          <t>შეარჩიე სწორი CRM</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Выбрать правильную CRM сложно</t>
+          <t>Выберите правильную CRM</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -6969,22 +6987,26 @@
           <t>hero.headline.line2.accent</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>20 minutes with me</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>20 წუთი ჩემთან</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>20 минут со мной</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>and save</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>და დაზოგე</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>и сэкономьте</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7007,22 +7029,14 @@
           <t>hero.headline.line2.plain</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>saves you</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>დაგიზოგავს</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>сэкономят вам</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7045,22 +7059,26 @@
           <t>hero.headline.line3.underline</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>100+ hours</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>100+ საათიან</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>100+ საათი</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>100+ часов</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -7083,21 +7101,9 @@
           <t>hero.headline.line3.plain</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>of research and trials</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>კვლევას და ტესტირებას</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>исследований и тестов</t>
-        </is>
-      </c>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Only on this landing</t>
@@ -7127,17 +7133,17 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>With 500+ successful implementations behind us, in 20 minutes I'll tell you which CRM fits your sales, what implementation costs and how fast it can go live. Free if you book now.</t>
+          <t>With 500+ implementations behind us, in 20 minutes we tell you which CRM fits your sales and what implementation costs. Free if you book now.</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>500+ წარმატებული დანერგვის გამოცდილებით, 20 წუთში მოგიყვები, რომელი CRM მოერგება შენს გაყიდვებს, რა ეღირება დანერგვა და რამდენ ხანში ამუშავდება. უფასოდ - თუ ახლავე დაჯავშნი.</t>
+          <t>500+ დანერგვის გამოცდილებით 20 წუთში გეტყვით, რომელი CRM მოერგება შენს გაყიდვებს და რა ეღირება დანერგვა. უფასოდ - თუ ახლავე დაჯავშნი.</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Опираясь на 500+ успешных внедрений, за 20 минут расскажу, какая CRM подойдёт вашим продажам, сколько стоит внедрение и как быстро она заработает. Бесплатно - если бронируете сейчас.</t>
+          <t>Опираясь на 500+ внедрений, за 20 минут скажем, какая CRM подойдёт вашим продажам и сколько стоит внедрение. Бесплатно - если бронируете сейчас.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -7245,17 +7251,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე უფასო ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -10673,17 +10679,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a Call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -10823,22 +10829,26 @@
           <t>faq.q1</t>
         </is>
       </c>
-      <c r="D106" s="3" t="inlineStr">
-        <is>
-          <t>How is this different from hiring a Zoho / Monday / ClickUp partner directly?</t>
-        </is>
-      </c>
-      <c r="E106" s="3" t="inlineStr">
-        <is>
-          <t>რით განსხვავდება ეს უშუალოდ Zoho-ს, Monday-ს ან ClickUp-ის პარტნიორის დაქირავებისგან?</t>
-        </is>
-      </c>
-      <c r="F106" s="3" t="inlineStr">
-        <is>
-          <t>Чем это отличается от работы напрямую с партнёром Zoho / Monday / ClickUp?</t>
-        </is>
-      </c>
-      <c r="G106" s="3" t="inlineStr"/>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>How are you different from a single-CRM partner?</t>
+        </is>
+      </c>
+      <c r="E106" s="9" t="inlineStr">
+        <is>
+          <t>რით განსხვავდებით კონკრეტული CRM-ის პარტნიორისგან?</t>
+        </is>
+      </c>
+      <c r="F106" s="9" t="inlineStr">
+        <is>
+          <t>Чем вы отличаетесь от партнёра одной CRM?</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -10861,22 +10871,26 @@
           <t>faq.a1</t>
         </is>
       </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>We're vendor-neutral. Zoho partners sell Zoho, Monday partners sell Monday. We tell you honestly which platform fits your case, and if it isn't a platform we work with, we say so. The 20-minute call is where we find out which one you need.</t>
-        </is>
-      </c>
-      <c r="E107" s="3" t="inlineStr">
-        <is>
-          <t>ჩვენ სრულიად დამოუკიდებლები (vendor-neutral) ვართ. Zoho-ს პარტნიორი გთავაზობს მხოლოდ Zoho-ს, Monday-ს პარტნიორი - Monday-ს. ჩვენ გულწრფელად გირჩევთ იმ სისტემას, რომელიც რეალურად მოერგება შენს ბიზნესს; და თუ ისეთ ხელსაწყოზეა საუბარი, რომელთანაც არ ვმუშაობთ, პირდაპირ გეტყვით. 20-წუთიანი ზარი სწორედ იმისთვისაა, რომ გავარკვიოთ, რა გჭირდება რეალურად.</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="inlineStr">
-        <is>
-          <t>Мы вендор-нейтральны. Партнёр Zoho продаёт Zoho, партнёр Monday - Monday. Мы честно говорим, какая платформа подходит именно вам, и если это не та, с которой мы работаем - так и скажем. 20-минутный звонок как раз о том, чтобы это выяснить.</t>
-        </is>
-      </c>
-      <c r="G107" s="3" t="inlineStr"/>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>We're vendor-neutral. A Zoho partner offers only Zoho, a Bitrix24 partner only Bitrix24. We recommend the system that actually fits your sales, and if the best option is one we don't implement, we tell you so.</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>ვართ დამოუკიდებელი (vendor-neutral). Zoho-ს პარტნიორი გთავაზობს მხოლოდ Zoho-ს, Bitrix24-ის პარტნიორი მხოლოდ Bitrix24-ს. ჩვენ გირჩევთ იმ სისტემას, რომელიც რეალურად მოერგება შენს გაყიდვებს, და თუ საუკეთესო ვარიანტი ისეთი სისტემაა, რომელსაც ჩვენ არ ვნერგავთ, ამასაც პირდაპირ გეტყვით.</t>
+        </is>
+      </c>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>Мы независимы (vendor-neutral). Партнёр Zoho предлагает только Zoho, партнёр Bitrix24 - только Bitrix24. Мы советуем систему, которая действительно подходит вашим продажам, а если лучший вариант - система, которую мы не внедряем, прямо скажем об этом.</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -10899,22 +10913,26 @@
           <t>faq.q2</t>
         </is>
       </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>Why only one sprint instead of a full roadmap?</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>რატომ ვიწყებთ ერთი კონკრეტული სპრინტით და არა გრძელვადიანი გეგმით?</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>Почему только один спринт, а не полная дорожная карта?</t>
-        </is>
-      </c>
-      <c r="G108" s="3" t="inlineStr"/>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>Which CRMs do you implement?</t>
+        </is>
+      </c>
+      <c r="E108" s="9" t="inlineStr">
+        <is>
+          <t>რომელ CRM-ებს ნერგავთ?</t>
+        </is>
+      </c>
+      <c r="F108" s="9" t="inlineStr">
+        <is>
+          <t>Какие CRM вы внедряете?</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -10937,22 +10955,26 @@
           <t>faq.a2</t>
         </is>
       </c>
-      <c r="D109" s="3" t="inlineStr">
-        <is>
-          <t>Because 31% of IT projects actually succeed, and the ones that fail usually failed because they were too big. We ship one real thing in 10-15 days, your team adopts it, then Sprint 2 is informed by what you learned. No lock-in, no 6-month contract.</t>
-        </is>
-      </c>
-      <c r="E109" s="3" t="inlineStr">
-        <is>
-          <t>იმიტომ, რომ IT პროექტების მხოლოდ 31% სრულდება წარმატებით, ჩავარდნის მთავარი მიზეზი კი ხშირად მათი ზედმეტი სირთულე და მოცულობაა. ჩვენ ვნერგავთ ერთ კონკრეტულ, გამართულ ფუნქციონალს 10-15 დღეში, შენი გუნდი უპრობლემოდ ითვისებს მას, მეორე სპრინტი კი უკვე მიღებულ პრაქტიკულ გამოცდილებას ეფუძნება. არანაირი ხელოვნური მიბმა და 6-თვიანი სავალდებულო კონტრაქტები.</t>
-        </is>
-      </c>
-      <c r="F109" s="3" t="inlineStr">
-        <is>
-          <t>Потому что успешны лишь 31% IT-проектов, а провалы обычно случаются из-за того, что проект слишком большой. Мы запускаем одну реальную вещь за 10-15 дней, команда её осваивает, а Спринт 2 строится уже на этом опыте. Никакой привязки, никаких шестимесячных контрактов.</t>
-        </is>
-      </c>
-      <c r="G109" s="3" t="inlineStr"/>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>We're a certified partner of Zoho, Pipedrive, Kommo, monday.com, Bitrix24 and Odoo (and also ClickUp and Manychat). On the call we tell you which one fits your team, processes and budget.</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>ვართ Zoho-ს, Pipedrive-ის, Kommo-ს, monday.com-ის, Bitrix24-ისა და Odoo-ს სერტიფიცირებული პარტნიორი (ასევე ClickUp-ის და Manychat-ის). ზარზე გეტყვით, რომელი ერგება შენს გუნდს, პროცესებს და ბიუჯეტს.</t>
+        </is>
+      </c>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>Мы сертифицированный партнёр Zoho, Pipedrive, Kommo, monday.com, Bitrix24 и Odoo (а также ClickUp и Manychat). На звонке скажем, какая подходит вашей команде, процессам и бюджету.</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H109" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -10975,22 +10997,26 @@
           <t>faq.q3</t>
         </is>
       </c>
-      <c r="D110" s="3" t="inlineStr">
-        <is>
-          <t>What does it actually cost?</t>
-        </is>
-      </c>
-      <c r="E110" s="3" t="inlineStr">
-        <is>
-          <t>რეალურად რა ჯდება მომსახურება?</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="inlineStr">
-        <is>
-          <t>Сколько это стоит на деле?</t>
-        </is>
-      </c>
-      <c r="G110" s="3" t="inlineStr"/>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>What does a CRM implementation cost?</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="inlineStr">
+        <is>
+          <t>რა ჯდება CRM-ის დანერგვა?</t>
+        </is>
+      </c>
+      <c r="F110" s="9" t="inlineStr">
+        <is>
+          <t>Сколько стоит внедрение CRM?</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11013,22 +11039,26 @@
           <t>faq.a3</t>
         </is>
       </c>
-      <c r="D111" s="3" t="inlineStr">
-        <is>
-          <t>Minimum engagement is €1,990 + VAT. Most first sprints land €2,000-5,000 depending on which solutions you pick. Licensing (Zoho, Monday, etc.) is billed separately by the vendor at their public prices. We tell you both numbers on the call.</t>
-        </is>
-      </c>
-      <c r="E111" s="3" t="inlineStr">
-        <is>
-          <t>მინიმალური ჩართულობა შეადგენს €1,990-ს (+ დღგ). პირველი სპრინტების უმრავლესობის ღირებულება შერჩეული გადაწყვეტების მიხედვით €2,000-დან €5,000-მდე მერყეობს. პლატფორმის ლიცენზიებს (Zoho, Monday და ა.შ.) პირდაპირ მწარმოებელს უხდით მათი ოფიციალური საჯარო ტარიფებით. ორივე ციფრს ზარზე დეტალურად დაგითვლით.</t>
-        </is>
-      </c>
-      <c r="F111" s="3" t="inlineStr">
-        <is>
-          <t>Минимальный заказ - €1,990 + НДС. Большинство первых спринтов - €2,000-5,000 в зависимости от выбранных решений. Лицензии (Zoho, Monday и т.д.) оплачиваются отдельно напрямую вендору по его публичным ценам. Обе цифры называем на звонке.</t>
-        </is>
-      </c>
-      <c r="G111" s="3" t="inlineStr"/>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>The price is set individually: it depends on the number of users, your processes, data migration and integrations. You pay the CRM licence directly to the vendor at its official price; we charge for the implementation. We give you both numbers on the 20-minute call.</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>ღირებულება ინდივიდუალურად განისაზღვრება: დამოკიდებულია მომხმარებლების რაოდენობაზე, პროცესებზე, მონაცემების გადმოტანასა და ინტეგრაციებზე. CRM-ის ლიცენზიას პირდაპირ მწარმოებელს უხდი მისი ოფიციალური ფასით, ჩვენ კი ვიღებთ დანერგვის საფასურს. ორივე ციფრს 20-წუთიან ზარზე გეტყვით.</t>
+        </is>
+      </c>
+      <c r="F111" s="9" t="inlineStr">
+        <is>
+          <t>Стоимость определяется индивидуально: зависит от числа пользователей, процессов, переноса данных и интеграций. Лицензию CRM вы оплачиваете напрямую производителю по официальной цене, а мы берём плату за внедрение. Обе цифры назовём на 20-минутном звонке.</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11051,22 +11081,26 @@
           <t>faq.q4</t>
         </is>
       </c>
-      <c r="D112" s="3" t="inlineStr">
-        <is>
-          <t>Do you work with my industry?</t>
-        </is>
-      </c>
-      <c r="E112" s="3" t="inlineStr">
-        <is>
-          <t>მუშაობთ თუ არა ჩემს კონკრეტულ ინდუსტრიაში?</t>
-        </is>
-      </c>
-      <c r="F112" s="3" t="inlineStr">
-        <is>
-          <t>Вы работаете в моей отрасли?</t>
-        </is>
-      </c>
-      <c r="G112" s="3" t="inlineStr"/>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>How long does implementation take?</t>
+        </is>
+      </c>
+      <c r="E112" s="9" t="inlineStr">
+        <is>
+          <t>რამდენ ხანს გრძელდება დანერგვა?</t>
+        </is>
+      </c>
+      <c r="F112" s="9" t="inlineStr">
+        <is>
+          <t>Сколько длится внедрение?</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11089,22 +11123,26 @@
           <t>faq.a4</t>
         </is>
       </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>We've deployed in real estate, education, logistics, hospitality, medical, retail, finance, construction, and services. If your work is on an Excel sheet, a shared inbox, or a WhatsApp group right now, we can help. If you need something only a very narrow vertical tool does (legal case management, specific medical records), we'll tell you.</t>
-        </is>
-      </c>
-      <c r="E113" s="3" t="inlineStr">
-        <is>
-          <t>ჩვენ განვახორციელეთ დანერგვები უძრავ ქონებაში, განათლებაში, ლოგისტიკაში, HoReCa სექტორში, მედიცინაში, რითეილში, ფინანსებში, მშენებლობასა და მომსახურების სფეროში. თუ დღეს შენი საქმე იმართება Excel-ის ცხრილებით, საერთო მეილით ან WhatsApp-ის ჩატებით - ჩვენ შეგვიძლია შენი დახმარება. ხოლო თუ სპეციფიკური ვიწრო-პროფილური სისტემა გჭირდება (მაგ. იურიდიული საქმისწარმოება ან სპეციფიკური სამედიცინო ბარათები), ამასაც პირდაპირ გეტყვით.</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>Мы внедряли в недвижимости, образовании, логистике, гостеприимстве, медицине, рознице, финансах, строительстве и сервисах. Если вы сейчас работаете в Excel, общем inbox или WhatsApp-группе - мы поможем. Если нужен узкоспециализированный вертикальный инструмент (управление юридическими кейсами, медицинские записи) - честно скажем.</t>
-        </is>
-      </c>
-      <c r="G113" s="3" t="inlineStr"/>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>A core CRM (sales stages, fields, data migration, team training) usually goes live in 1-2 weeks. We start with what matters most, your team adopts it, then we add automations and integrations. That keeps risk low and you see results fast.</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>საბაზისო CRM (გაყიდვების ეტაპები, ველები, მონაცემების გადმოტანა, გუნდის ტრენინგი) როგორც წესი 1-2 კვირაში ეშვება. ვიწყებთ ყველაზე მნიშვნელოვანით, გუნდი ითვისებს და მერე ვამატებთ ავტომატიზაციებსა და ინტეგრაციებს. ასე რისკი მინიმალურია და შედეგს სწრაფად ხედავ.</t>
+        </is>
+      </c>
+      <c r="F113" s="9" t="inlineStr">
+        <is>
+          <t>Базовая CRM (этапы продаж, поля, перенос данных, обучение команды) обычно запускается за 1-2 недели. Начинаем с самого важного, команда осваивает систему, затем добавляем автоматизации и интеграции. Так риск минимален, а результат виден быстро.</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11127,22 +11165,26 @@
           <t>faq.q5</t>
         </is>
       </c>
-      <c r="D114" s="3" t="inlineStr">
-        <is>
-          <t>What if I don't know what my problem is?</t>
-        </is>
-      </c>
-      <c r="E114" s="3" t="inlineStr">
-        <is>
-          <t>რა ვქნა, თუ ზუსტად არ ვიცი, რა არის ჩემი მთავარი პრობლემა?</t>
-        </is>
-      </c>
-      <c r="F114" s="3" t="inlineStr">
-        <is>
-          <t>А если я не знаю, в чём моя проблема?</t>
-        </is>
-      </c>
-      <c r="G114" s="3" t="inlineStr"/>
+      <c r="D114" s="9" t="inlineStr">
+        <is>
+          <t>Can you move our data from Excel or another CRM?</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="inlineStr">
+        <is>
+          <t>შეგიძლიათ მონაცემები Excel-იდან ან სხვა CRM-იდან გადმოიტანოთ?</t>
+        </is>
+      </c>
+      <c r="F114" s="9" t="inlineStr">
+        <is>
+          <t>Можете перенести данные из Excel или другой CRM?</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11165,22 +11207,26 @@
           <t>faq.a5</t>
         </is>
       </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>That's what the 20 minutes are for. Most founders arrive with a vague "I need a CRM" and leave with a specific one-page plan. If after the call it's still unclear, we offer a paid Discovery (€99/h) to go deeper - only when it genuinely helps.</t>
-        </is>
-      </c>
-      <c r="E115" s="3" t="inlineStr">
-        <is>
-          <t>20-წუთიანი ზარი სწორედ ამისთვისაა. დამფუძნებლების უმეტესობა მოდის ზოგადი ფრაზით „CRM მჭირდება“ და ზარიდან გადის კონკრეტული 1-გვერდიანი სამოქმედო გეგმით. თუ ზარის შემდეგ მაინც საჭირო გახდა სიღრმისეული ანალიზი, გთავაზობთ ფასიან Discovery სესიას (€99/სთ) - მხოლოდ იმ შემთხვევაში, თუ ეს რეალურ სარგებელს მოგიტანს.</t>
-        </is>
-      </c>
-      <c r="F115" s="3" t="inlineStr">
-        <is>
-          <t>Для этого и нужны 20 минут. Большинство основателей приходят с размытым "мне нужна CRM", а уходят с конкретным планом на одну страницу. Если после звонка всё ещё непонятно - предлагаем платный Discovery (€99/ч), чтобы копнуть глубже. Только если это реально поможет.</t>
-        </is>
-      </c>
-      <c r="G115" s="3" t="inlineStr"/>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>Yes. We move clients, contacts, deals and history from Excel, Google Sheets or another CRM. Before the move we clean duplicates and normalise phone numbers, so the new system starts with a clean database.</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="inlineStr">
+        <is>
+          <t>კი. კლიენტებს, კონტაქტებს, გარიგებებს და ისტორიას გადმოვიტანთ Excel-იდან, Google Sheets-იდან ან სხვა CRM-იდან. გადმოტანამდე ვასუფთავებთ დუბლიკატებს და ვაწესრიგებთ ტელეფონის ნომრებს, რომ ახალი სისტემა სუფთა ბაზით დაიწყოს.</t>
+        </is>
+      </c>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>Да. Переносим клиентов, контакты, сделки и историю из Excel, Google Sheets или другой CRM. Перед переносом чистим дубликаты и приводим номера телефонов к единому формату, чтобы новая система стартовала с чистой базой.</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H115" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11203,22 +11249,26 @@
           <t>faq.q6</t>
         </is>
       </c>
-      <c r="D116" s="3" t="inlineStr">
-        <is>
-          <t>Who owns the system you build?</t>
-        </is>
-      </c>
-      <c r="E116" s="3" t="inlineStr">
-        <is>
-          <t>ვის საკუთრებაში რჩება აწყობილი სისტემა?</t>
-        </is>
-      </c>
-      <c r="F116" s="3" t="inlineStr">
-        <is>
-          <t>Кому принадлежит система, которую вы строите?</t>
-        </is>
-      </c>
-      <c r="G116" s="3" t="inlineStr"/>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>Can the CRM connect chats, website forms and telephony?</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="inlineStr">
+        <is>
+          <t>შეიძლება CRM-ს ჩატები, საიტის ფორმები და ტელეფონია მივაბა?</t>
+        </is>
+      </c>
+      <c r="F116" s="9" t="inlineStr">
+        <is>
+          <t>Можно подключить к CRM чаты, формы сайта и телефонию?</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11241,22 +11291,26 @@
           <t>faq.a6</t>
         </is>
       </c>
-      <c r="D117" s="3" t="inlineStr">
-        <is>
-          <t>You own all your data and all platform accounts - they're registered under your company. The implementation IP (configurations, custom code) belongs to us, but you can take your data anywhere, anytime. Anything we host on our side is a transparent paid subscription you can cancel.</t>
-        </is>
-      </c>
-      <c r="E117" s="3" t="inlineStr">
-        <is>
-          <t>ყველა შენი მონაცემი და პლატფორმის ანგარიში რეგისტრირდება შენი კომპანიის სახელზე და რჩება შენს სრულ მფლობელობაში. დანერგვის ინტელექტუალური საკუთრება (კონფიგურაცია, custom კოდი) ეკუთვნის ჩვენს გუნდს, თუმცა შენი მონაცემების ექსპორტი და წაღება ნებისმიერ დროს შეგიძლია. ნებისმიერი სერვისი, რომელსაც ჩვენს მხარეს ვჰოსტავთ, წარმოადგენს გამჭვირვალე ყოველთვიურ გამოწერას, რომლის გაუქმებაც ნებისმიერ მომენტშია შესაძლებელი.</t>
-        </is>
-      </c>
-      <c r="F117" s="3" t="inlineStr">
-        <is>
-          <t>Все ваши данные и аккаунты платформ принадлежат вам - они зарегистрированы на вашу компанию. Интеллектуальная собственность на внедрение (конфигурации, кастомный код) принадлежит нам, но данные вы можете забрать куда угодно и когда угодно. Всё, что мы хостим у себя - прозрачная платная подписка, её можно отменить.</t>
-        </is>
-      </c>
-      <c r="G117" s="3" t="inlineStr"/>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>Yes. WhatsApp, Instagram, Facebook Messenger, website forms, Meta ad leads and telephony (including GEONET) can all land in one CRM, so every request is in one place. On the call we confirm what connects to the CRM you choose and how.</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="inlineStr">
+        <is>
+          <t>კი. WhatsApp, Instagram, Facebook Messenger, საიტის ფორმები, Meta-ს რეკლამის ლიდები და ტელეფონია (მათ შორის GEONET) შეგვიძლია ერთ CRM-ში შევკრიბოთ, რომ ყველა მომართვა ერთ ადგილას ჩანდეს. რა და როგორ უკავშირდება შენს არჩეულ CRM-ს, ზარზე დაგიზუსტებთ.</t>
+        </is>
+      </c>
+      <c r="F117" s="9" t="inlineStr">
+        <is>
+          <t>Да. WhatsApp, Instagram, Facebook Messenger, формы сайта, лиды из рекламы Meta и телефонию (включая GEONET) можно собрать в одной CRM, чтобы все обращения были в одном месте. Что и как подключается к выбранной CRM, уточним на звонке.</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11279,22 +11333,26 @@
           <t>faq.q7</t>
         </is>
       </c>
-      <c r="D118" s="3" t="inlineStr">
-        <is>
-          <t>What happens after the sprint delivers?</t>
-        </is>
-      </c>
-      <c r="E118" s="3" t="inlineStr">
-        <is>
-          <t>რა ხდება სპრინტის დასრულებისა და ჩაბარების შემდეგ?</t>
-        </is>
-      </c>
-      <c r="F118" s="3" t="inlineStr">
-        <is>
-          <t>Что происходит после сдачи спринта?</t>
-        </is>
-      </c>
-      <c r="G118" s="3" t="inlineStr"/>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>Do you work with my industry?</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="inlineStr">
+        <is>
+          <t>მუშაობთ თუ არა ჩემს ინდუსტრიაში?</t>
+        </is>
+      </c>
+      <c r="F118" s="9" t="inlineStr">
+        <is>
+          <t>Работаете ли вы в моей отрасли?</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11317,22 +11375,26 @@
           <t>faq.a7</t>
         </is>
       </c>
-      <c r="D119" s="3" t="inlineStr">
-        <is>
-          <t>Three business days to review and accept. Then your team runs it. Technical support is available at €69/h - only if you need it. Many clients then book Sprint 2 (automations, integrations) or move to Managed Services for ongoing optimization.</t>
-        </is>
-      </c>
-      <c r="E119" s="3" t="inlineStr">
-        <is>
-          <t>გაქვს 3 სამუშაო დღე სისტემის შესამოწმებლად და ჩასაბარებლად, რის შემდეგაც შენი გუნდი სრულფასოვნად იწყებს მუშაობას. ტექნიკური მხარდაჭერა ხელმისაწვდომია ტარიფით €69/სთ - მხოლოდ საჭიროების შემთხვევაში. ბევრი კლიენტი შემდგომ ჯავშნის მეორე სპრინტს (ავტომატიზაციები, ინტეგრაციები) ან გადადის მუდმივი ოპტიმიზაციის მხარდაჭერის პაკეტზე (Managed Services).</t>
-        </is>
-      </c>
-      <c r="F119" s="3" t="inlineStr">
-        <is>
-          <t>Три рабочих дня на проверку и приёмку. Дальше система работает у вашей команды. Техподдержка доступна за €69/ч - только по необходимости. Многие клиенты затем бронируют Спринт 2 (автоматизация, интеграции) или переходят на Managed Services для постоянной оптимизации.</t>
-        </is>
-      </c>
-      <c r="G119" s="3" t="inlineStr"/>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>We've implemented CRM in real estate, education, logistics, hospitality, healthcare, retail, finance, construction and services. If your sales run on Excel, a shared inbox or WhatsApp chats today, we can help.</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="inlineStr">
+        <is>
+          <t>CRM დაგვინერგავს უძრავ ქონებაში, განათლებაში, ლოგისტიკაში, HoReCa სექტორში, მედიცინაში, რითეილში, ფინანსებში, მშენებლობასა და მომსახურების სფეროში. თუ დღეს გაყიდვები Excel-ში, საერთო მეილში ან WhatsApp-ის ჩატებში იმართება, შეგვიძლია დაგეხმაროთ.</t>
+        </is>
+      </c>
+      <c r="F119" s="9" t="inlineStr">
+        <is>
+          <t>Мы внедряли CRM в недвижимости, образовании, логистике, HoReCa, медицине, ритейле, финансах, строительстве и сфере услуг. Если сегодня продажи ведутся в Excel, общей почте или чатах WhatsApp, мы поможем.</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11355,22 +11417,26 @@
           <t>faq.q8</t>
         </is>
       </c>
-      <c r="D120" s="3" t="inlineStr">
-        <is>
-          <t>Can I pick 5 solutions and combine them?</t>
-        </is>
-      </c>
-      <c r="E120" s="3" t="inlineStr">
-        <is>
-          <t>შემიძლია ავირჩიო 5 სხვადასხვა გადაწყვეტა და ერთად გავაერთიანო?</t>
-        </is>
-      </c>
-      <c r="F120" s="3" t="inlineStr">
-        <is>
-          <t>Можно выбрать 5 решений и объединить их?</t>
-        </is>
-      </c>
-      <c r="G120" s="3" t="inlineStr"/>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>What if I don't know which CRM I need?</t>
+        </is>
+      </c>
+      <c r="E120" s="9" t="inlineStr">
+        <is>
+          <t>რა ვქნა, თუ არ ვიცი, რომელი CRM მჭირდება?</t>
+        </is>
+      </c>
+      <c r="F120" s="9" t="inlineStr">
+        <is>
+          <t>Что делать, если я не знаю, какая CRM мне нужна?</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11393,22 +11459,26 @@
           <t>faq.a8</t>
         </is>
       </c>
-      <c r="D121" s="3" t="inlineStr">
-        <is>
-          <t>Yes, that's what the "Add to request" list is for. On the call we help you order them by sequence (what has to come first) and sprint capacity. You usually won't ship all 5 at once, but you can.</t>
-        </is>
-      </c>
-      <c r="E121" s="3" t="inlineStr">
-        <is>
-          <t>რა თქმა უნდა! ღილაკი „სიაში დამატება“ სწორედ ამისთვისაა. ზარზე ერთად განვსაზღვრავთ პრიორიტეტებს - რა უნდა გაკეთდეს პირველ ეტაპზე და რა გადანაწილდეს შემდგომ სპრინტებზე. როგორც წესი, ხუთივე ერთდროულად არ ეშვება, თუმცა ტექნიკურად ეს სრულიად შესაძლებელია.</t>
-        </is>
-      </c>
-      <c r="F121" s="3" t="inlineStr">
-        <is>
-          <t>Да, именно для этого и существует список "Добавить в запрос". На звонке мы помогаем расставить их по порядку (что должно идти первым) и по ёмкости спринта. Обычно 5 сразу не внедряют, но технически это возможно.</t>
-        </is>
-      </c>
-      <c r="G121" s="3" t="inlineStr"/>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>That is exactly what the 20-minute call is for. Most people arrive with "I need a CRM" and leave with a specific recommendation: which system, what the licence and implementation cost, and how long it takes.</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="inlineStr">
+        <is>
+          <t>20-წუთიანი ზარი სწორედ ამისთვისაა. უმეტესობა მოდის ფრაზით „CRM მჭირდება“ და ზარიდან გადის კონკრეტული რეკომენდაციით: რომელი სისტემა, რა ეღირება ლიცენზია და დანერგვა, რა ვადაში ეშვება.</t>
+        </is>
+      </c>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>Для этого и нужен 20-минутный звонок. Большинство приходит с фразой «мне нужна CRM» и уходит с конкретной рекомендацией: какая система, сколько стоят лицензия и внедрение, за какой срок запускается.</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11431,22 +11501,26 @@
           <t>faq.q9</t>
         </is>
       </c>
-      <c r="D122" s="3" t="inlineStr">
-        <is>
-          <t>Do you work with international clients, or Georgia only?</t>
-        </is>
-      </c>
-      <c r="E122" s="3" t="inlineStr">
-        <is>
-          <t>მუშაობთ საერთაშორისო კლიენტებთან, თუ მხოლოდ საქართველოში?</t>
-        </is>
-      </c>
-      <c r="F122" s="3" t="inlineStr">
-        <is>
-          <t>Вы работаете с международными клиентами или только в Грузии?</t>
-        </is>
-      </c>
-      <c r="G122" s="3" t="inlineStr"/>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>What happens after launch?</t>
+        </is>
+      </c>
+      <c r="E122" s="9" t="inlineStr">
+        <is>
+          <t>რა ხდება დანერგვის შემდეგ?</t>
+        </is>
+      </c>
+      <c r="F122" s="9" t="inlineStr">
+        <is>
+          <t>Что происходит после запуска?</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H122" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11469,22 +11543,26 @@
           <t>faq.a9</t>
         </is>
       </c>
-      <c r="D123" s="3" t="inlineStr">
-        <is>
-          <t>We focus on Georgia because of language, local banking, and GEONET telephony integrations. We also serve select international clients - the call is in English or Russian or Georgian, whichever works for you.</t>
-        </is>
-      </c>
-      <c r="E123" s="3" t="inlineStr">
-        <is>
-          <t>ჩვენი მთავარი ფოკუსი საქართველოა ქართული ენის, ადგილობრივი ბანკინგისა და GEONET-ის ტელეფონიის ინტეგრაციების გამო. თუმცა ვთანამშრომლობთ შერჩეულ საერთაშორისო კლიენტებთანაც - საკონსულტაციო ზარი შეგვიძლია ჩავატაროთ ქართულად, ინგლისურად ან რუსულად, შენი სურვილისამებრ.</t>
-        </is>
-      </c>
-      <c r="F123" s="3" t="inlineStr">
-        <is>
-          <t>Мы сфокусированы на Грузии из-за языка, местного банкинга и интеграций с GEONET-телефонией. Работаем и с избранными международными клиентами - звонок на английском, русском или грузинском, как вам удобно.</t>
-        </is>
-      </c>
-      <c r="G123" s="3" t="inlineStr"/>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>You have 3 business days to review and accept the system, then your team works in the CRM. Technical support is available when you need it, and for those who want the system to keep improving we offer monthly support.</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr">
+        <is>
+          <t>გაქვს 3 სამუშაო დღე სისტემის შესამოწმებლად და ჩასაბარებლად, მერე გუნდი უკვე CRM-ში მუშაობს. ტექნიკური მხარდაჭერა ხელმისაწვდომია საჭიროებისამებრ, ხოლო ვისაც უნდა, რომ სისტემა მუდმივად ვითარდებოდეს, ვთავაზობთ ყოველთვიურ მხარდაჭერას.</t>
+        </is>
+      </c>
+      <c r="F123" s="9" t="inlineStr">
+        <is>
+          <t>У вас есть 3 рабочих дня, чтобы проверить и принять систему, после чего команда работает в CRM. Техподдержка доступна по необходимости, а тем, кто хочет постоянно развивать систему, предлагаем ежемесячное сопровождение.</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11507,22 +11585,26 @@
           <t>faq.q10</t>
         </is>
       </c>
-      <c r="D124" s="3" t="inlineStr">
-        <is>
-          <t>What if 20 minutes isn't enough?</t>
-        </is>
-      </c>
-      <c r="E124" s="3" t="inlineStr">
-        <is>
-          <t>რა მოხდება, თუ 20 წუთი საკმარისი არ აღმოჩნდება?</t>
-        </is>
-      </c>
-      <c r="F124" s="3" t="inlineStr">
-        <is>
-          <t>А если 20 минут не хватит?</t>
-        </is>
-      </c>
-      <c r="G124" s="3" t="inlineStr"/>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>Who owns the CRM and the data?</t>
+        </is>
+      </c>
+      <c r="E124" s="9" t="inlineStr">
+        <is>
+          <t>ვის საკუთრებაში რჩება CRM და მონაცემები?</t>
+        </is>
+      </c>
+      <c r="F124" s="9" t="inlineStr">
+        <is>
+          <t>Кому принадлежат CRM и данные?</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11545,22 +11627,26 @@
           <t>faq.a10</t>
         </is>
       </c>
-      <c r="D125" s="3" t="inlineStr">
-        <is>
-          <t>Then we schedule a second call, or you book paid Discovery. We've never had a founder arrive and leave more confused - the agenda is tight on purpose. If you have a complex multi-system case, mention it on the booking form and we'll block 45 minutes instead.</t>
-        </is>
-      </c>
-      <c r="E125" s="3" t="inlineStr">
-        <is>
-          <t>ასეთ შემთხვევაში დავნიშნავთ მეორე ზარს, ან შევთანხმდებით სიღრმისეულ Discovery-ზე. არ ყოფილა შემთხვევა, რომ დამფუძნებელი ჩვენი ზარიდან უფრო დაბნეული გასულიყო - დღის წესრიგი მიზანმიმართულად მკაფიო და ლაკონიურია. თუ გაქვს კომპლექსური, მრავალსისტემიანი ქეისი, უბრალოდ მიუთითე ჯავშნის ფორმაში და შენთვის წინასწარ 45 წუთს დავჯავშნით.</t>
-        </is>
-      </c>
-      <c r="F125" s="3" t="inlineStr">
-        <is>
-          <t>Тогда назначим второй звонок или вы бронируете платный Discovery. У нас не было случая, когда основатель уходил бы ещё более запутанным - повестка намеренно плотная. Если у вас сложный мульти-системный кейс, отметьте это в форме бронирования, и мы выделим 45 минут.</t>
-        </is>
-      </c>
-      <c r="G125" s="3" t="inlineStr"/>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>The CRM account and all data are registered to your company and stay fully yours. You can export your data at any time. Anything we host on our side is a transparent monthly subscription you can cancel at any time.</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>CRM-ის ანგარიში და ყველა მონაცემი რეგისტრირდება შენი კომპანიის სახელზე და რჩება შენს სრულ მფლობელობაში. მონაცემების ექსპორტი ნებისმიერ დროს შეგიძლია. თუ რამეს ჩვენს მხარეს ვჰოსტავთ, ეს არის გამჭვირვალე ყოველთვიური გამოწერა, რომელსაც ნებისმიერ დროს გააუქმებ.</t>
+        </is>
+      </c>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>Аккаунт CRM и все данные зарегистрированы на вашу компанию и полностью принадлежат вам. Экспортировать данные можно в любой момент. Всё, что мы размещаем на своей стороне, - прозрачная ежемесячная подписка, которую можно отменить в любое время.</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -11851,17 +11937,17 @@
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>Sound familiar?</t>
+          <t>Do these situations sound familiar?</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>ნაცნობია?</t>
+          <t>გეცნობა ეს სიტუაციები?</t>
         </is>
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>Знакомо?</t>
+          <t>Знакомы такие ситуации?</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr"/>
@@ -11927,17 +12013,17 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Request a free call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე უფასო ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G135" s="3" t="inlineStr"/>
@@ -13843,7 +13929,7 @@
       <c r="G185" s="3" t="inlineStr"/>
       <c r="H185" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -14565,7 +14651,7 @@
       <c r="G204" s="3" t="inlineStr"/>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -14587,17 +14673,17 @@
       </c>
       <c r="D205" s="3" t="inlineStr">
         <is>
-          <t>Start with a free consultation</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E205" s="3" t="inlineStr">
         <is>
-          <t>დაიწყე უფასო კონსულტაციით</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F205" s="3" t="inlineStr">
         <is>
-          <t>Начните с бесплатной консультации</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G205" s="3" t="inlineStr"/>
@@ -14607,10 +14693,1342 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>pain.manager.left</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>Ana left the chat</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>ანამ დატოვა ჩატი</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="inlineStr">
+        <is>
+          <t>Анна покинула чат</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr"/>
+      <c r="H206" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>pain.owner.note</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>Today!!</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>დღეს!!</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>Сегодня!!</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="inlineStr"/>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>pain.chats.more</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>+11 unanswered</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>+11 უპასუხო</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>+11 без ответа</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr"/>
+      <c r="H208" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>fit.title</t>
+        </is>
+      </c>
+      <c r="D209" s="9" t="inlineStr">
+        <is>
+          <t>Which CRM fits you?</t>
+        </is>
+      </c>
+      <c r="E209" s="9" t="inlineStr">
+        <is>
+          <t>რომელი CRM გერგება?</t>
+        </is>
+      </c>
+      <c r="F209" s="9" t="inlineStr">
+        <is>
+          <t>Какая CRM вам подходит?</t>
+        </is>
+      </c>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>fit.sub</t>
+        </is>
+      </c>
+      <c r="D210" s="9" t="inlineStr">
+        <is>
+          <t>We're an independent partner: we recommend what fits your sales, not what we'd like to sell.</t>
+        </is>
+      </c>
+      <c r="E210" s="9" t="inlineStr">
+        <is>
+          <t>ვართ დამოუკიდებელი პარტნიორი: გირჩევთ იმას, რაც შენს გაყიდვებს ერგება, და არა იმას, რისი გაყიდვაც გვინდა.</t>
+        </is>
+      </c>
+      <c r="F210" s="9" t="inlineStr">
+        <is>
+          <t>Мы независимый партнёр: советуем то, что подходит вашим продажам, а не то, что нам выгодно продать.</t>
+        </is>
+      </c>
+      <c r="G210" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>fit.zoho.when</t>
+        </is>
+      </c>
+      <c r="D211" s="9" t="inlineStr">
+        <is>
+          <t>When your processes are complex and you want deep customisation, automations and analytics in one ecosystem.</t>
+        </is>
+      </c>
+      <c r="E211" s="9" t="inlineStr">
+        <is>
+          <t>როცა პროცესები რთულია და გინდა ღრმა მორგება, ავტომატიზაციები და ანალიტიკა ერთ ეკოსისტემაში.</t>
+        </is>
+      </c>
+      <c r="F211" s="9" t="inlineStr">
+        <is>
+          <t>Когда процессы сложные и нужна глубокая настройка, автоматизации и аналитика в одной экосистеме.</t>
+        </is>
+      </c>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>fit.zoho.t1</t>
+        </is>
+      </c>
+      <c r="D212" s="9" t="inlineStr">
+        <is>
+          <t>Customisation</t>
+        </is>
+      </c>
+      <c r="E212" s="9" t="inlineStr">
+        <is>
+          <t>მორგება</t>
+        </is>
+      </c>
+      <c r="F212" s="9" t="inlineStr">
+        <is>
+          <t>Настройка</t>
+        </is>
+      </c>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>fit.zoho.t2</t>
+        </is>
+      </c>
+      <c r="D213" s="9" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="E213" s="9" t="inlineStr">
+        <is>
+          <t>ავტომატიზაცია</t>
+        </is>
+      </c>
+      <c r="F213" s="9" t="inlineStr">
+        <is>
+          <t>Автоматизация</t>
+        </is>
+      </c>
+      <c r="G213" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>fit.zoho.t3</t>
+        </is>
+      </c>
+      <c r="D214" s="9" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="E214" s="9" t="inlineStr">
+        <is>
+          <t>ანალიტიკა</t>
+        </is>
+      </c>
+      <c r="F214" s="9" t="inlineStr">
+        <is>
+          <t>Аналитика</t>
+        </is>
+      </c>
+      <c r="G214" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H214" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>fit.pipedrive.when</t>
+        </is>
+      </c>
+      <c r="D215" s="9" t="inlineStr">
+        <is>
+          <t>When your sales team needs a simple, visual pipeline and a fast start.</t>
+        </is>
+      </c>
+      <c r="E215" s="9" t="inlineStr">
+        <is>
+          <t>როცა გაყიდვების გუნდს მარტივი, ვიზუალური გაყიდვების ძაბრი და სწრაფი სტარტი სჭირდება.</t>
+        </is>
+      </c>
+      <c r="F215" s="9" t="inlineStr">
+        <is>
+          <t>Когда отделу продаж нужна простая наглядная воронка и быстрый старт.</t>
+        </is>
+      </c>
+      <c r="G215" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H215" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>fit.pipedrive.t1</t>
+        </is>
+      </c>
+      <c r="D216" s="9" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="E216" s="9" t="inlineStr">
+        <is>
+          <t>მარტივი</t>
+        </is>
+      </c>
+      <c r="F216" s="9" t="inlineStr">
+        <is>
+          <t>Просто</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H216" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>fit.pipedrive.t2</t>
+        </is>
+      </c>
+      <c r="D217" s="9" t="inlineStr">
+        <is>
+          <t>Visual pipeline</t>
+        </is>
+      </c>
+      <c r="E217" s="9" t="inlineStr">
+        <is>
+          <t>ვიზუალური ძაბრი</t>
+        </is>
+      </c>
+      <c r="F217" s="9" t="inlineStr">
+        <is>
+          <t>Наглядная воронка</t>
+        </is>
+      </c>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H217" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>fit.pipedrive.t3</t>
+        </is>
+      </c>
+      <c r="D218" s="9" t="inlineStr">
+        <is>
+          <t>Fast start</t>
+        </is>
+      </c>
+      <c r="E218" s="9" t="inlineStr">
+        <is>
+          <t>სწრაფი სტარტი</t>
+        </is>
+      </c>
+      <c r="F218" s="9" t="inlineStr">
+        <is>
+          <t>Быстрый старт</t>
+        </is>
+      </c>
+      <c r="G218" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H218" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>fit.kommo.when</t>
+        </is>
+      </c>
+      <c r="D219" s="9" t="inlineStr">
+        <is>
+          <t>When most of your sales happen in chats: WhatsApp, Instagram, Facebook.</t>
+        </is>
+      </c>
+      <c r="E219" s="9" t="inlineStr">
+        <is>
+          <t>როცა გაყიდვები ძირითადად ჩატებში მიდის: WhatsApp, Instagram, Facebook.</t>
+        </is>
+      </c>
+      <c r="F219" s="9" t="inlineStr">
+        <is>
+          <t>Когда продажи идут в основном в чатах: WhatsApp, Instagram, Facebook.</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>fit.kommo.t1</t>
+        </is>
+      </c>
+      <c r="D220" s="9" t="inlineStr">
+        <is>
+          <t>Chats</t>
+        </is>
+      </c>
+      <c r="E220" s="9" t="inlineStr">
+        <is>
+          <t>ჩატები</t>
+        </is>
+      </c>
+      <c r="F220" s="9" t="inlineStr">
+        <is>
+          <t>Чаты</t>
+        </is>
+      </c>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr">
+        <is>
+          <t>fit.kommo.t2</t>
+        </is>
+      </c>
+      <c r="D221" s="9" t="inlineStr">
+        <is>
+          <t>Messengers</t>
+        </is>
+      </c>
+      <c r="E221" s="9" t="inlineStr">
+        <is>
+          <t>მესენჯერები</t>
+        </is>
+      </c>
+      <c r="F221" s="9" t="inlineStr">
+        <is>
+          <t>Мессенджеры</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>fit.kommo.t3</t>
+        </is>
+      </c>
+      <c r="D222" s="9" t="inlineStr">
+        <is>
+          <t>Chatbots</t>
+        </is>
+      </c>
+      <c r="E222" s="9" t="inlineStr">
+        <is>
+          <t>ჩატბოტები</t>
+        </is>
+      </c>
+      <c r="F222" s="9" t="inlineStr">
+        <is>
+          <t>Чат-боты</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr">
+        <is>
+          <t>fit.monday.when</t>
+        </is>
+      </c>
+      <c r="D223" s="9" t="inlineStr">
+        <is>
+          <t>When you want to run sales and projects on the same flexible boards.</t>
+        </is>
+      </c>
+      <c r="E223" s="9" t="inlineStr">
+        <is>
+          <t>როცა გაყიდვები და პროექტები ერთ, მოქნილ დაფებზე გინდა მართო.</t>
+        </is>
+      </c>
+      <c r="F223" s="9" t="inlineStr">
+        <is>
+          <t>Когда хотите вести продажи и проекты на одних гибких досках.</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>fit.monday.t1</t>
+        </is>
+      </c>
+      <c r="D224" s="9" t="inlineStr">
+        <is>
+          <t>Flexible boards</t>
+        </is>
+      </c>
+      <c r="E224" s="9" t="inlineStr">
+        <is>
+          <t>მოქნილი დაფები</t>
+        </is>
+      </c>
+      <c r="F224" s="9" t="inlineStr">
+        <is>
+          <t>Гибкие доски</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>fit.monday.t2</t>
+        </is>
+      </c>
+      <c r="D225" s="9" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="E225" s="9" t="inlineStr">
+        <is>
+          <t>პროექტები</t>
+        </is>
+      </c>
+      <c r="F225" s="9" t="inlineStr">
+        <is>
+          <t>Проекты</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>fit.monday.t3</t>
+        </is>
+      </c>
+      <c r="D226" s="9" t="inlineStr">
+        <is>
+          <t>Teamwork</t>
+        </is>
+      </c>
+      <c r="E226" s="9" t="inlineStr">
+        <is>
+          <t>გუნდური მუშაობა</t>
+        </is>
+      </c>
+      <c r="F226" s="9" t="inlineStr">
+        <is>
+          <t>Командная работа</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H226" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>fit.bitrix.when</t>
+        </is>
+      </c>
+      <c r="D227" s="9" t="inlineStr">
+        <is>
+          <t>When you need internal chat, tasks and telephony in the same place as your CRM.</t>
+        </is>
+      </c>
+      <c r="E227" s="9" t="inlineStr">
+        <is>
+          <t>როცა CRM-თან ერთად შიდა ჩატი, დავალებები და ტელეფონია ერთ სივრცეში გჭირდება.</t>
+        </is>
+      </c>
+      <c r="F227" s="9" t="inlineStr">
+        <is>
+          <t>Когда рядом с CRM нужны внутренний чат, задачи и телефония в одном месте.</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H227" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>fit.bitrix.t1</t>
+        </is>
+      </c>
+      <c r="D228" s="9" t="inlineStr">
+        <is>
+          <t>Tasks</t>
+        </is>
+      </c>
+      <c r="E228" s="9" t="inlineStr">
+        <is>
+          <t>დავალებები</t>
+        </is>
+      </c>
+      <c r="F228" s="9" t="inlineStr">
+        <is>
+          <t>Задачи</t>
+        </is>
+      </c>
+      <c r="G228" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H228" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>fit.bitrix.t2</t>
+        </is>
+      </c>
+      <c r="D229" s="9" t="inlineStr">
+        <is>
+          <t>Internal chat</t>
+        </is>
+      </c>
+      <c r="E229" s="9" t="inlineStr">
+        <is>
+          <t>შიდა ჩატი</t>
+        </is>
+      </c>
+      <c r="F229" s="9" t="inlineStr">
+        <is>
+          <t>Внутренний чат</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>fit.bitrix.t3</t>
+        </is>
+      </c>
+      <c r="D230" s="9" t="inlineStr">
+        <is>
+          <t>Telephony</t>
+        </is>
+      </c>
+      <c r="E230" s="9" t="inlineStr">
+        <is>
+          <t>ტელეფონია</t>
+        </is>
+      </c>
+      <c r="F230" s="9" t="inlineStr">
+        <is>
+          <t>Телефония</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>fit.odoo.when</t>
+        </is>
+      </c>
+      <c r="D231" s="9" t="inlineStr">
+        <is>
+          <t>When you want inventory, invoicing and accounting in the same system as sales.</t>
+        </is>
+      </c>
+      <c r="E231" s="9" t="inlineStr">
+        <is>
+          <t>როცა გაყიდვებთან ერთად საწყობი, ინვოისები და ბუღალტერია ერთ სისტემაში გინდა.</t>
+        </is>
+      </c>
+      <c r="F231" s="9" t="inlineStr">
+        <is>
+          <t>Когда вместе с продажами нужны склад, счета и бухгалтерия в одной системе.</t>
+        </is>
+      </c>
+      <c r="G231" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H231" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>fit.odoo.t1</t>
+        </is>
+      </c>
+      <c r="D232" s="9" t="inlineStr">
+        <is>
+          <t>CRM + ERP</t>
+        </is>
+      </c>
+      <c r="E232" s="9" t="inlineStr">
+        <is>
+          <t>CRM + ERP</t>
+        </is>
+      </c>
+      <c r="F232" s="9" t="inlineStr">
+        <is>
+          <t>CRM + ERP</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H232" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr">
+        <is>
+          <t>fit.odoo.t2</t>
+        </is>
+      </c>
+      <c r="D233" s="9" t="inlineStr">
+        <is>
+          <t>Inventory</t>
+        </is>
+      </c>
+      <c r="E233" s="9" t="inlineStr">
+        <is>
+          <t>საწყობი</t>
+        </is>
+      </c>
+      <c r="F233" s="9" t="inlineStr">
+        <is>
+          <t>Склад</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>fit.odoo.t3</t>
+        </is>
+      </c>
+      <c r="D234" s="9" t="inlineStr">
+        <is>
+          <t>Invoicing</t>
+        </is>
+      </c>
+      <c r="E234" s="9" t="inlineStr">
+        <is>
+          <t>ინვოისები</t>
+        </is>
+      </c>
+      <c r="F234" s="9" t="inlineStr">
+        <is>
+          <t>Счета</t>
+        </is>
+      </c>
+      <c r="G234" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H234" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr">
+        <is>
+          <t>fit.foot.title</t>
+        </is>
+      </c>
+      <c r="D235" s="9" t="inlineStr">
+        <is>
+          <t>Not sure which one?</t>
+        </is>
+      </c>
+      <c r="E235" s="9" t="inlineStr">
+        <is>
+          <t>არ იცი, რომელი?</t>
+        </is>
+      </c>
+      <c r="F235" s="9" t="inlineStr">
+        <is>
+          <t>Не знаете, какую выбрать?</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>fit.foot.note</t>
+        </is>
+      </c>
+      <c r="D236" s="9" t="inlineStr">
+        <is>
+          <t>We'll choose together in 20 minutes. We're a certified partner of these platforms; you pay the licence directly to the vendor.</t>
+        </is>
+      </c>
+      <c r="E236" s="9" t="inlineStr">
+        <is>
+          <t>20 წუთში ერთად შევარჩევთ. ვართ ამ პლატფორმების სერტიფიცირებული პარტნიორები; ლიცენზიას პირდაპირ მწარმოებელს უხდი.</t>
+        </is>
+      </c>
+      <c r="F236" s="9" t="inlineStr">
+        <is>
+          <t>Выберем вместе за 20 минут. Мы сертифицированный партнёр этих платформ; лицензию вы оплачиваете напрямую производителю.</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H236" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>fit.cta</t>
+        </is>
+      </c>
+      <c r="D237" s="9" t="inlineStr">
+        <is>
+          <t>Request a free 20-minute call</t>
+        </is>
+      </c>
+      <c r="E237" s="9" t="inlineStr">
+        <is>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+        </is>
+      </c>
+      <c r="F237" s="9" t="inlineStr">
+        <is>
+          <t>Запросить бесплатный 20-минутный звонок</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H205"/>
+  <autoFilter ref="A1:H237"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H404" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H436" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -14624,7 +16042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H205"/>
+  <dimension ref="A1:H208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -15091,17 +16509,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე უფასო ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -18519,17 +19937,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a Call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -19697,17 +21115,17 @@
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>Sound familiar?</t>
+          <t>Do these situations sound familiar?</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>ნაცნობია?</t>
+          <t>გეცნობა ეს სიტუაციები?</t>
         </is>
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>Знакомо?</t>
+          <t>Знакомы такие ситуации?</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr"/>
@@ -19773,17 +21191,17 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Request a free call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე უფასო ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G135" s="3" t="inlineStr"/>
@@ -21693,7 +23111,7 @@
       <c r="G185" s="3" t="inlineStr"/>
       <c r="H185" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -22415,7 +23833,7 @@
       <c r="G204" s="3" t="inlineStr"/>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -22437,17 +23855,17 @@
       </c>
       <c r="D205" s="3" t="inlineStr">
         <is>
-          <t>Start with a free consultation</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E205" s="3" t="inlineStr">
         <is>
-          <t>დაიწყე უფასო კონსულტაციით</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F205" s="3" t="inlineStr">
         <is>
-          <t>Начните с бесплатной консультации</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G205" s="3" t="inlineStr"/>
@@ -22457,10 +23875,124 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>pain.manager.left</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>Ana left the chat</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>ანამ დატოვა ჩატი</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="inlineStr">
+        <is>
+          <t>Анна покинула чат</t>
+        </is>
+      </c>
+      <c r="G206" s="3" t="inlineStr"/>
+      <c r="H206" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>pain.owner.note</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>Today!!</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>დღეს!!</t>
+        </is>
+      </c>
+      <c r="F207" s="3" t="inlineStr">
+        <is>
+          <t>Сегодня!!</t>
+        </is>
+      </c>
+      <c r="G207" s="3" t="inlineStr"/>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>pain.chats.more</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>+11 unanswered</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>+11 უპასუხო</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>+11 без ответа</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr"/>
+      <c r="H208" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H205"/>
+  <autoFilter ref="A1:H208"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H404" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H407" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -22941,17 +24473,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე უფასო ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -26369,17 +27901,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a Call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -28019,7 +29551,7 @@
       <c r="G145" s="3" t="inlineStr"/>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -28741,7 +30273,7 @@
       <c r="G164" s="3" t="inlineStr"/>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -28763,17 +30295,17 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Start with a free consultation</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>დაიწყე უფასო კონსულტაციით</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Начните с бесплатной консультации</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr"/>
@@ -29263,17 +30795,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე უფასო ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -32683,17 +34215,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a Call</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე ზარი</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить звонок</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -34333,7 +35865,7 @@
       <c r="G145" s="3" t="inlineStr"/>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -35055,7 +36587,7 @@
       <c r="G164" s="3" t="inlineStr"/>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>New</t>
         </is>
       </c>
     </row>
@@ -35077,17 +36609,17 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Start with a free consultation</t>
+          <t>Request a free 20-minute call</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>დაიწყე უფასო კონსულტაციით</t>
+          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Начните с бесплатной консультации</t>
+          <t>Запросить бесплатный 20-минутный звонок</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr"/>
@@ -35576,7 +37108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -36487,7 +38019,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Choose a slot that works for you</t>
+          <t>Choose a time that works for you</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -36705,10 +38237,48 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Thank-you (all landings)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>ty.bonus.text</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Your bonus: &lt;b&gt;Productivity Stack 2026&lt;/b&gt; - 10 tools for research, call transcripts, scheduling, analytics, CRM and automation. For each: what it is for, why this one, and the setting most people miss.</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>შენი ბონუსი: &lt;b&gt;Productivity Stack 2026&lt;/b&gt; - 10 ინსტრუმენტი კვლევისთვის, ზარების ტრანსკრიპტისთვის, დაგეგმვისთვის, ანალიტიკისთვის, CRM-ისთვის და ავტომატიზაციისთვის. თითოეულზე: რისთვის, რატომ და რომელი პარამეტრი გამოგრჩება.</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Ваш бонус: &lt;b&gt;Productivity Stack 2026&lt;/b&gt; - 10 инструментов для исследований, транскрипции звонков, планирования, аналитики, CRM и автоматизации. Для каждого: для чего, почему именно он и какую настройку обычно упускают.</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H27"/>
+  <autoFilter ref="A1:H28"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H227" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
v61 style + crm-v62
</commit_message>
<xml_diff>
--- a/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
+++ b/Claude outputs/Unitty Solutions — Translations (EN_KA_RU).xlsx
@@ -13,11 +13,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed keys" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Start'!$A$1:$H$166</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CRM'!$A$1:$H$291</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AI'!$A$1:$H$284</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Banks'!$A$1:$H$166</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Solutions'!$A$1:$H$177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Start'!$A$1:$H$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CRM'!$A$1:$H$292</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'AI'!$A$1:$H$285</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Banks'!$A$1:$H$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Solutions'!$A$1:$H$178</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Thank-you'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:H167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -798,7 +798,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>კვლევას და ძიებას</t>
+          <t>კვლევას</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -945,17 +945,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -4365,17 +4365,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -5353,17 +5353,17 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>დარეკვა</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Позвонить</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr"/>
@@ -6759,17 +6759,17 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr"/>
@@ -6821,10 +6821,48 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>Nav</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>nav.cta</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>Free call</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>უფასო ზარი</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>Бесплатный звонок</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="inlineStr"/>
+      <c r="H167" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H166"/>
+  <autoFilter ref="A1:H167"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H365" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H366" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6838,7 +6876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H291"/>
+  <dimension ref="A1:H292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -7285,17 +7323,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -10709,17 +10747,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -11777,17 +11815,17 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>დარეკვა</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Позвонить</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr"/>
@@ -13231,17 +13269,17 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr"/>
@@ -13301,34 +13339,30 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Nav</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>process.go</t>
-        </is>
-      </c>
-      <c r="D167" s="9" t="inlineStr">
-        <is>
-          <t>Request now</t>
-        </is>
-      </c>
-      <c r="E167" s="9" t="inlineStr">
-        <is>
-          <t>მოითხოვე ახლავე</t>
-        </is>
-      </c>
-      <c r="F167" s="9" t="inlineStr">
-        <is>
-          <t>Запросить сейчас</t>
-        </is>
-      </c>
-      <c r="G167" s="3" t="inlineStr">
-        <is>
-          <t>Only on this landing</t>
-        </is>
-      </c>
+          <t>nav.cta</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>Free call</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>უფასო ზარი</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>Бесплатный звонок</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="inlineStr"/>
       <c r="H167" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -13343,27 +13377,27 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>Cp</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>cp.cx.p</t>
+          <t>process.go</t>
         </is>
       </c>
       <c r="D168" s="9" t="inlineStr">
         <is>
-          <t>Excel slows sales down and creates risks</t>
+          <t>Request now</t>
         </is>
       </c>
       <c r="E168" s="9" t="inlineStr">
         <is>
-          <t>Excel ანელებს გაყიდვებს და ქმნის რისკებს</t>
+          <t>მოითხოვე ახლავე</t>
         </is>
       </c>
       <c r="F168" s="9" t="inlineStr">
         <is>
-          <t>Excel тормозит продажи и создаёт риски</t>
+          <t>Запросить сейчас</t>
         </is>
       </c>
       <c r="G168" s="3" t="inlineStr">
@@ -13390,22 +13424,22 @@
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>cp.cx.s</t>
+          <t>cp.cx.p</t>
         </is>
       </c>
       <c r="D169" s="9" t="inlineStr">
         <is>
-          <t>Zoho CRM: every deal in one system</t>
+          <t>Excel slows sales down and creates risks</t>
         </is>
       </c>
       <c r="E169" s="9" t="inlineStr">
         <is>
-          <t>Zoho CRM: ყველა გარიგება ერთ სისტემაში</t>
+          <t>Excel ანელებს გაყიდვებს და ქმნის რისკებს</t>
         </is>
       </c>
       <c r="F169" s="9" t="inlineStr">
         <is>
-          <t>Zoho CRM: все сделки в одной системе</t>
+          <t>Excel тормозит продажи и создаёт риски</t>
         </is>
       </c>
       <c r="G169" s="3" t="inlineStr">
@@ -13432,22 +13466,22 @@
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>cp.cc.p</t>
+          <t>cp.cx.s</t>
         </is>
       </c>
       <c r="D170" s="9" t="inlineStr">
         <is>
-          <t>Work without a system creates chaos</t>
+          <t>Zoho CRM: every deal in one system</t>
         </is>
       </c>
       <c r="E170" s="9" t="inlineStr">
         <is>
-          <t>არასისტემური მუშაობა ქაოსს ქმნის</t>
+          <t>Zoho CRM: ყველა გარიგება ერთ სისტემაში</t>
         </is>
       </c>
       <c r="F170" s="9" t="inlineStr">
         <is>
-          <t>Работа без системы создаёт хаос</t>
+          <t>Zoho CRM: все сделки в одной системе</t>
         </is>
       </c>
       <c r="G170" s="3" t="inlineStr">
@@ -13474,22 +13508,22 @@
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>cp.cc.s</t>
+          <t>cp.cc.p</t>
         </is>
       </c>
       <c r="D171" s="9" t="inlineStr">
         <is>
-          <t>Blueprint: every step by the rules, in order</t>
+          <t>Work without a system creates chaos</t>
         </is>
       </c>
       <c r="E171" s="9" t="inlineStr">
         <is>
-          <t>Blueprint: ყველა ნაბიჯი წესით და თანმიმდევრობით</t>
+          <t>არასისტემური მუშაობა ქაოსს ქმნის</t>
         </is>
       </c>
       <c r="F171" s="9" t="inlineStr">
         <is>
-          <t>Blueprint: каждый шаг по правилам и по порядку</t>
+          <t>Работа без системы создаёт хаос</t>
         </is>
       </c>
       <c r="G171" s="3" t="inlineStr">
@@ -13516,22 +13550,22 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>cp.cd.p</t>
+          <t>cp.cc.s</t>
         </is>
       </c>
       <c r="D172" s="9" t="inlineStr">
         <is>
-          <t>Scattered data, wrong decisions</t>
+          <t>Blueprint: every step by the rules, in order</t>
         </is>
       </c>
       <c r="E172" s="9" t="inlineStr">
         <is>
-          <t>გაფანტული მონაცემები — არასწორი გადაწყვეტილებები</t>
+          <t>Blueprint: ყველა ნაბიჯი წესით და თანმიმდევრობით</t>
         </is>
       </c>
       <c r="F172" s="9" t="inlineStr">
         <is>
-          <t>Разрозненные данные — неверные решения</t>
+          <t>Blueprint: каждый шаг по правилам и по порядку</t>
         </is>
       </c>
       <c r="G172" s="3" t="inlineStr">
@@ -13558,22 +13592,22 @@
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>cp.cd.s</t>
+          <t>cp.cd.p</t>
         </is>
       </c>
       <c r="D173" s="9" t="inlineStr">
         <is>
-          <t>Analytics: exact numbers on one dashboard</t>
+          <t>Scattered data, wrong decisions</t>
         </is>
       </c>
       <c r="E173" s="9" t="inlineStr">
         <is>
-          <t>ანალიტიკა: ზუსტი ციფრები ერთ დეშბორდზე</t>
+          <t>გაფანტული მონაცემები — არასწორი გადაწყვეტილებები</t>
         </is>
       </c>
       <c r="F173" s="9" t="inlineStr">
         <is>
-          <t>Аналитика: точные цифры на одном дашборде</t>
+          <t>Разрозненные данные — неверные решения</t>
         </is>
       </c>
       <c r="G173" s="3" t="inlineStr">
@@ -13595,27 +13629,27 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>Pk</t>
+          <t>Cp</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>pk.title</t>
+          <t>cp.cd.s</t>
         </is>
       </c>
       <c r="D174" s="9" t="inlineStr">
         <is>
-          <t>Choose where to start</t>
+          <t>Analytics: exact numbers on one dashboard</t>
         </is>
       </c>
       <c r="E174" s="9" t="inlineStr">
         <is>
-          <t>აირჩიე, საიდან დაიწყო</t>
+          <t>ანალიტიკა: ზუსტი ციფრები ერთ დეშბორდზე</t>
         </is>
       </c>
       <c r="F174" s="9" t="inlineStr">
         <is>
-          <t>Выберите, с чего начать</t>
+          <t>Аналитика: точные цифры на одном дашборде</t>
         </is>
       </c>
       <c r="G174" s="3" t="inlineStr">
@@ -13642,22 +13676,22 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>pk.sub</t>
+          <t>pk.title</t>
         </is>
       </c>
       <c r="D175" s="9" t="inlineStr">
         <is>
-          <t>Fixed price, fixed timeline. Start small and add the rest later.</t>
+          <t>Choose where to start</t>
         </is>
       </c>
       <c r="E175" s="9" t="inlineStr">
         <is>
-          <t>ფიქსირებული ფასი და მკაფიო ვადები. დაიწყე მცირე პაკეტით, დანარჩენს მოგვიანებით დაამატებ.</t>
+          <t>აირჩიე, საიდან დაიწყო</t>
         </is>
       </c>
       <c r="F175" s="9" t="inlineStr">
         <is>
-          <t>Фиксированная цена и срок. Начните с малого, остальное добавите потом.</t>
+          <t>Выберите, с чего начать</t>
         </is>
       </c>
       <c r="G175" s="3" t="inlineStr">
@@ -13684,22 +13718,22 @@
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>pk.popular</t>
+          <t>pk.sub</t>
         </is>
       </c>
       <c r="D176" s="9" t="inlineStr">
         <is>
-          <t>Most popular</t>
+          <t>Fixed price, fixed timeline. Start small and add the rest later.</t>
         </is>
       </c>
       <c r="E176" s="9" t="inlineStr">
         <is>
-          <t>ყველაზე ხშირად ირჩევენ</t>
+          <t>ფიქსირებული ფასი და მკაფიო ვადები. დაიწყე მცირე პაკეტით, დანარჩენს მოგვიანებით დაამატებ.</t>
         </is>
       </c>
       <c r="F176" s="9" t="inlineStr">
         <is>
-          <t>Выбирают чаще всего</t>
+          <t>Фиксированная цена и срок. Начните с малого, остальное добавите потом.</t>
         </is>
       </c>
       <c r="G176" s="3" t="inlineStr">
@@ -13726,22 +13760,22 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>pk.deal</t>
+          <t>pk.popular</t>
         </is>
       </c>
       <c r="D177" s="9" t="inlineStr">
         <is>
-          <t>Discount valid for 1 week from the day the offer is sent.</t>
+          <t>Most popular</t>
         </is>
       </c>
       <c r="E177" s="9" t="inlineStr">
         <is>
-          <t>ფასდაკლება მოქმედებს ოფერის გაგზავნიდან 1 კვირის განმავლობაში.</t>
+          <t>ყველაზე ხშირად ირჩევენ</t>
         </is>
       </c>
       <c r="F177" s="9" t="inlineStr">
         <is>
-          <t>Скидка действует 1 неделю с момента отправки предложения.</t>
+          <t>Выбирают чаще всего</t>
         </is>
       </c>
       <c r="G177" s="3" t="inlineStr">
@@ -13768,22 +13802,22 @@
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>pk.once</t>
+          <t>pk.deal</t>
         </is>
       </c>
       <c r="D178" s="9" t="inlineStr">
         <is>
-          <t>one-time</t>
+          <t>Discount valid for 1 week from the day the offer is sent.</t>
         </is>
       </c>
       <c r="E178" s="9" t="inlineStr">
         <is>
-          <t>ერთჯერადად</t>
+          <t>ფასდაკლება მოქმედებს ოფერის გაგზავნიდან 1 კვირის განმავლობაში.</t>
         </is>
       </c>
       <c r="F178" s="9" t="inlineStr">
         <is>
-          <t>разово</t>
+          <t>Скидка действует 1 неделю с момента отправки предложения.</t>
         </is>
       </c>
       <c r="G178" s="3" t="inlineStr">
@@ -13810,22 +13844,22 @@
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>pk.days</t>
+          <t>pk.once</t>
         </is>
       </c>
       <c r="D179" s="9" t="inlineStr">
         <is>
-          <t>working days</t>
+          <t>one-time</t>
         </is>
       </c>
       <c r="E179" s="9" t="inlineStr">
         <is>
-          <t>სამუშაო დღე</t>
+          <t>ერთჯერადად</t>
         </is>
       </c>
       <c r="F179" s="9" t="inlineStr">
         <is>
-          <t>рабочих дней</t>
+          <t>разово</t>
         </is>
       </c>
       <c r="G179" s="3" t="inlineStr">
@@ -13852,22 +13886,22 @@
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>pk.full</t>
+          <t>pk.days</t>
         </is>
       </c>
       <c r="D180" s="9" t="inlineStr">
         <is>
-          <t>Everything included</t>
+          <t>working days</t>
         </is>
       </c>
       <c r="E180" s="9" t="inlineStr">
         <is>
-          <t>სრული ჩამონათვალი</t>
+          <t>სამუშაო დღე</t>
         </is>
       </c>
       <c r="F180" s="9" t="inlineStr">
         <is>
-          <t>Всё, что входит</t>
+          <t>рабочих дней</t>
         </is>
       </c>
       <c r="G180" s="3" t="inlineStr">
@@ -13894,22 +13928,22 @@
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>pk.choose</t>
+          <t>pk.full</t>
         </is>
       </c>
       <c r="D181" s="9" t="inlineStr">
         <is>
-          <t>Choose this package</t>
+          <t>Everything included</t>
         </is>
       </c>
       <c r="E181" s="9" t="inlineStr">
         <is>
-          <t>ამ პაკეტის არჩევა</t>
+          <t>სრული ჩამონათვალი</t>
         </is>
       </c>
       <c r="F181" s="9" t="inlineStr">
         <is>
-          <t>Выбрать этот пакет</t>
+          <t>Всё, что входит</t>
         </is>
       </c>
       <c r="G181" s="3" t="inlineStr">
@@ -13936,22 +13970,22 @@
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>pk.chosen</t>
+          <t>pk.choose</t>
         </is>
       </c>
       <c r="D182" s="9" t="inlineStr">
         <is>
-          <t>Selected</t>
+          <t>Choose this package</t>
         </is>
       </c>
       <c r="E182" s="9" t="inlineStr">
         <is>
-          <t>არჩეულია</t>
+          <t>ამ პაკეტის არჩევა</t>
         </is>
       </c>
       <c r="F182" s="9" t="inlineStr">
         <is>
-          <t>Выбран</t>
+          <t>Выбрать этот пакет</t>
         </is>
       </c>
       <c r="G182" s="3" t="inlineStr">
@@ -13978,22 +14012,22 @@
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>pk.note</t>
+          <t>pk.chosen</t>
         </is>
       </c>
       <c r="D183" s="9" t="inlineStr">
         <is>
-          <t>VAT (18%) is added. The CRM licence is paid separately, directly to the vendor.</t>
+          <t>Selected</t>
         </is>
       </c>
       <c r="E183" s="9" t="inlineStr">
         <is>
-          <t>ფასს ემატება დღგ (18%). CRM-ის ლიცენზიას ცალკე, პირდაპირ მწარმოებელს უხდი.</t>
+          <t>არჩეულია</t>
         </is>
       </c>
       <c r="F183" s="9" t="inlineStr">
         <is>
-          <t>Добавляется НДС (18%). Лицензия CRM оплачивается отдельно, напрямую производителю.</t>
+          <t>Выбран</t>
         </is>
       </c>
       <c r="G183" s="3" t="inlineStr">
@@ -14020,22 +14054,22 @@
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>pk.cur</t>
+          <t>pk.note</t>
         </is>
       </c>
       <c r="D184" s="9" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>VAT (18%) is added. The CRM licence is paid separately, directly to the vendor.</t>
         </is>
       </c>
       <c r="E184" s="9" t="inlineStr">
         <is>
-          <t>ვალუტა</t>
+          <t>ფასს ემატება დღგ (18%). CRM-ის ლიცენზიას ცალკე, პირდაპირ მწარმოებელს უხდი.</t>
         </is>
       </c>
       <c r="F184" s="9" t="inlineStr">
         <is>
-          <t>Валюта</t>
+          <t>Добавляется НДС (18%). Лицензия CRM оплачивается отдельно, напрямую производителю.</t>
         </is>
       </c>
       <c r="G184" s="3" t="inlineStr">
@@ -14057,27 +14091,27 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Ao</t>
+          <t>Pk</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>ao.title</t>
+          <t>pk.cur</t>
         </is>
       </c>
       <c r="D185" s="9" t="inlineStr">
         <is>
-          <t>Extra features</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="E185" s="9" t="inlineStr">
         <is>
-          <t>დამატებითი ფუნქციები</t>
+          <t>ვალუტა</t>
         </is>
       </c>
       <c r="F185" s="9" t="inlineStr">
         <is>
-          <t>Дополнительные функции</t>
+          <t>Валюта</t>
         </is>
       </c>
       <c r="G185" s="3" t="inlineStr">
@@ -14104,22 +14138,22 @@
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>ao.sub</t>
+          <t>ao.title</t>
         </is>
       </c>
       <c r="D186" s="9" t="inlineStr">
         <is>
-          <t>Optional. Add only if you need them</t>
+          <t>Extra features</t>
         </is>
       </c>
       <c r="E186" s="9" t="inlineStr">
         <is>
-          <t>არასავალდებულოა. დაამატე მხოლოდ საჭიროებისამებრ</t>
+          <t>დამატებითი ფუნქციები</t>
         </is>
       </c>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>Необязательно. Добавьте, если нужно</t>
+          <t>Дополнительные функции</t>
         </is>
       </c>
       <c r="G186" s="3" t="inlineStr">
@@ -14146,22 +14180,22 @@
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>ao.popular</t>
+          <t>ao.sub</t>
         </is>
       </c>
       <c r="D187" s="9" t="inlineStr">
         <is>
-          <t>Often added</t>
+          <t>Optional. Add only if you need them</t>
         </is>
       </c>
       <c r="E187" s="9" t="inlineStr">
         <is>
-          <t>ხშირად ამატებენ</t>
+          <t>არასავალდებულოა. დაამატე მხოლოდ საჭიროებისამებრ</t>
         </is>
       </c>
       <c r="F187" s="9" t="inlineStr">
         <is>
-          <t>Часто добавляют</t>
+          <t>Необязательно. Добавьте, если нужно</t>
         </is>
       </c>
       <c r="G187" s="3" t="inlineStr">
@@ -14188,22 +14222,22 @@
       </c>
       <c r="C188" s="3" t="inlineStr">
         <is>
-          <t>ao.more</t>
+          <t>ao.popular</t>
         </is>
       </c>
       <c r="D188" s="9" t="inlineStr">
         <is>
-          <t>All add-ons by category</t>
+          <t>Often added</t>
         </is>
       </c>
       <c r="E188" s="9" t="inlineStr">
         <is>
-          <t>ყველა დამატებითი ფუნქცია კატეგორიების მიხედვით</t>
+          <t>ხშირად ამატებენ</t>
         </is>
       </c>
       <c r="F188" s="9" t="inlineStr">
         <is>
-          <t>Все дополнения по категориям</t>
+          <t>Часто добавляют</t>
         </is>
       </c>
       <c r="G188" s="3" t="inlineStr">
@@ -14230,22 +14264,22 @@
       </c>
       <c r="C189" s="3" t="inlineStr">
         <is>
-          <t>ao.catalog</t>
+          <t>ao.more</t>
         </is>
       </c>
       <c r="D189" s="9" t="inlineStr">
         <is>
-          <t>We show the full catalog (75+ solutions) on the call.</t>
+          <t>All add-ons by category</t>
         </is>
       </c>
       <c r="E189" s="9" t="inlineStr">
         <is>
-          <t>სრულ კატალოგს (75+ გადაწყვეტა) ზარზე გაჩვენებთ.</t>
+          <t>ყველა დამატებითი ფუნქცია კატეგორიების მიხედვით</t>
         </is>
       </c>
       <c r="F189" s="9" t="inlineStr">
         <is>
-          <t>Полный каталог (75+ решений) покажем на звонке.</t>
+          <t>Все дополнения по категориям</t>
         </is>
       </c>
       <c r="G189" s="3" t="inlineStr">
@@ -14267,27 +14301,27 @@
       </c>
       <c r="B190" s="3" t="inlineStr">
         <is>
-          <t>Sum</t>
+          <t>Ao</t>
         </is>
       </c>
       <c r="C190" s="3" t="inlineStr">
         <is>
-          <t>sum.empty</t>
+          <t>ao.catalog</t>
         </is>
       </c>
       <c r="D190" s="9" t="inlineStr">
         <is>
-          <t>Choose a package</t>
+          <t>We show the full catalog (75+ solutions) on the call.</t>
         </is>
       </c>
       <c r="E190" s="9" t="inlineStr">
         <is>
-          <t>აირჩიე პაკეტი</t>
+          <t>სრულ კატალოგს (75+ გადაწყვეტა) ზარზე გაჩვენებთ.</t>
         </is>
       </c>
       <c r="F190" s="9" t="inlineStr">
         <is>
-          <t>Выберите пакет</t>
+          <t>Полный каталог (75+ решений) покажем на звонке.</t>
         </is>
       </c>
       <c r="G190" s="3" t="inlineStr">
@@ -14314,22 +14348,22 @@
       </c>
       <c r="C191" s="3" t="inlineStr">
         <is>
-          <t>sum.addons</t>
+          <t>sum.empty</t>
         </is>
       </c>
       <c r="D191" s="9" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>Choose a package</t>
         </is>
       </c>
       <c r="E191" s="9" t="inlineStr">
         <is>
-          <t>ფუნქცია</t>
+          <t>აირჩიე პაკეტი</t>
         </is>
       </c>
       <c r="F191" s="9" t="inlineStr">
         <is>
-          <t>функц.</t>
+          <t>Выберите пакет</t>
         </is>
       </c>
       <c r="G191" s="3" t="inlineStr">
@@ -14356,22 +14390,22 @@
       </c>
       <c r="C192" s="3" t="inlineStr">
         <is>
-          <t>sum.vat</t>
+          <t>sum.addons</t>
         </is>
       </c>
       <c r="D192" s="9" t="inlineStr">
         <is>
-          <t>+ VAT</t>
+          <t>features</t>
         </is>
       </c>
       <c r="E192" s="9" t="inlineStr">
         <is>
-          <t>+ დღგ</t>
+          <t>ფუნქცია</t>
         </is>
       </c>
       <c r="F192" s="9" t="inlineStr">
         <is>
-          <t>+ НДС</t>
+          <t>функц.</t>
         </is>
       </c>
       <c r="G192" s="3" t="inlineStr">
@@ -14398,22 +14432,22 @@
       </c>
       <c r="C193" s="3" t="inlineStr">
         <is>
-          <t>sum.cta</t>
+          <t>sum.vat</t>
         </is>
       </c>
       <c r="D193" s="9" t="inlineStr">
         <is>
-          <t>Request a call</t>
+          <t>+ VAT</t>
         </is>
       </c>
       <c r="E193" s="9" t="inlineStr">
         <is>
-          <t>მოითხოვე ზარი</t>
+          <t>+ დღგ</t>
         </is>
       </c>
       <c r="F193" s="9" t="inlineStr">
         <is>
-          <t>Запросить звонок</t>
+          <t>+ НДС</t>
         </is>
       </c>
       <c r="G193" s="3" t="inlineStr">
@@ -14440,22 +14474,22 @@
       </c>
       <c r="C194" s="3" t="inlineStr">
         <is>
-          <t>sum.picked</t>
+          <t>sum.cta</t>
         </is>
       </c>
       <c r="D194" s="9" t="inlineStr">
         <is>
-          <t>Your selection:</t>
+          <t>Request a call</t>
         </is>
       </c>
       <c r="E194" s="9" t="inlineStr">
         <is>
-          <t>შენი არჩევანი:</t>
+          <t>მოითხოვე ზარი</t>
         </is>
       </c>
       <c r="F194" s="9" t="inlineStr">
         <is>
-          <t>Ваш выбор:</t>
+          <t>Запросить звонок</t>
         </is>
       </c>
       <c r="G194" s="3" t="inlineStr">
@@ -14477,27 +14511,27 @@
       </c>
       <c r="B195" s="3" t="inlineStr">
         <is>
-          <t>Pk</t>
+          <t>Sum</t>
         </is>
       </c>
       <c r="C195" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.name</t>
+          <t>sum.picked</t>
         </is>
       </c>
       <c r="D195" s="9" t="inlineStr">
         <is>
-          <t>Starter</t>
+          <t>Your selection:</t>
         </is>
       </c>
       <c r="E195" s="9" t="inlineStr">
         <is>
-          <t>სტარტი</t>
+          <t>შენი არჩევანი:</t>
         </is>
       </c>
       <c r="F195" s="9" t="inlineStr">
         <is>
-          <t>Старт</t>
+          <t>Ваш выбор:</t>
         </is>
       </c>
       <c r="G195" s="3" t="inlineStr">
@@ -14524,22 +14558,22 @@
       </c>
       <c r="C196" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.short</t>
+          <t>pk.starter.name</t>
         </is>
       </c>
       <c r="D196" s="9" t="inlineStr">
         <is>
-          <t>To move from Excel into a CRM</t>
+          <t>Starter</t>
         </is>
       </c>
       <c r="E196" s="9" t="inlineStr">
         <is>
-          <t>Excel-იდან CRM-ზე გადასასვლელად</t>
+          <t>სტარტი</t>
         </is>
       </c>
       <c r="F196" s="9" t="inlineStr">
         <is>
-          <t>Чтобы перейти с Excel на CRM</t>
+          <t>Старт</t>
         </is>
       </c>
       <c r="G196" s="3" t="inlineStr">
@@ -14566,22 +14600,22 @@
       </c>
       <c r="C197" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.out</t>
+          <t>pk.starter.short</t>
         </is>
       </c>
       <c r="D197" s="9" t="inlineStr">
         <is>
-          <t>You move from Excel to a CRM: every client and lead in one system.</t>
+          <t>To move from Excel into a CRM</t>
         </is>
       </c>
       <c r="E197" s="9" t="inlineStr">
         <is>
-          <t>Excel-იდან CRM-ზე გადახვალ: ყველა კლიენტი და ლიდი ერთ სისტემაშია.</t>
+          <t>Excel-იდან CRM-ზე გადასასვლელად</t>
         </is>
       </c>
       <c r="F197" s="9" t="inlineStr">
         <is>
-          <t>Переходите с Excel на CRM: все клиенты и лиды в одной системе.</t>
+          <t>Чтобы перейти с Excel на CRM</t>
         </is>
       </c>
       <c r="G197" s="3" t="inlineStr">
@@ -14608,22 +14642,22 @@
       </c>
       <c r="C198" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.h1</t>
+          <t>pk.starter.out</t>
         </is>
       </c>
       <c r="D198" s="9" t="inlineStr">
         <is>
-          <t>4 core modules</t>
+          <t>You move from Excel to a CRM: every client and lead in one system.</t>
         </is>
       </c>
       <c r="E198" s="9" t="inlineStr">
         <is>
-          <t>4 ძირითადი მოდული</t>
+          <t>Excel-იდან CRM-ზე გადახვალ: ყველა კლიენტი და ლიდი ერთ სისტემაშია.</t>
         </is>
       </c>
       <c r="F198" s="9" t="inlineStr">
         <is>
-          <t>4 базовых модуля</t>
+          <t>Переходите с Excel на CRM: все клиенты и лиды в одной системе.</t>
         </is>
       </c>
       <c r="G198" s="3" t="inlineStr">
@@ -14650,22 +14684,22 @@
       </c>
       <c r="C199" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.h2</t>
+          <t>pk.starter.h1</t>
         </is>
       </c>
       <c r="D199" s="9" t="inlineStr">
         <is>
-          <t>Email and Facebook inside the CRM</t>
+          <t>4 core modules</t>
         </is>
       </c>
       <c r="E199" s="9" t="inlineStr">
         <is>
-          <t>ელფოსტა და Facebook CRM-ში</t>
+          <t>4 ძირითადი მოდული</t>
         </is>
       </c>
       <c r="F199" s="9" t="inlineStr">
         <is>
-          <t>Почта и Facebook внутри CRM</t>
+          <t>4 базовых модуля</t>
         </is>
       </c>
       <c r="G199" s="3" t="inlineStr">
@@ -14692,22 +14726,22 @@
       </c>
       <c r="C200" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.h3</t>
+          <t>pk.starter.h2</t>
         </is>
       </c>
       <c r="D200" s="9" t="inlineStr">
         <is>
-          <t>Lead form and KPI dashboard</t>
+          <t>Email and Facebook inside the CRM</t>
         </is>
       </c>
       <c r="E200" s="9" t="inlineStr">
         <is>
-          <t>ლიდების ფორმა და KPI დაფა</t>
+          <t>ელფოსტა და Facebook CRM-ში</t>
         </is>
       </c>
       <c r="F200" s="9" t="inlineStr">
         <is>
-          <t>Форма лидов и дашборд KPI</t>
+          <t>Почта и Facebook внутри CRM</t>
         </is>
       </c>
       <c r="G200" s="3" t="inlineStr">
@@ -14734,22 +14768,22 @@
       </c>
       <c r="C201" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.i1</t>
+          <t>pk.starter.h3</t>
         </is>
       </c>
       <c r="D201" s="9" t="inlineStr">
         <is>
-          <t>4 core modules: Leads, Contacts, Accounts, Deals</t>
+          <t>Lead form and KPI dashboard</t>
         </is>
       </c>
       <c r="E201" s="9" t="inlineStr">
         <is>
-          <t>4 ძირითადი მოდული: ლიდები, კონტაქტები, კომპანიები, გარიგებები</t>
+          <t>ლიდების ფორმა და KPI დაფა</t>
         </is>
       </c>
       <c r="F201" s="9" t="inlineStr">
         <is>
-          <t>4 базовых модуля: лиды, контакты, компании, сделки</t>
+          <t>Форма лидов и дашборд KPI</t>
         </is>
       </c>
       <c r="G201" s="3" t="inlineStr">
@@ -14776,22 +14810,22 @@
       </c>
       <c r="C202" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.i2</t>
+          <t>pk.starter.i1</t>
         </is>
       </c>
       <c r="D202" s="9" t="inlineStr">
         <is>
-          <t>2-way email sync (Google or Microsoft 365)</t>
+          <t>4 core modules: Leads, Contacts, Accounts, Deals</t>
         </is>
       </c>
       <c r="E202" s="9" t="inlineStr">
         <is>
-          <t>ელფოსტის ორმხრივი სინქრონიზაცია (Google ან Microsoft 365)</t>
+          <t>4 ძირითადი მოდული: ლიდები, კონტაქტები, კომპანიები, გარიგებები</t>
         </is>
       </c>
       <c r="F202" s="9" t="inlineStr">
         <is>
-          <t>Двусторонняя синхронизация почты (Google или Microsoft 365)</t>
+          <t>4 базовых модуля: лиды, контакты, компании, сделки</t>
         </is>
       </c>
       <c r="G202" s="3" t="inlineStr">
@@ -14818,22 +14852,22 @@
       </c>
       <c r="C203" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.i3</t>
+          <t>pk.starter.i2</t>
         </is>
       </c>
       <c r="D203" s="9" t="inlineStr">
         <is>
-          <t>Facebook messages right inside the CRM</t>
+          <t>2-way email sync (Google or Microsoft 365)</t>
         </is>
       </c>
       <c r="E203" s="9" t="inlineStr">
         <is>
-          <t>Facebook-ის შეტყობინებები პირდაპირ CRM-ში</t>
+          <t>ელფოსტის ორმხრივი სინქრონიზაცია (Google ან Microsoft 365)</t>
         </is>
       </c>
       <c r="F203" s="9" t="inlineStr">
         <is>
-          <t>Сообщения Facebook прямо в CRM</t>
+          <t>Двусторонняя синхронизация почты (Google или Microsoft 365)</t>
         </is>
       </c>
       <c r="G203" s="3" t="inlineStr">
@@ -14860,22 +14894,22 @@
       </c>
       <c r="C204" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.i4</t>
+          <t>pk.starter.i3</t>
         </is>
       </c>
       <c r="D204" s="9" t="inlineStr">
         <is>
-          <t>1 web form to capture leads</t>
+          <t>Facebook messages right inside the CRM</t>
         </is>
       </c>
       <c r="E204" s="9" t="inlineStr">
         <is>
-          <t>1 ვებფორმა ლიდების მისაღებად</t>
+          <t>Facebook-ის შეტყობინებები პირდაპირ CRM-ში</t>
         </is>
       </c>
       <c r="F204" s="9" t="inlineStr">
         <is>
-          <t>1 веб-форма для приёма лидов</t>
+          <t>Сообщения Facebook прямо в CRM</t>
         </is>
       </c>
       <c r="G204" s="3" t="inlineStr">
@@ -14902,22 +14936,22 @@
       </c>
       <c r="C205" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.i5</t>
+          <t>pk.starter.i4</t>
         </is>
       </c>
       <c r="D205" s="9" t="inlineStr">
         <is>
-          <t>1 sales-pipeline KPI dashboard</t>
+          <t>1 web form to capture leads</t>
         </is>
       </c>
       <c r="E205" s="9" t="inlineStr">
         <is>
-          <t>გაყიდვების ძაბრის KPI დაფა</t>
+          <t>1 ვებფორმა ლიდების მისაღებად</t>
         </is>
       </c>
       <c r="F205" s="9" t="inlineStr">
         <is>
-          <t>Дашборд KPI воронки продаж</t>
+          <t>1 веб-форма для приёма лидов</t>
         </is>
       </c>
       <c r="G205" s="3" t="inlineStr">
@@ -14944,22 +14978,22 @@
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>pk.starter.i6</t>
+          <t>pk.starter.i5</t>
         </is>
       </c>
       <c r="D206" s="9" t="inlineStr">
         <is>
-          <t>Recorded video instructions for the team</t>
+          <t>1 sales-pipeline KPI dashboard</t>
         </is>
       </c>
       <c r="E206" s="9" t="inlineStr">
         <is>
-          <t>ჩაწერილი ვიდეო ინსტრუქციები გუნდისთვის</t>
+          <t>გაყიდვების ძაბრის KPI დაფა</t>
         </is>
       </c>
       <c r="F206" s="9" t="inlineStr">
         <is>
-          <t>Видеоинструкции для команды</t>
+          <t>Дашборд KPI воронки продаж</t>
         </is>
       </c>
       <c r="G206" s="3" t="inlineStr">
@@ -14986,22 +15020,22 @@
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.name</t>
+          <t>pk.starter.i6</t>
         </is>
       </c>
       <c r="D207" s="9" t="inlineStr">
         <is>
-          <t>Essentials</t>
+          <t>Recorded video instructions for the team</t>
         </is>
       </c>
       <c r="E207" s="9" t="inlineStr">
         <is>
-          <t>ოპტიმალური</t>
+          <t>ჩაწერილი ვიდეო ინსტრუქციები გუნდისთვის</t>
         </is>
       </c>
       <c r="F207" s="9" t="inlineStr">
         <is>
-          <t>Оптимальный</t>
+          <t>Видеоинструкции для команды</t>
         </is>
       </c>
       <c r="G207" s="3" t="inlineStr">
@@ -15028,22 +15062,22 @@
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.short</t>
+          <t>pk.essentials.name</t>
         </is>
       </c>
       <c r="D208" s="9" t="inlineStr">
         <is>
-          <t>For a 5-10 person sales team</t>
+          <t>Essentials</t>
         </is>
       </c>
       <c r="E208" s="9" t="inlineStr">
         <is>
-          <t>5-10-წევრიანი გაყიდვების გუნდისთვის</t>
+          <t>ოპტიმალური</t>
         </is>
       </c>
       <c r="F208" s="9" t="inlineStr">
         <is>
-          <t>Для отдела продаж из 5-10 человек</t>
+          <t>Оптимальный</t>
         </is>
       </c>
       <c r="G208" s="3" t="inlineStr">
@@ -15070,22 +15104,22 @@
       </c>
       <c r="C209" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.base</t>
+          <t>pk.essentials.short</t>
         </is>
       </c>
       <c r="D209" s="9" t="inlineStr">
         <is>
-          <t>Everything in Starter, plus:</t>
+          <t>For a 5-10 person sales team</t>
         </is>
       </c>
       <c r="E209" s="9" t="inlineStr">
         <is>
-          <t>სტარტ პაკეტის სრული ფუნქციონალი, პლუს:</t>
+          <t>5-10-წევრიანი გაყიდვების გუნდისთვის</t>
         </is>
       </c>
       <c r="F209" s="9" t="inlineStr">
         <is>
-          <t>Всё из «Старта», плюс:</t>
+          <t>Для отдела продаж из 5-10 человек</t>
         </is>
       </c>
       <c r="G209" s="3" t="inlineStr">
@@ -15112,22 +15146,22 @@
       </c>
       <c r="C210" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.out</t>
+          <t>pk.essentials.base</t>
         </is>
       </c>
       <c r="D210" s="9" t="inlineStr">
         <is>
-          <t>Sales in order: leads come in automatically and go to the right people.</t>
+          <t>Everything in Starter, plus:</t>
         </is>
       </c>
       <c r="E210" s="9" t="inlineStr">
         <is>
-          <t>მოწესრიგებული გაყიდვები: ლიდები ავტომატურად შემოდის და გუნდზე სწორად ნაწილდება.</t>
+          <t>სტარტ პაკეტის სრული ფუნქციონალი, პლუს:</t>
         </is>
       </c>
       <c r="F210" s="9" t="inlineStr">
         <is>
-          <t>Продажи в порядке: лиды приходят автоматически и правильно распределяются по команде.</t>
+          <t>Всё из «Старта», плюс:</t>
         </is>
       </c>
       <c r="G210" s="3" t="inlineStr">
@@ -15154,22 +15188,22 @@
       </c>
       <c r="C211" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.h1</t>
+          <t>pk.essentials.out</t>
         </is>
       </c>
       <c r="D211" s="9" t="inlineStr">
         <is>
-          <t>Everything in Starter</t>
+          <t>Sales in order: leads come in automatically and go to the right people.</t>
         </is>
       </c>
       <c r="E211" s="9" t="inlineStr">
         <is>
-          <t>სტარტ პაკეტის სრული ფუნქციონალი</t>
+          <t>მოწესრიგებული გაყიდვები: ლიდები ავტომატურად შემოდის და გუნდზე სწორად ნაწილდება.</t>
         </is>
       </c>
       <c r="F211" s="9" t="inlineStr">
         <is>
-          <t>Всё из «Старта»</t>
+          <t>Продажи в порядке: лиды приходят автоматически и правильно распределяются по команде.</t>
         </is>
       </c>
       <c r="G211" s="3" t="inlineStr">
@@ -15196,22 +15230,22 @@
       </c>
       <c r="C212" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.h2</t>
+          <t>pk.essentials.h1</t>
         </is>
       </c>
       <c r="D212" s="9" t="inlineStr">
         <is>
-          <t>Meta and Google Ads leads, automatically</t>
+          <t>Everything in Starter</t>
         </is>
       </c>
       <c r="E212" s="9" t="inlineStr">
         <is>
-          <t>Meta და Google Ads-ის ლიდები ავტომატურად</t>
+          <t>სტარტ პაკეტის სრული ფუნქციონალი</t>
         </is>
       </c>
       <c r="F212" s="9" t="inlineStr">
         <is>
-          <t>Лиды из Meta и Google Ads автоматически</t>
+          <t>Всё из «Старта»</t>
         </is>
       </c>
       <c r="G212" s="3" t="inlineStr">
@@ -15238,22 +15272,22 @@
       </c>
       <c r="C213" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.h3</t>
+          <t>pk.essentials.h2</t>
         </is>
       </c>
       <c r="D213" s="9" t="inlineStr">
         <is>
-          <t>Stage rules and lead assignment</t>
+          <t>Meta and Google Ads leads, automatically</t>
         </is>
       </c>
       <c r="E213" s="9" t="inlineStr">
         <is>
-          <t>გაყიდვის ეტაპები მკაფიო წესებით და ლიდების განაწილება</t>
+          <t>Meta და Google Ads-ის ლიდები ავტომატურად</t>
         </is>
       </c>
       <c r="F213" s="9" t="inlineStr">
         <is>
-          <t>Правила этапов и распределение лидов</t>
+          <t>Лиды из Meta и Google Ads автоматически</t>
         </is>
       </c>
       <c r="G213" s="3" t="inlineStr">
@@ -15280,22 +15314,22 @@
       </c>
       <c r="C214" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i1</t>
+          <t>pk.essentials.h3</t>
         </is>
       </c>
       <c r="D214" s="9" t="inlineStr">
         <is>
-          <t>Up to 15 custom fields</t>
+          <t>Stage rules and lead assignment</t>
         </is>
       </c>
       <c r="E214" s="9" t="inlineStr">
         <is>
-          <t>15-მდე დამატებითი ველი</t>
+          <t>გაყიდვის ეტაპები მკაფიო წესებით და ლიდების განაწილება</t>
         </is>
       </c>
       <c r="F214" s="9" t="inlineStr">
         <is>
-          <t>До 15 дополнительных полей</t>
+          <t>Правила этапов и распределение лидов</t>
         </is>
       </c>
       <c r="G214" s="3" t="inlineStr">
@@ -15322,22 +15356,22 @@
       </c>
       <c r="C215" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i2</t>
+          <t>pk.essentials.i1</t>
         </is>
       </c>
       <c r="D215" s="9" t="inlineStr">
         <is>
-          <t>Products and invoices, with your invoice template</t>
+          <t>Up to 15 custom fields</t>
         </is>
       </c>
       <c r="E215" s="9" t="inlineStr">
         <is>
-          <t>პროდუქტები და ინვოისები, შენი ინვოისის შაბლონით</t>
+          <t>15-მდე დამატებითი ველი</t>
         </is>
       </c>
       <c r="F215" s="9" t="inlineStr">
         <is>
-          <t>Товары и счета с вашим шаблоном счёта</t>
+          <t>До 15 дополнительных полей</t>
         </is>
       </c>
       <c r="G215" s="3" t="inlineStr">
@@ -15364,22 +15398,22 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i3</t>
+          <t>pk.essentials.i2</t>
         </is>
       </c>
       <c r="D216" s="9" t="inlineStr">
         <is>
-          <t>Sales stages with rules: no skipped steps</t>
+          <t>Products and invoices, with your invoice template</t>
         </is>
       </c>
       <c r="E216" s="9" t="inlineStr">
         <is>
-          <t>გაყიდვის ეტაპები მკაფიო წესებით: ეტაპს ვერ გამოტოვებ</t>
+          <t>პროდუქტები და ინვოისები, შენი ინვოისის შაბლონით</t>
         </is>
       </c>
       <c r="F216" s="9" t="inlineStr">
         <is>
-          <t>Этапы продаж с правилами: этап не пропустить</t>
+          <t>Товары и счета с вашим шаблоном счёта</t>
         </is>
       </c>
       <c r="G216" s="3" t="inlineStr">
@@ -15406,22 +15440,22 @@
       </c>
       <c r="C217" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i4</t>
+          <t>pk.essentials.i3</t>
         </is>
       </c>
       <c r="D217" s="9" t="inlineStr">
         <is>
-          <t>Phone validation (+995) and deduplication</t>
+          <t>Sales stages with rules: no skipped steps</t>
         </is>
       </c>
       <c r="E217" s="9" t="inlineStr">
         <is>
-          <t>ტელეფონის ნომრების ვალიდაცია (+995) და დუბლიკატების გასუფთავება</t>
+          <t>გაყიდვის ეტაპები მკაფიო წესებით: ეტაპს ვერ გამოტოვებ</t>
         </is>
       </c>
       <c r="F217" s="9" t="inlineStr">
         <is>
-          <t>Проверка номеров (+995) и удаление дублей</t>
+          <t>Этапы продаж с правилами: этап не пропустить</t>
         </is>
       </c>
       <c r="G217" s="3" t="inlineStr">
@@ -15448,22 +15482,22 @@
       </c>
       <c r="C218" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i5</t>
+          <t>pk.essentials.i4</t>
         </is>
       </c>
       <c r="D218" s="9" t="inlineStr">
         <is>
-          <t>Meta and Google Ads leads synced automatically</t>
+          <t>Phone validation (+995) and deduplication</t>
         </is>
       </c>
       <c r="E218" s="9" t="inlineStr">
         <is>
-          <t>Meta-სა და Google Ads-ის ლიდები ავტომატურად CRM-ში</t>
+          <t>ტელეფონის ნომრების ვალიდაცია (+995) და დუბლიკატების გასუფთავება</t>
         </is>
       </c>
       <c r="F218" s="9" t="inlineStr">
         <is>
-          <t>Лиды из Meta и Google Ads автоматически в CRM</t>
+          <t>Проверка номеров (+995) и удаление дублей</t>
         </is>
       </c>
       <c r="G218" s="3" t="inlineStr">
@@ -15490,22 +15524,22 @@
       </c>
       <c r="C219" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i6</t>
+          <t>pk.essentials.i5</t>
         </is>
       </c>
       <c r="D219" s="9" t="inlineStr">
         <is>
-          <t>Automatic lead assignment across managers</t>
+          <t>Meta and Google Ads leads synced automatically</t>
         </is>
       </c>
       <c r="E219" s="9" t="inlineStr">
         <is>
-          <t>ლიდების ავტომატური განაწილება მენეჯერებზე</t>
+          <t>Meta-სა და Google Ads-ის ლიდები ავტომატურად CRM-ში</t>
         </is>
       </c>
       <c r="F219" s="9" t="inlineStr">
         <is>
-          <t>Автоматическое распределение лидов по менеджерам</t>
+          <t>Лиды из Meta и Google Ads автоматически в CRM</t>
         </is>
       </c>
       <c r="G219" s="3" t="inlineStr">
@@ -15532,22 +15566,22 @@
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i7</t>
+          <t>pk.essentials.i6</t>
         </is>
       </c>
       <c r="D220" s="9" t="inlineStr">
         <is>
-          <t>Follow-up reminders</t>
+          <t>Automatic lead assignment across managers</t>
         </is>
       </c>
       <c r="E220" s="9" t="inlineStr">
         <is>
-          <t>follow-up შეხსენებები</t>
+          <t>ლიდების ავტომატური განაწილება მენეჯერებზე</t>
         </is>
       </c>
       <c r="F220" s="9" t="inlineStr">
         <is>
-          <t>Напоминания о follow-up</t>
+          <t>Автоматическое распределение лидов по менеджерам</t>
         </is>
       </c>
       <c r="G220" s="3" t="inlineStr">
@@ -15574,22 +15608,22 @@
       </c>
       <c r="C221" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i8</t>
+          <t>pk.essentials.i7</t>
         </is>
       </c>
       <c r="D221" s="9" t="inlineStr">
         <is>
-          <t>Contacts and products migration</t>
+          <t>Follow-up reminders</t>
         </is>
       </c>
       <c r="E221" s="9" t="inlineStr">
         <is>
-          <t>კონტაქტებისა და პროდუქტების გადმოტანა</t>
+          <t>follow-up შეხსენებები</t>
         </is>
       </c>
       <c r="F221" s="9" t="inlineStr">
         <is>
-          <t>Перенос контактов и товаров</t>
+          <t>Напоминания о follow-up</t>
         </is>
       </c>
       <c r="G221" s="3" t="inlineStr">
@@ -15616,22 +15650,22 @@
       </c>
       <c r="C222" s="3" t="inlineStr">
         <is>
-          <t>pk.essentials.i9</t>
+          <t>pk.essentials.i8</t>
         </is>
       </c>
       <c r="D222" s="9" t="inlineStr">
         <is>
-          <t>30-minute training, recorded</t>
+          <t>Contacts and products migration</t>
         </is>
       </c>
       <c r="E222" s="9" t="inlineStr">
         <is>
-          <t>30-წუთიანი ტრენინგი (ჩანაწერით)</t>
+          <t>კონტაქტებისა და პროდუქტების გადმოტანა</t>
         </is>
       </c>
       <c r="F222" s="9" t="inlineStr">
         <is>
-          <t>30-минутное обучение с записью</t>
+          <t>Перенос контактов и товаров</t>
         </is>
       </c>
       <c r="G222" s="3" t="inlineStr">
@@ -15658,22 +15692,22 @@
       </c>
       <c r="C223" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.name</t>
+          <t>pk.essentials.i9</t>
         </is>
       </c>
       <c r="D223" s="9" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>30-minute training, recorded</t>
         </is>
       </c>
       <c r="E223" s="9" t="inlineStr">
         <is>
-          <t>ზრდა</t>
+          <t>30-წუთიანი ტრენინგი (ჩანაწერით)</t>
         </is>
       </c>
       <c r="F223" s="9" t="inlineStr">
         <is>
-          <t>Рост</t>
+          <t>30-минутное обучение с записью</t>
         </is>
       </c>
       <c r="G223" s="3" t="inlineStr">
@@ -15700,22 +15734,22 @@
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.short</t>
+          <t>pk.growth.name</t>
         </is>
       </c>
       <c r="D224" s="9" t="inlineStr">
         <is>
-          <t>For a growing 15-25 person team</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E224" s="9" t="inlineStr">
         <is>
-          <t>15-25-წევრიანი მზარდი გუნდისთვის</t>
+          <t>ზრდა</t>
         </is>
       </c>
       <c r="F224" s="9" t="inlineStr">
         <is>
-          <t>Для растущей команды из 15-25 человек</t>
+          <t>Рост</t>
         </is>
       </c>
       <c r="G224" s="3" t="inlineStr">
@@ -15742,22 +15776,22 @@
       </c>
       <c r="C225" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.base</t>
+          <t>pk.growth.short</t>
         </is>
       </c>
       <c r="D225" s="9" t="inlineStr">
         <is>
-          <t>Everything in Essentials, plus:</t>
+          <t>For a growing 15-25 person team</t>
         </is>
       </c>
       <c r="E225" s="9" t="inlineStr">
         <is>
-          <t>ოპტიმალურის სრული ფუნქციონალი, პლუს:</t>
+          <t>15-25-წევრიანი მზარდი გუნდისთვის</t>
         </is>
       </c>
       <c r="F225" s="9" t="inlineStr">
         <is>
-          <t>Всё из «Оптимального», плюс:</t>
+          <t>Для растущей команды из 15-25 человек</t>
         </is>
       </c>
       <c r="G225" s="3" t="inlineStr">
@@ -15784,22 +15818,22 @@
       </c>
       <c r="C226" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.out</t>
+          <t>pk.growth.base</t>
         </is>
       </c>
       <c r="D226" s="9" t="inlineStr">
         <is>
-          <t>A complete sales system: calls, automations and AI in one place.</t>
+          <t>Everything in Essentials, plus:</t>
         </is>
       </c>
       <c r="E226" s="9" t="inlineStr">
         <is>
-          <t>გაყიდვების სრული სისტემა: ზარები, ავტომატიზაციები და AI ერთ სივრცეში.</t>
+          <t>ოპტიმალურის სრული ფუნქციონალი, პლუს:</t>
         </is>
       </c>
       <c r="F226" s="9" t="inlineStr">
         <is>
-          <t>Полная система продаж: звонки, автоматизации и AI в одном месте.</t>
+          <t>Всё из «Оптимального», плюс:</t>
         </is>
       </c>
       <c r="G226" s="3" t="inlineStr">
@@ -15826,22 +15860,22 @@
       </c>
       <c r="C227" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.h1</t>
+          <t>pk.growth.out</t>
         </is>
       </c>
       <c r="D227" s="9" t="inlineStr">
         <is>
-          <t>Everything in Essentials</t>
+          <t>A complete sales system: calls, automations and AI in one place.</t>
         </is>
       </c>
       <c r="E227" s="9" t="inlineStr">
         <is>
-          <t>ოპტიმალურის სრული ფუნქციონალი</t>
+          <t>გაყიდვების სრული სისტემა: ზარები, ავტომატიზაციები და AI ერთ სივრცეში.</t>
         </is>
       </c>
       <c r="F227" s="9" t="inlineStr">
         <is>
-          <t>Всё из «Оптимального»</t>
+          <t>Полная система продаж: звонки, автоматизации и AI в одном месте.</t>
         </is>
       </c>
       <c r="G227" s="3" t="inlineStr">
@@ -15868,22 +15902,22 @@
       </c>
       <c r="C228" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.h2</t>
+          <t>pk.growth.h1</t>
         </is>
       </c>
       <c r="D228" s="9" t="inlineStr">
         <is>
-          <t>Telephony and call processing</t>
+          <t>Everything in Essentials</t>
         </is>
       </c>
       <c r="E228" s="9" t="inlineStr">
         <is>
-          <t>ტელეფონია და ზარების დამუშავება</t>
+          <t>ოპტიმალურის სრული ფუნქციონალი</t>
         </is>
       </c>
       <c r="F228" s="9" t="inlineStr">
         <is>
-          <t>Телефония и обработка звонков</t>
+          <t>Всё из «Оптимального»</t>
         </is>
       </c>
       <c r="G228" s="3" t="inlineStr">
@@ -15910,22 +15944,22 @@
       </c>
       <c r="C229" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.h3</t>
+          <t>pk.growth.h2</t>
         </is>
       </c>
       <c r="D229" s="9" t="inlineStr">
         <is>
-          <t>Automations and AI (Claude)</t>
+          <t>Telephony and call processing</t>
         </is>
       </c>
       <c r="E229" s="9" t="inlineStr">
         <is>
-          <t>ავტომატიზაციები და AI (Claude)</t>
+          <t>ტელეფონია და ზარების დამუშავება</t>
         </is>
       </c>
       <c r="F229" s="9" t="inlineStr">
         <is>
-          <t>Автоматизации и AI (Claude)</t>
+          <t>Телефония и обработка звонков</t>
         </is>
       </c>
       <c r="G229" s="3" t="inlineStr">
@@ -15952,22 +15986,22 @@
       </c>
       <c r="C230" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i1</t>
+          <t>pk.growth.h3</t>
         </is>
       </c>
       <c r="D230" s="9" t="inlineStr">
         <is>
-          <t>Up to 3 additional modules</t>
+          <t>Automations and AI (Claude)</t>
         </is>
       </c>
       <c r="E230" s="9" t="inlineStr">
         <is>
-          <t>3-მდე დამატებითი მოდული</t>
+          <t>ავტომატიზაციები და AI (Claude)</t>
         </is>
       </c>
       <c r="F230" s="9" t="inlineStr">
         <is>
-          <t>До 3 дополнительных модулей</t>
+          <t>Автоматизации и AI (Claude)</t>
         </is>
       </c>
       <c r="G230" s="3" t="inlineStr">
@@ -15994,22 +16028,22 @@
       </c>
       <c r="C231" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i2</t>
+          <t>pk.growth.i1</t>
         </is>
       </c>
       <c r="D231" s="9" t="inlineStr">
         <is>
-          <t>Up to 5 no-code automations</t>
+          <t>Up to 3 additional modules</t>
         </is>
       </c>
       <c r="E231" s="9" t="inlineStr">
         <is>
-          <t>5-მდე ავტომატიზაცია</t>
+          <t>3-მდე დამატებითი მოდული</t>
         </is>
       </c>
       <c r="F231" s="9" t="inlineStr">
         <is>
-          <t>До 5 автоматизаций</t>
+          <t>До 3 дополнительных модулей</t>
         </is>
       </c>
       <c r="G231" s="3" t="inlineStr">
@@ -16036,22 +16070,22 @@
       </c>
       <c r="C232" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i3</t>
+          <t>pk.growth.i2</t>
         </is>
       </c>
       <c r="D232" s="9" t="inlineStr">
         <is>
-          <t>Up to 3 automations with custom functions</t>
+          <t>Up to 5 no-code automations</t>
         </is>
       </c>
       <c r="E232" s="9" t="inlineStr">
         <is>
-          <t>3-მდე ავტომატიზაცია custom ფუნქციებით</t>
+          <t>5-მდე ავტომატიზაცია</t>
         </is>
       </c>
       <c r="F232" s="9" t="inlineStr">
         <is>
-          <t>До 3 автоматизаций с custom-функциями</t>
+          <t>До 5 автоматизаций</t>
         </is>
       </c>
       <c r="G232" s="3" t="inlineStr">
@@ -16078,22 +16112,22 @@
       </c>
       <c r="C233" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i4</t>
+          <t>pk.growth.i3</t>
         </is>
       </c>
       <c r="D233" s="9" t="inlineStr">
         <is>
-          <t>Telephony: GEONET or another cloud PBX</t>
+          <t>Up to 3 automations with custom functions</t>
         </is>
       </c>
       <c r="E233" s="9" t="inlineStr">
         <is>
-          <t>ტელეფონია: GEONET ან სხვა cloud PBX</t>
+          <t>3-მდე ავტომატიზაცია custom ფუნქციებით</t>
         </is>
       </c>
       <c r="F233" s="9" t="inlineStr">
         <is>
-          <t>Телефония: GEONET или другая облачная АТС</t>
+          <t>До 3 автоматизаций с custom-функциями</t>
         </is>
       </c>
       <c r="G233" s="3" t="inlineStr">
@@ -16120,22 +16154,22 @@
       </c>
       <c r="C234" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i5</t>
+          <t>pk.growth.i4</t>
         </is>
       </c>
       <c r="D234" s="9" t="inlineStr">
         <is>
-          <t>Call processing workflow in the CRM</t>
+          <t>Telephony: GEONET or another cloud PBX</t>
         </is>
       </c>
       <c r="E234" s="9" t="inlineStr">
         <is>
-          <t>ზარების დამუშავება CRM-ში</t>
+          <t>ტელეფონია: GEONET ან სხვა cloud PBX</t>
         </is>
       </c>
       <c r="F234" s="9" t="inlineStr">
         <is>
-          <t>Обработка звонков в CRM</t>
+          <t>Телефония: GEONET или другая облачная АТС</t>
         </is>
       </c>
       <c r="G234" s="3" t="inlineStr">
@@ -16162,22 +16196,22 @@
       </c>
       <c r="C235" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i6</t>
+          <t>pk.growth.i5</t>
         </is>
       </c>
       <c r="D235" s="9" t="inlineStr">
         <is>
-          <t>Website form + secure webhook</t>
+          <t>Call processing workflow in the CRM</t>
         </is>
       </c>
       <c r="E235" s="9" t="inlineStr">
         <is>
-          <t>საიტის ფორმა + დაცული webhook</t>
+          <t>ზარების დამუშავება CRM-ში</t>
         </is>
       </c>
       <c r="F235" s="9" t="inlineStr">
         <is>
-          <t>Форма сайта + защищённый webhook</t>
+          <t>Обработка звонков в CRM</t>
         </is>
       </c>
       <c r="G235" s="3" t="inlineStr">
@@ -16204,22 +16238,22 @@
       </c>
       <c r="C236" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i7</t>
+          <t>pk.growth.i6</t>
         </is>
       </c>
       <c r="D236" s="9" t="inlineStr">
         <is>
-          <t>Up to 10 reports</t>
+          <t>Website form + secure webhook</t>
         </is>
       </c>
       <c r="E236" s="9" t="inlineStr">
         <is>
-          <t>10-მდე რეპორტი</t>
+          <t>საიტის ფორმა + დაცული webhook</t>
         </is>
       </c>
       <c r="F236" s="9" t="inlineStr">
         <is>
-          <t>До 10 отчётов</t>
+          <t>Форма сайта + защищённый webhook</t>
         </is>
       </c>
       <c r="G236" s="3" t="inlineStr">
@@ -16246,22 +16280,22 @@
       </c>
       <c r="C237" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i8</t>
+          <t>pk.growth.i7</t>
         </is>
       </c>
       <c r="D237" s="9" t="inlineStr">
         <is>
-          <t>AI: Claude connected to your CRM</t>
+          <t>Up to 10 reports</t>
         </is>
       </c>
       <c r="E237" s="9" t="inlineStr">
         <is>
-          <t>AI: Claude დაკავშირებული შენს CRM-თან</t>
+          <t>10-მდე რეპორტი</t>
         </is>
       </c>
       <c r="F237" s="9" t="inlineStr">
         <is>
-          <t>AI: Claude, подключённый к вашей CRM</t>
+          <t>До 10 отчётов</t>
         </is>
       </c>
       <c r="G237" s="3" t="inlineStr">
@@ -16288,22 +16322,22 @@
       </c>
       <c r="C238" s="3" t="inlineStr">
         <is>
-          <t>pk.growth.i9</t>
+          <t>pk.growth.i8</t>
         </is>
       </c>
       <c r="D238" s="9" t="inlineStr">
         <is>
-          <t>60-minute training, recorded</t>
+          <t>AI: Claude connected to your CRM</t>
         </is>
       </c>
       <c r="E238" s="9" t="inlineStr">
         <is>
-          <t>60-წუთიანი ტრენინგი (ჩანაწერით)</t>
+          <t>AI: Claude დაკავშირებული შენს CRM-თან</t>
         </is>
       </c>
       <c r="F238" s="9" t="inlineStr">
         <is>
-          <t>60-минутное обучение с записью</t>
+          <t>AI: Claude, подключённый к вашей CRM</t>
         </is>
       </c>
       <c r="G238" s="3" t="inlineStr">
@@ -16325,27 +16359,27 @@
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
-          <t>Ao</t>
+          <t>Pk</t>
         </is>
       </c>
       <c r="C239" s="3" t="inlineStr">
         <is>
-          <t>ao.4</t>
+          <t>pk.growth.i9</t>
         </is>
       </c>
       <c r="D239" s="9" t="inlineStr">
         <is>
-          <t>Automated lead routing (round-robin)</t>
+          <t>60-minute training, recorded</t>
         </is>
       </c>
       <c r="E239" s="9" t="inlineStr">
         <is>
-          <t>ლიდების ავტომატური განაწილება (round-robin)</t>
+          <t>60-წუთიანი ტრენინგი (ჩანაწერით)</t>
         </is>
       </c>
       <c r="F239" s="9" t="inlineStr">
         <is>
-          <t>Автораспределение лидов (round-robin)</t>
+          <t>60-минутное обучение с записью</t>
         </is>
       </c>
       <c r="G239" s="3" t="inlineStr">
@@ -16372,22 +16406,22 @@
       </c>
       <c r="C240" s="3" t="inlineStr">
         <is>
-          <t>ao.5</t>
+          <t>ao.4</t>
         </is>
       </c>
       <c r="D240" s="9" t="inlineStr">
         <is>
-          <t>Enforced sales stage blueprint</t>
+          <t>Automated lead routing (round-robin)</t>
         </is>
       </c>
       <c r="E240" s="9" t="inlineStr">
         <is>
-          <t>გაყიდვის ეტაპები წესებით (Blueprint)</t>
+          <t>ლიდების ავტომატური განაწილება (round-robin)</t>
         </is>
       </c>
       <c r="F240" s="9" t="inlineStr">
         <is>
-          <t>Этапы продаж с правилами (Blueprint)</t>
+          <t>Автораспределение лидов (round-robin)</t>
         </is>
       </c>
       <c r="G240" s="3" t="inlineStr">
@@ -16414,22 +16448,22 @@
       </c>
       <c r="C241" s="3" t="inlineStr">
         <is>
-          <t>ao.10</t>
+          <t>ao.5</t>
         </is>
       </c>
       <c r="D241" s="9" t="inlineStr">
         <is>
-          <t>Cloud telephony integration (GEONET)</t>
+          <t>Enforced sales stage blueprint</t>
         </is>
       </c>
       <c r="E241" s="9" t="inlineStr">
         <is>
-          <t>ტელეფონიის ინტეგრაცია (GEONET)</t>
+          <t>გაყიდვის ეტაპები წესებით (Blueprint)</t>
         </is>
       </c>
       <c r="F241" s="9" t="inlineStr">
         <is>
-          <t>Интеграция телефонии (GEONET)</t>
+          <t>Этапы продаж с правилами (Blueprint)</t>
         </is>
       </c>
       <c r="G241" s="3" t="inlineStr">
@@ -16456,22 +16490,22 @@
       </c>
       <c r="C242" s="3" t="inlineStr">
         <is>
-          <t>ao.11</t>
+          <t>ao.10</t>
         </is>
       </c>
       <c r="D242" s="9" t="inlineStr">
         <is>
-          <t>WhatsApp Business integration</t>
+          <t>Cloud telephony integration (GEONET)</t>
         </is>
       </c>
       <c r="E242" s="9" t="inlineStr">
         <is>
-          <t>WhatsApp Business-ის ინტეგრაცია</t>
+          <t>ტელეფონიის ინტეგრაცია (GEONET)</t>
         </is>
       </c>
       <c r="F242" s="9" t="inlineStr">
         <is>
-          <t>Интеграция WhatsApp Business</t>
+          <t>Интеграция телефонии (GEONET)</t>
         </is>
       </c>
       <c r="G242" s="3" t="inlineStr">
@@ -16498,22 +16532,22 @@
       </c>
       <c r="C243" s="3" t="inlineStr">
         <is>
-          <t>ao.18</t>
+          <t>ao.11</t>
         </is>
       </c>
       <c r="D243" s="9" t="inlineStr">
         <is>
-          <t>TBC/BOG bank wire deposit matching</t>
+          <t>WhatsApp Business integration</t>
         </is>
       </c>
       <c r="E243" s="9" t="inlineStr">
         <is>
-          <t>TBC/BOG გადარიცხვების ავტომატური შეჯერება</t>
+          <t>WhatsApp Business-ის ინტეგრაცია</t>
         </is>
       </c>
       <c r="F243" s="9" t="inlineStr">
         <is>
-          <t>Автосверка переводов TBC/BOG</t>
+          <t>Интеграция WhatsApp Business</t>
         </is>
       </c>
       <c r="G243" s="3" t="inlineStr">
@@ -16540,22 +16574,22 @@
       </c>
       <c r="C244" s="3" t="inlineStr">
         <is>
-          <t>ao.30</t>
+          <t>ao.18</t>
         </is>
       </c>
       <c r="D244" s="9" t="inlineStr">
         <is>
-          <t>Autonomous web chat assistant (Unitty AI)</t>
+          <t>TBC/BOG bank wire deposit matching</t>
         </is>
       </c>
       <c r="E244" s="9" t="inlineStr">
         <is>
-          <t>AI ჩატ-ასისტენტი საიტზე (Unitty AI)</t>
+          <t>TBC/BOG გადარიცხვების ავტომატური შეჯერება</t>
         </is>
       </c>
       <c r="F244" s="9" t="inlineStr">
         <is>
-          <t>AI чат-ассистент на сайте (Unitty AI)</t>
+          <t>Автосверка переводов TBC/BOG</t>
         </is>
       </c>
       <c r="G244" s="3" t="inlineStr">
@@ -16582,22 +16616,22 @@
       </c>
       <c r="C245" s="3" t="inlineStr">
         <is>
-          <t>ao.38</t>
+          <t>ao.30</t>
         </is>
       </c>
       <c r="D245" s="9" t="inlineStr">
         <is>
-          <t>Enterprise ERP sync (1C / FINA / SAP)</t>
+          <t>Autonomous web chat assistant (Unitty AI)</t>
         </is>
       </c>
       <c r="E245" s="9" t="inlineStr">
         <is>
-          <t>ERP სინქრონიზაცია (1C / FINA / SAP)</t>
+          <t>AI ჩატ-ასისტენტი საიტზე (Unitty AI)</t>
         </is>
       </c>
       <c r="F245" s="9" t="inlineStr">
         <is>
-          <t>Синхронизация с ERP (1C / FINA / SAP)</t>
+          <t>AI чат-ассистент на сайте (Unitty AI)</t>
         </is>
       </c>
       <c r="G245" s="3" t="inlineStr">
@@ -16624,22 +16658,22 @@
       </c>
       <c r="C246" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.data</t>
+          <t>ao.38</t>
         </is>
       </c>
       <c r="D246" s="9" t="inlineStr">
         <is>
-          <t>Data foundation</t>
+          <t>Enterprise ERP sync (1C / FINA / SAP)</t>
         </is>
       </c>
       <c r="E246" s="9" t="inlineStr">
         <is>
-          <t>მონაცემები</t>
+          <t>ERP სინქრონიზაცია (1C / FINA / SAP)</t>
         </is>
       </c>
       <c r="F246" s="9" t="inlineStr">
         <is>
-          <t>Данные</t>
+          <t>Синхронизация с ERP (1C / FINA / SAP)</t>
         </is>
       </c>
       <c r="G246" s="3" t="inlineStr">
@@ -16666,22 +16700,22 @@
       </c>
       <c r="C247" s="3" t="inlineStr">
         <is>
-          <t>ao.1</t>
+          <t>ao.cat.data</t>
         </is>
       </c>
       <c r="D247" s="9" t="inlineStr">
         <is>
-          <t>Georgian phone validation &amp; deduplication (+995)</t>
+          <t>Data foundation</t>
         </is>
       </c>
       <c r="E247" s="9" t="inlineStr">
         <is>
-          <t>ტელეფონის ნომრების ვალიდაცია (+995) და დუბლიკატების გასუფთავება</t>
+          <t>მონაცემები</t>
         </is>
       </c>
       <c r="F247" s="9" t="inlineStr">
         <is>
-          <t>Проверка номеров (+995) и дубли</t>
+          <t>Данные</t>
         </is>
       </c>
       <c r="G247" s="3" t="inlineStr">
@@ -16708,22 +16742,22 @@
       </c>
       <c r="C248" s="3" t="inlineStr">
         <is>
-          <t>ao.2</t>
+          <t>ao.1</t>
         </is>
       </c>
       <c r="D248" s="9" t="inlineStr">
         <is>
-          <t>Legacy spreadsheet → CRM migration</t>
+          <t>Georgian phone validation &amp; deduplication (+995)</t>
         </is>
       </c>
       <c r="E248" s="9" t="inlineStr">
         <is>
-          <t>Excel-ის ცხრილების გადმოტანა CRM-ში</t>
+          <t>ტელეფონის ნომრების ვალიდაცია (+995) და დუბლიკატების გასუფთავება</t>
         </is>
       </c>
       <c r="F248" s="9" t="inlineStr">
         <is>
-          <t>Перенос таблиц Excel в CRM</t>
+          <t>Проверка номеров (+995) и дубли</t>
         </is>
       </c>
       <c r="G248" s="3" t="inlineStr">
@@ -16750,22 +16784,22 @@
       </c>
       <c r="C249" s="3" t="inlineStr">
         <is>
-          <t>ao.3</t>
+          <t>ao.2</t>
         </is>
       </c>
       <c r="D249" s="9" t="inlineStr">
         <is>
-          <t>Property stock database migration</t>
+          <t>Legacy spreadsheet → CRM migration</t>
         </is>
       </c>
       <c r="E249" s="9" t="inlineStr">
         <is>
-          <t>უძრავი ქონების / ობიექტების ბაზის მიგრაცია</t>
+          <t>Excel-ის ცხრილების გადმოტანა CRM-ში</t>
         </is>
       </c>
       <c r="F249" s="9" t="inlineStr">
         <is>
-          <t>Перенос базы объектов недвижимости</t>
+          <t>Перенос таблиц Excel в CRM</t>
         </is>
       </c>
       <c r="G249" s="3" t="inlineStr">
@@ -16792,22 +16826,22 @@
       </c>
       <c r="C250" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.sales</t>
+          <t>ao.3</t>
         </is>
       </c>
       <c r="D250" s="9" t="inlineStr">
         <is>
-          <t>Sales automation</t>
+          <t>Property stock database migration</t>
         </is>
       </c>
       <c r="E250" s="9" t="inlineStr">
         <is>
-          <t>გაყიდვების ავტომატიზაცია</t>
+          <t>უძრავი ქონების / ობიექტების ბაზის მიგრაცია</t>
         </is>
       </c>
       <c r="F250" s="9" t="inlineStr">
         <is>
-          <t>Автоматизация продаж</t>
+          <t>Перенос базы объектов недвижимости</t>
         </is>
       </c>
       <c r="G250" s="3" t="inlineStr">
@@ -16834,22 +16868,22 @@
       </c>
       <c r="C251" s="3" t="inlineStr">
         <is>
-          <t>ao.6</t>
+          <t>ao.cat.sales</t>
         </is>
       </c>
       <c r="D251" s="9" t="inlineStr">
         <is>
-          <t>Follow-up reminders &amp; alerts</t>
+          <t>Sales automation</t>
         </is>
       </c>
       <c r="E251" s="9" t="inlineStr">
         <is>
-          <t>follow-up შეხსენებები და შეტყობინებები</t>
+          <t>გაყიდვების ავტომატიზაცია</t>
         </is>
       </c>
       <c r="F251" s="9" t="inlineStr">
         <is>
-          <t>Напоминания и уведомления о follow-up</t>
+          <t>Автоматизация продаж</t>
         </is>
       </c>
       <c r="G251" s="3" t="inlineStr">
@@ -16876,22 +16910,22 @@
       </c>
       <c r="C252" s="3" t="inlineStr">
         <is>
-          <t>ao.7</t>
+          <t>ao.6</t>
         </is>
       </c>
       <c r="D252" s="9" t="inlineStr">
         <is>
-          <t>One-click agreement PDF generator</t>
+          <t>Follow-up reminders &amp; alerts</t>
         </is>
       </c>
       <c r="E252" s="9" t="inlineStr">
         <is>
-          <t>ხელშეკრულების PDF ერთი დაჭერით</t>
+          <t>follow-up შეხსენებები და შეტყობინებები</t>
         </is>
       </c>
       <c r="F252" s="9" t="inlineStr">
         <is>
-          <t>PDF договора в один клик</t>
+          <t>Напоминания и уведомления о follow-up</t>
         </is>
       </c>
       <c r="G252" s="3" t="inlineStr">
@@ -16918,22 +16952,22 @@
       </c>
       <c r="C253" s="3" t="inlineStr">
         <is>
-          <t>ao.8</t>
+          <t>ao.7</t>
         </is>
       </c>
       <c r="D253" s="9" t="inlineStr">
         <is>
-          <t>First-response SLA tracker</t>
+          <t>One-click agreement PDF generator</t>
         </is>
       </c>
       <c r="E253" s="9" t="inlineStr">
         <is>
-          <t>პირველი პასუხის დროის (SLA) კონტროლი</t>
+          <t>ხელშეკრულების PDF ერთი დაჭერით</t>
         </is>
       </c>
       <c r="F253" s="9" t="inlineStr">
         <is>
-          <t>Контроль времени первого ответа (SLA)</t>
+          <t>PDF договора в один клик</t>
         </is>
       </c>
       <c r="G253" s="3" t="inlineStr">
@@ -16960,22 +16994,22 @@
       </c>
       <c r="C254" s="3" t="inlineStr">
         <is>
-          <t>ao.9</t>
+          <t>ao.8</t>
         </is>
       </c>
       <c r="D254" s="9" t="inlineStr">
         <is>
-          <t>Broker commission tracking</t>
+          <t>First-response SLA tracker</t>
         </is>
       </c>
       <c r="E254" s="9" t="inlineStr">
         <is>
-          <t>ბროკერების საკომისიოების აღრიცხვა</t>
+          <t>პირველი პასუხის დროის (SLA) კონტროლი</t>
         </is>
       </c>
       <c r="F254" s="9" t="inlineStr">
         <is>
-          <t>Учёт комиссий брокеров</t>
+          <t>Контроль времени первого ответа (SLA)</t>
         </is>
       </c>
       <c r="G254" s="3" t="inlineStr">
@@ -17002,22 +17036,22 @@
       </c>
       <c r="C255" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.comms</t>
+          <t>ao.9</t>
         </is>
       </c>
       <c r="D255" s="9" t="inlineStr">
         <is>
-          <t>Communication</t>
+          <t>Broker commission tracking</t>
         </is>
       </c>
       <c r="E255" s="9" t="inlineStr">
         <is>
-          <t>კომუნიკაცია</t>
+          <t>ბროკერების საკომისიოების აღრიცხვა</t>
         </is>
       </c>
       <c r="F255" s="9" t="inlineStr">
         <is>
-          <t>Коммуникации</t>
+          <t>Учёт комиссий брокеров</t>
         </is>
       </c>
       <c r="G255" s="3" t="inlineStr">
@@ -17044,22 +17078,22 @@
       </c>
       <c r="C256" s="3" t="inlineStr">
         <is>
-          <t>ao.12</t>
+          <t>ao.cat.comms</t>
         </is>
       </c>
       <c r="D256" s="9" t="inlineStr">
         <is>
-          <t>Email + calendar 2-way sync</t>
+          <t>Communication</t>
         </is>
       </c>
       <c r="E256" s="9" t="inlineStr">
         <is>
-          <t>ელფოსტისა და კალენდრის ორმხრივი სინქრონიზაცია</t>
+          <t>კომუნიკაცია</t>
         </is>
       </c>
       <c r="F256" s="9" t="inlineStr">
         <is>
-          <t>Двусторонняя синхронизация почты и календаря</t>
+          <t>Коммуникации</t>
         </is>
       </c>
       <c r="G256" s="3" t="inlineStr">
@@ -17086,22 +17120,22 @@
       </c>
       <c r="C257" s="3" t="inlineStr">
         <is>
-          <t>ao.13</t>
+          <t>ao.12</t>
         </is>
       </c>
       <c r="D257" s="9" t="inlineStr">
         <is>
-          <t>Missed-call recovery &amp; SMS callback</t>
+          <t>Email + calendar 2-way sync</t>
         </is>
       </c>
       <c r="E257" s="9" t="inlineStr">
         <is>
-          <t>გამოტოვებული ზარების დამუშავება და ავტომატური SMS</t>
+          <t>ელფოსტისა და კალენდრის ორმხრივი სინქრონიზაცია</t>
         </is>
       </c>
       <c r="F257" s="9" t="inlineStr">
         <is>
-          <t>Возврат пропущенных звонков и SMS</t>
+          <t>Двусторонняя синхронизация почты и календаря</t>
         </is>
       </c>
       <c r="G257" s="3" t="inlineStr">
@@ -17128,22 +17162,22 @@
       </c>
       <c r="C258" s="3" t="inlineStr">
         <is>
-          <t>ao.14</t>
+          <t>ao.13</t>
         </is>
       </c>
       <c r="D258" s="9" t="inlineStr">
         <is>
-          <t>Messaging bot lead capture webhook</t>
+          <t>Missed-call recovery &amp; SMS callback</t>
         </is>
       </c>
       <c r="E258" s="9" t="inlineStr">
         <is>
-          <t>ჩატბოტის ლიდების პირდაპირი ინტეგრაცია CRM-ში</t>
+          <t>გამოტოვებული ზარების დამუშავება და ავტომატური SMS</t>
         </is>
       </c>
       <c r="F258" s="9" t="inlineStr">
         <is>
-          <t>Лиды из чат-бота сразу в CRM</t>
+          <t>Возврат пропущенных звонков и SMS</t>
         </is>
       </c>
       <c r="G258" s="3" t="inlineStr">
@@ -17170,22 +17204,22 @@
       </c>
       <c r="C259" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.mkt</t>
+          <t>ao.14</t>
         </is>
       </c>
       <c r="D259" s="9" t="inlineStr">
         <is>
-          <t>Marketing &amp; growth</t>
+          <t>Messaging bot lead capture webhook</t>
         </is>
       </c>
       <c r="E259" s="9" t="inlineStr">
         <is>
-          <t>მარკეტინგი</t>
+          <t>ჩატბოტის ლიდების პირდაპირი ინტეგრაცია CRM-ში</t>
         </is>
       </c>
       <c r="F259" s="9" t="inlineStr">
         <is>
-          <t>Маркетинг</t>
+          <t>Лиды из чат-бота сразу в CRM</t>
         </is>
       </c>
       <c r="G259" s="3" t="inlineStr">
@@ -17212,22 +17246,22 @@
       </c>
       <c r="C260" s="3" t="inlineStr">
         <is>
-          <t>ao.15</t>
+          <t>ao.cat.mkt</t>
         </is>
       </c>
       <c r="D260" s="9" t="inlineStr">
         <is>
-          <t>Website lead form + webhook</t>
+          <t>Marketing &amp; growth</t>
         </is>
       </c>
       <c r="E260" s="9" t="inlineStr">
         <is>
-          <t>საიტის ფორმა + webhook</t>
+          <t>მარკეტინგი</t>
         </is>
       </c>
       <c r="F260" s="9" t="inlineStr">
         <is>
-          <t>Форма сайта + webhook</t>
+          <t>Маркетинг</t>
         </is>
       </c>
       <c r="G260" s="3" t="inlineStr">
@@ -17254,22 +17288,22 @@
       </c>
       <c r="C261" s="3" t="inlineStr">
         <is>
-          <t>ao.16</t>
+          <t>ao.15</t>
         </is>
       </c>
       <c r="D261" s="9" t="inlineStr">
         <is>
-          <t>Lead source ROI &amp; campaign attribution</t>
+          <t>Website lead form + webhook</t>
         </is>
       </c>
       <c r="E261" s="9" t="inlineStr">
         <is>
-          <t>ლიდების წყაროების ROI და კამპანიების ატრიბუცია</t>
+          <t>საიტის ფორმა + webhook</t>
         </is>
       </c>
       <c r="F261" s="9" t="inlineStr">
         <is>
-          <t>ROI источников и атрибуция кампаний</t>
+          <t>Форма сайта + webhook</t>
         </is>
       </c>
       <c r="G261" s="3" t="inlineStr">
@@ -17296,22 +17330,22 @@
       </c>
       <c r="C262" s="3" t="inlineStr">
         <is>
-          <t>ao.17</t>
+          <t>ao.16</t>
         </is>
       </c>
       <c r="D262" s="9" t="inlineStr">
         <is>
-          <t>Email campaigns: account setup &amp; contact sync</t>
+          <t>Lead source ROI &amp; campaign attribution</t>
         </is>
       </c>
       <c r="E262" s="9" t="inlineStr">
         <is>
-          <t>იმეილ კამპანიები: ანგარიშის გამართვა და კონტაქტების სინქრონიზაცია</t>
+          <t>ლიდების წყაროების ROI და კამპანიების ატრიბუცია</t>
         </is>
       </c>
       <c r="F262" s="9" t="inlineStr">
         <is>
-          <t>Email-рассылки: настройка и синхронизация контактов</t>
+          <t>ROI источников и атрибуция кампаний</t>
         </is>
       </c>
       <c r="G262" s="3" t="inlineStr">
@@ -17338,22 +17372,22 @@
       </c>
       <c r="C263" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.fin</t>
+          <t>ao.17</t>
         </is>
       </c>
       <c r="D263" s="9" t="inlineStr">
         <is>
-          <t>Fintech &amp; accounting</t>
+          <t>Email campaigns: account setup &amp; contact sync</t>
         </is>
       </c>
       <c r="E263" s="9" t="inlineStr">
         <is>
-          <t>ფინანსები და ბანკები</t>
+          <t>იმეილ კამპანიები: ანგარიშის გამართვა და კონტაქტების სინქრონიზაცია</t>
         </is>
       </c>
       <c r="F263" s="9" t="inlineStr">
         <is>
-          <t>Финансы и банки</t>
+          <t>Email-рассылки: настройка и синхронизация контактов</t>
         </is>
       </c>
       <c r="G263" s="3" t="inlineStr">
@@ -17380,22 +17414,22 @@
       </c>
       <c r="C264" s="3" t="inlineStr">
         <is>
-          <t>ao.19</t>
+          <t>ao.cat.fin</t>
         </is>
       </c>
       <c r="D264" s="9" t="inlineStr">
         <is>
-          <t>Multi-currency reconciliation (GEL/USD/EUR)</t>
+          <t>Fintech &amp; accounting</t>
         </is>
       </c>
       <c r="E264" s="9" t="inlineStr">
         <is>
-          <t>მრავალვალუტიანი ავტომატური შეჯერება (GEL/USD/EUR)</t>
+          <t>ფინანსები და ბანკები</t>
         </is>
       </c>
       <c r="F264" s="9" t="inlineStr">
         <is>
-          <t>Мультивалютная сверка (GEL/USD/EUR)</t>
+          <t>Финансы и банки</t>
         </is>
       </c>
       <c r="G264" s="3" t="inlineStr">
@@ -17422,22 +17456,22 @@
       </c>
       <c r="C265" s="3" t="inlineStr">
         <is>
-          <t>ao.20</t>
+          <t>ao.19</t>
         </is>
       </c>
       <c r="D265" s="9" t="inlineStr">
         <is>
-          <t>NBG daily exchange rate sync</t>
+          <t>Multi-currency reconciliation (GEL/USD/EUR)</t>
         </is>
       </c>
       <c r="E265" s="9" t="inlineStr">
         <is>
-          <t>ეროვნული ბანკის (NBG) კურსის ყოველდღიური სინქრონიზაცია</t>
+          <t>მრავალვალუტიანი ავტომატური შეჯერება (GEL/USD/EUR)</t>
         </is>
       </c>
       <c r="F265" s="9" t="inlineStr">
         <is>
-          <t>Ежедневный курс НБГ</t>
+          <t>Мультивалютная сверка (GEL/USD/EUR)</t>
         </is>
       </c>
       <c r="G265" s="3" t="inlineStr">
@@ -17464,22 +17498,22 @@
       </c>
       <c r="C266" s="3" t="inlineStr">
         <is>
-          <t>ao.21</t>
+          <t>ao.20</t>
         </is>
       </c>
       <c r="D266" s="9" t="inlineStr">
         <is>
-          <t>Ambiguous payment reference fallback queue</t>
+          <t>NBG daily exchange rate sync</t>
         </is>
       </c>
       <c r="E266" s="9" t="inlineStr">
         <is>
-          <t>დაუზუსტებელი გადარიცხვების დამუშავების რიგი</t>
+          <t>ეროვნული ბანკის (NBG) კურსის ყოველდღიური სინქრონიზაცია</t>
         </is>
       </c>
       <c r="F266" s="9" t="inlineStr">
         <is>
-          <t>Очередь неопознанных платежей</t>
+          <t>Ежедневный курс НБГ</t>
         </is>
       </c>
       <c r="G266" s="3" t="inlineStr">
@@ -17506,22 +17540,22 @@
       </c>
       <c r="C267" s="3" t="inlineStr">
         <is>
-          <t>ao.22</t>
+          <t>ao.21</t>
         </is>
       </c>
       <c r="D267" s="9" t="inlineStr">
         <is>
-          <t>Dynamic installment payment schedule</t>
+          <t>Ambiguous payment reference fallback queue</t>
         </is>
       </c>
       <c r="E267" s="9" t="inlineStr">
         <is>
-          <t>შიდა განვადების დინამიკური გრაფიკი</t>
+          <t>დაუზუსტებელი გადარიცხვების დამუშავების რიგი</t>
         </is>
       </c>
       <c r="F267" s="9" t="inlineStr">
         <is>
-          <t>График рассрочки</t>
+          <t>Очередь неопознанных платежей</t>
         </is>
       </c>
       <c r="G267" s="3" t="inlineStr">
@@ -17548,22 +17582,22 @@
       </c>
       <c r="C268" s="3" t="inlineStr">
         <is>
-          <t>ao.23</t>
+          <t>ao.22</t>
         </is>
       </c>
       <c r="D268" s="9" t="inlineStr">
         <is>
-          <t>Overdue debt alert &amp; SMS warning</t>
+          <t>Dynamic installment payment schedule</t>
         </is>
       </c>
       <c r="E268" s="9" t="inlineStr">
         <is>
-          <t>ვადაგადაცილებული დავალიანების SMS შეხსენება</t>
+          <t>შიდა განვადების დინამიკური გრაფიკი</t>
         </is>
       </c>
       <c r="F268" s="9" t="inlineStr">
         <is>
-          <t>SMS о просроченной задолженности</t>
+          <t>График рассрочки</t>
         </is>
       </c>
       <c r="G268" s="3" t="inlineStr">
@@ -17590,22 +17624,22 @@
       </c>
       <c r="C269" s="3" t="inlineStr">
         <is>
-          <t>ao.24</t>
+          <t>ao.23</t>
         </is>
       </c>
       <c r="D269" s="9" t="inlineStr">
         <is>
-          <t>SMS gateway &amp; OTP verification</t>
+          <t>Overdue debt alert &amp; SMS warning</t>
         </is>
       </c>
       <c r="E269" s="9" t="inlineStr">
         <is>
-          <t>SMS გეითვეი და OTP ვერიფიკაცია</t>
+          <t>ვადაგადაცილებული დავალიანების SMS შეხსენება</t>
         </is>
       </c>
       <c r="F269" s="9" t="inlineStr">
         <is>
-          <t>SMS-шлюз и OTP-верификация</t>
+          <t>SMS о просроченной задолженности</t>
         </is>
       </c>
       <c r="G269" s="3" t="inlineStr">
@@ -17632,22 +17666,22 @@
       </c>
       <c r="C270" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.cx</t>
+          <t>ao.24</t>
         </is>
       </c>
       <c r="D270" s="9" t="inlineStr">
         <is>
-          <t>Customer experience</t>
+          <t>SMS gateway &amp; OTP verification</t>
         </is>
       </c>
       <c r="E270" s="9" t="inlineStr">
         <is>
-          <t>მომხმარებლის მომსახურება</t>
+          <t>SMS გეითვეი და OTP ვერიფიკაცია</t>
         </is>
       </c>
       <c r="F270" s="9" t="inlineStr">
         <is>
-          <t>Клиентский сервис</t>
+          <t>SMS-шлюз и OTP-верификация</t>
         </is>
       </c>
       <c r="G270" s="3" t="inlineStr">
@@ -17674,22 +17708,22 @@
       </c>
       <c r="C271" s="3" t="inlineStr">
         <is>
-          <t>ao.25</t>
+          <t>ao.cat.cx</t>
         </is>
       </c>
       <c r="D271" s="9" t="inlineStr">
         <is>
-          <t>Omnichannel support ticketing (Zoho Desk)</t>
+          <t>Customer experience</t>
         </is>
       </c>
       <c r="E271" s="9" t="inlineStr">
         <is>
-          <t>ომნიარხული (Omnichannel) მხარდაჭერის ტიკეტები (Zoho Desk)</t>
+          <t>მომხმარებლის მომსახურება</t>
         </is>
       </c>
       <c r="F271" s="9" t="inlineStr">
         <is>
-          <t>Омниканальные тикеты (Zoho Desk)</t>
+          <t>Клиентский сервис</t>
         </is>
       </c>
       <c r="G271" s="3" t="inlineStr">
@@ -17716,22 +17750,22 @@
       </c>
       <c r="C272" s="3" t="inlineStr">
         <is>
-          <t>ao.26</t>
+          <t>ao.25</t>
         </is>
       </c>
       <c r="D272" s="9" t="inlineStr">
         <is>
-          <t>Multi-tier SLA escalation matrix</t>
+          <t>Omnichannel support ticketing (Zoho Desk)</t>
         </is>
       </c>
       <c r="E272" s="9" t="inlineStr">
         <is>
-          <t>მრავალდონიანი SLA-ს ესკალაციის მატრიცა</t>
+          <t>ომნიარხული (Omnichannel) მხარდაჭერის ტიკეტები (Zoho Desk)</t>
         </is>
       </c>
       <c r="F272" s="9" t="inlineStr">
         <is>
-          <t>Матрица эскалации SLA</t>
+          <t>Омниканальные тикеты (Zoho Desk)</t>
         </is>
       </c>
       <c r="G272" s="3" t="inlineStr">
@@ -17758,22 +17792,22 @@
       </c>
       <c r="C273" s="3" t="inlineStr">
         <is>
-          <t>ao.27</t>
+          <t>ao.26</t>
         </is>
       </c>
       <c r="D273" s="9" t="inlineStr">
         <is>
-          <t>Post-ticket NPS/CSAT feedback loop</t>
+          <t>Multi-tier SLA escalation matrix</t>
         </is>
       </c>
       <c r="E273" s="9" t="inlineStr">
         <is>
-          <t>NPS/CSAT კმაყოფილების შეფასება ტიკეტის დახურვის შემდეგ</t>
+          <t>მრავალდონიანი SLA-ს ესკალაციის მატრიცა</t>
         </is>
       </c>
       <c r="F273" s="9" t="inlineStr">
         <is>
-          <t>Оценка NPS/CSAT после тикета</t>
+          <t>Матрица эскалации SLA</t>
         </is>
       </c>
       <c r="G273" s="3" t="inlineStr">
@@ -17800,22 +17834,22 @@
       </c>
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>ao.28</t>
+          <t>ao.27</t>
         </is>
       </c>
       <c r="D274" s="9" t="inlineStr">
         <is>
-          <t>Dynamic KYC intake smart form</t>
+          <t>Post-ticket NPS/CSAT feedback loop</t>
         </is>
       </c>
       <c r="E274" s="9" t="inlineStr">
         <is>
-          <t>KYC-ის დინამიკური ჭკვიანი ფორმა</t>
+          <t>NPS/CSAT კმაყოფილების შეფასება ტიკეტის დახურვის შემდეგ</t>
         </is>
       </c>
       <c r="F274" s="9" t="inlineStr">
         <is>
-          <t>Умная KYC-форма</t>
+          <t>Оценка NPS/CSAT после тикета</t>
         </is>
       </c>
       <c r="G274" s="3" t="inlineStr">
@@ -17842,22 +17876,22 @@
       </c>
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>ao.29</t>
+          <t>ao.28</t>
         </is>
       </c>
       <c r="D275" s="9" t="inlineStr">
         <is>
-          <t>Warranty expiration alerts</t>
+          <t>Dynamic KYC intake smart form</t>
         </is>
       </c>
       <c r="E275" s="9" t="inlineStr">
         <is>
-          <t>გარანტიის ვადის შეხსენებები</t>
+          <t>KYC-ის დინამიკური ჭკვიანი ფორმა</t>
         </is>
       </c>
       <c r="F275" s="9" t="inlineStr">
         <is>
-          <t>Напоминания об окончании гарантии</t>
+          <t>Умная KYC-форма</t>
         </is>
       </c>
       <c r="G275" s="3" t="inlineStr">
@@ -17884,22 +17918,22 @@
       </c>
       <c r="C276" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.ai</t>
+          <t>ao.29</t>
         </is>
       </c>
       <c r="D276" s="9" t="inlineStr">
         <is>
-          <t>AI &amp; automation</t>
+          <t>Warranty expiration alerts</t>
         </is>
       </c>
       <c r="E276" s="9" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>გარანტიის ვადის შეხსენებები</t>
         </is>
       </c>
       <c r="F276" s="9" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Напоминания об окончании гарантии</t>
         </is>
       </c>
       <c r="G276" s="3" t="inlineStr">
@@ -17926,22 +17960,22 @@
       </c>
       <c r="C277" s="3" t="inlineStr">
         <is>
-          <t>ao.31</t>
+          <t>ao.cat.ai</t>
         </is>
       </c>
       <c r="D277" s="9" t="inlineStr">
         <is>
-          <t>Georgian voice meeting transcription</t>
+          <t>AI &amp; automation</t>
         </is>
       </c>
       <c r="E277" s="9" t="inlineStr">
         <is>
-          <t>ქართული შეხვედრების ტრანსკრიფცია</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="F277" s="9" t="inlineStr">
         <is>
-          <t>Транскрипция встреч на грузинском</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="G277" s="3" t="inlineStr">
@@ -17968,22 +18002,22 @@
       </c>
       <c r="C278" s="3" t="inlineStr">
         <is>
-          <t>ao.32</t>
+          <t>ao.31</t>
         </is>
       </c>
       <c r="D278" s="9" t="inlineStr">
         <is>
-          <t>Audio call sentiment extractor</t>
+          <t>Georgian voice meeting transcription</t>
         </is>
       </c>
       <c r="E278" s="9" t="inlineStr">
         <is>
-          <t>სატელეფონო ზარის ემოციური განწყობის (Sentiment) ანალიზი</t>
+          <t>ქართული შეხვედრების ტრანსკრიფცია</t>
         </is>
       </c>
       <c r="F278" s="9" t="inlineStr">
         <is>
-          <t>Анализ тональности звонков</t>
+          <t>Транскрипция встреч на грузинском</t>
         </is>
       </c>
       <c r="G278" s="3" t="inlineStr">
@@ -18010,22 +18044,22 @@
       </c>
       <c r="C279" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.ind</t>
+          <t>ao.32</t>
         </is>
       </c>
       <c r="D279" s="9" t="inlineStr">
         <is>
-          <t>Industry solutions</t>
+          <t>Audio call sentiment extractor</t>
         </is>
       </c>
       <c r="E279" s="9" t="inlineStr">
         <is>
-          <t>დარგობრივი</t>
+          <t>სატელეფონო ზარის ემოციური განწყობის (Sentiment) ანალიზი</t>
         </is>
       </c>
       <c r="F279" s="9" t="inlineStr">
         <is>
-          <t>Отраслевые</t>
+          <t>Анализ тональности звонков</t>
         </is>
       </c>
       <c r="G279" s="3" t="inlineStr">
@@ -18052,22 +18086,22 @@
       </c>
       <c r="C280" s="3" t="inlineStr">
         <is>
-          <t>ao.33</t>
+          <t>ao.cat.ind</t>
         </is>
       </c>
       <c r="D280" s="9" t="inlineStr">
         <is>
-          <t>Real estate unit inventory &amp; anti-double-booking</t>
+          <t>Industry solutions</t>
         </is>
       </c>
       <c r="E280" s="9" t="inlineStr">
         <is>
-          <t>უძრავი ქონება: ბინების ინვენტარიზაცია ორმაგი ჯავშნების პრევენციით</t>
+          <t>დარგობრივი</t>
         </is>
       </c>
       <c r="F280" s="9" t="inlineStr">
         <is>
-          <t>Недвижимость: учёт квартир без двойной брони</t>
+          <t>Отраслевые</t>
         </is>
       </c>
       <c r="G280" s="3" t="inlineStr">
@@ -18094,22 +18128,22 @@
       </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
-          <t>ao.34</t>
+          <t>ao.33</t>
         </is>
       </c>
       <c r="D281" s="9" t="inlineStr">
         <is>
-          <t>Client preference proactive matcher</t>
+          <t>Real estate unit inventory &amp; anti-double-booking</t>
         </is>
       </c>
       <c r="E281" s="9" t="inlineStr">
         <is>
-          <t>კლიენტის მოთხოვნებთან ობიექტების ავტომატური შეთავსება (Matching)</t>
+          <t>უძრავი ქონება: ბინების ინვენტარიზაცია ორმაგი ჯავშნების პრევენციით</t>
         </is>
       </c>
       <c r="F281" s="9" t="inlineStr">
         <is>
-          <t>Автоподбор по пожеланиям клиента</t>
+          <t>Недвижимость: учёт квартир без двойной брони</t>
         </is>
       </c>
       <c r="G281" s="3" t="inlineStr">
@@ -18136,22 +18170,22 @@
       </c>
       <c r="C282" s="3" t="inlineStr">
         <is>
-          <t>ao.35</t>
+          <t>ao.34</t>
         </is>
       </c>
       <c r="D282" s="9" t="inlineStr">
         <is>
-          <t>Reservation expiration timer</t>
+          <t>Client preference proactive matcher</t>
         </is>
       </c>
       <c r="E282" s="9" t="inlineStr">
         <is>
-          <t>ჯავშნის ვადის ავტომატური ტაიმერი</t>
+          <t>კლიენტის მოთხოვნებთან ობიექტების ავტომატური შეთავსება (Matching)</t>
         </is>
       </c>
       <c r="F282" s="9" t="inlineStr">
         <is>
-          <t>Таймер истечения брони</t>
+          <t>Автоподбор по пожеланиям клиента</t>
         </is>
       </c>
       <c r="G282" s="3" t="inlineStr">
@@ -18178,22 +18212,22 @@
       </c>
       <c r="C283" s="3" t="inlineStr">
         <is>
-          <t>ao.36</t>
+          <t>ao.35</t>
         </is>
       </c>
       <c r="D283" s="9" t="inlineStr">
         <is>
-          <t>Floor plan &amp; proposal PDF generator</t>
+          <t>Reservation expiration timer</t>
         </is>
       </c>
       <c r="E283" s="9" t="inlineStr">
         <is>
-          <t>გეგმარებისა და შეთავაზების PDF-ის გენერირება ერთი დაჭერით</t>
+          <t>ჯავშნის ვადის ავტომატური ტაიმერი</t>
         </is>
       </c>
       <c r="F283" s="9" t="inlineStr">
         <is>
-          <t>PDF планировки и предложения</t>
+          <t>Таймер истечения брони</t>
         </is>
       </c>
       <c r="G283" s="3" t="inlineStr">
@@ -18220,22 +18254,22 @@
       </c>
       <c r="C284" s="3" t="inlineStr">
         <is>
-          <t>ao.37</t>
+          <t>ao.36</t>
         </is>
       </c>
       <c r="D284" s="9" t="inlineStr">
         <is>
-          <t>Field service visit tracking + approval</t>
+          <t>Floor plan &amp; proposal PDF generator</t>
         </is>
       </c>
       <c r="E284" s="9" t="inlineStr">
         <is>
-          <t>საველე ვიზიტების მართვა და დადასტურება</t>
+          <t>გეგმარებისა და შეთავაზების PDF-ის გენერირება ერთი დაჭერით</t>
         </is>
       </c>
       <c r="F284" s="9" t="inlineStr">
         <is>
-          <t>Учёт выездов и подтверждение</t>
+          <t>PDF планировки и предложения</t>
         </is>
       </c>
       <c r="G284" s="3" t="inlineStr">
@@ -18262,22 +18296,22 @@
       </c>
       <c r="C285" s="3" t="inlineStr">
         <is>
-          <t>ao.cat.ops</t>
+          <t>ao.37</t>
         </is>
       </c>
       <c r="D285" s="9" t="inlineStr">
         <is>
-          <t>Operations &amp; ERP</t>
+          <t>Field service visit tracking + approval</t>
         </is>
       </c>
       <c r="E285" s="9" t="inlineStr">
         <is>
-          <t>ოპერაციები და ERP</t>
+          <t>საველე ვიზიტების მართვა და დადასტურება</t>
         </is>
       </c>
       <c r="F285" s="9" t="inlineStr">
         <is>
-          <t>Операции и ERP</t>
+          <t>Учёт выездов и подтверждение</t>
         </is>
       </c>
       <c r="G285" s="3" t="inlineStr">
@@ -18304,22 +18338,22 @@
       </c>
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>ao.39</t>
+          <t>ao.cat.ops</t>
         </is>
       </c>
       <c r="D286" s="9" t="inlineStr">
         <is>
-          <t>Cold storage WMS &amp; automated billing</t>
+          <t>Operations &amp; ERP</t>
         </is>
       </c>
       <c r="E286" s="9" t="inlineStr">
         <is>
-          <t>სამაცივრე საწყობის WMS სისტემა და ავტომატური ბილინგი</t>
+          <t>ოპერაციები და ERP</t>
         </is>
       </c>
       <c r="F286" s="9" t="inlineStr">
         <is>
-          <t>WMS холодного склада и биллинг</t>
+          <t>Операции и ERP</t>
         </is>
       </c>
       <c r="G286" s="3" t="inlineStr">
@@ -18346,22 +18380,22 @@
       </c>
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>ao.40</t>
+          <t>ao.39</t>
         </is>
       </c>
       <c r="D287" s="9" t="inlineStr">
         <is>
-          <t>Construction operations &amp; budget tracker</t>
+          <t>Cold storage WMS &amp; automated billing</t>
         </is>
       </c>
       <c r="E287" s="9" t="inlineStr">
         <is>
-          <t>სამშენებლო ოპერაციებისა და ბიუჯეტის მართვა</t>
+          <t>სამაცივრე საწყობის WMS სისტემა და ავტომატური ბილინგი</t>
         </is>
       </c>
       <c r="F287" s="9" t="inlineStr">
         <is>
-          <t>Стройка: операции и бюджет</t>
+          <t>WMS холодного склада и биллинг</t>
         </is>
       </c>
       <c r="G287" s="3" t="inlineStr">
@@ -18388,22 +18422,22 @@
       </c>
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>ao.41</t>
+          <t>ao.40</t>
         </is>
       </c>
       <c r="D288" s="9" t="inlineStr">
         <is>
-          <t>Predictive debtor call queue</t>
+          <t>Construction operations &amp; budget tracker</t>
         </is>
       </c>
       <c r="E288" s="9" t="inlineStr">
         <is>
-          <t>მოვალეებთან დაკავშირების ჭკვიანი რიგი (Predictive Queue)</t>
+          <t>სამშენებლო ოპერაციებისა და ბიუჯეტის მართვა</t>
         </is>
       </c>
       <c r="F288" s="9" t="inlineStr">
         <is>
-          <t>Умная очередь звонков должникам</t>
+          <t>Стройка: операции и бюджет</t>
         </is>
       </c>
       <c r="G288" s="3" t="inlineStr">
@@ -18430,22 +18464,22 @@
       </c>
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>ao.42</t>
+          <t>ao.41</t>
         </is>
       </c>
       <c r="D289" s="9" t="inlineStr">
         <is>
-          <t>Agent attendance tracker</t>
+          <t>Predictive debtor call queue</t>
         </is>
       </c>
       <c r="E289" s="9" t="inlineStr">
         <is>
-          <t>აგენტების/თანამშრომლების დასწრების აღრიცხვა</t>
+          <t>მოვალეებთან დაკავშირების ჭკვიანი რიგი (Predictive Queue)</t>
         </is>
       </c>
       <c r="F289" s="9" t="inlineStr">
         <is>
-          <t>Учёт посещаемости агентов</t>
+          <t>Умная очередь звонков должникам</t>
         </is>
       </c>
       <c r="G289" s="3" t="inlineStr">
@@ -18472,22 +18506,22 @@
       </c>
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>ao.43</t>
+          <t>ao.42</t>
         </is>
       </c>
       <c r="D290" s="9" t="inlineStr">
         <is>
-          <t>Round-robin appointment balancing</t>
+          <t>Agent attendance tracker</t>
         </is>
       </c>
       <c r="E290" s="9" t="inlineStr">
         <is>
-          <t>შეხვედრების თანაბარი როტაციული განაწილება (Round-robin)</t>
+          <t>აგენტების/თანამშრომლების დასწრების აღრიცხვა</t>
         </is>
       </c>
       <c r="F290" s="9" t="inlineStr">
         <is>
-          <t>Равномерное распределение встреч</t>
+          <t>Учёт посещаемости агентов</t>
         </is>
       </c>
       <c r="G290" s="3" t="inlineStr">
@@ -18514,39 +18548,81 @@
       </c>
       <c r="C291" s="3" t="inlineStr">
         <is>
+          <t>ao.43</t>
+        </is>
+      </c>
+      <c r="D291" s="9" t="inlineStr">
+        <is>
+          <t>Round-robin appointment balancing</t>
+        </is>
+      </c>
+      <c r="E291" s="9" t="inlineStr">
+        <is>
+          <t>შეხვედრების თანაბარი როტაციული განაწილება (Round-robin)</t>
+        </is>
+      </c>
+      <c r="F291" s="9" t="inlineStr">
+        <is>
+          <t>Равномерное распределение встреч</t>
+        </is>
+      </c>
+      <c r="G291" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H291" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="3" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B292" s="3" t="inlineStr">
+        <is>
+          <t>Ao</t>
+        </is>
+      </c>
+      <c r="C292" s="3" t="inlineStr">
+        <is>
           <t>ao.44</t>
         </is>
       </c>
-      <c r="D291" s="9" t="inlineStr">
+      <c r="D292" s="9" t="inlineStr">
         <is>
           <t>Discovery call auto-scheduling</t>
         </is>
       </c>
-      <c r="E291" s="9" t="inlineStr">
+      <c r="E292" s="9" t="inlineStr">
         <is>
           <t>Discovery ზარის ავტომატური დაჯავშნა</t>
         </is>
       </c>
-      <c r="F291" s="9" t="inlineStr">
+      <c r="F292" s="9" t="inlineStr">
         <is>
           <t>Автозапись на discovery-звонок</t>
         </is>
       </c>
-      <c r="G291" s="3" t="inlineStr">
+      <c r="G292" s="3" t="inlineStr">
         <is>
           <t>Only on this landing</t>
         </is>
       </c>
-      <c r="H291" s="3" t="inlineStr">
+      <c r="H292" s="3" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H291"/>
+  <autoFilter ref="A1:H292"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H490" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H491" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -18560,7 +18636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H284"/>
+  <dimension ref="A1:H285"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -19031,17 +19107,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -22459,17 +22535,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -23527,17 +23603,17 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>დარეკვა</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Позвонить</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr"/>
@@ -23793,17 +23869,17 @@
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G135" s="3" t="inlineStr"/>
@@ -26457,17 +26533,17 @@
       </c>
       <c r="D205" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E205" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F205" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G205" s="3" t="inlineStr"/>
@@ -29483,10 +29559,48 @@
         </is>
       </c>
     </row>
+    <row r="285">
+      <c r="A285" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B285" s="3" t="inlineStr">
+        <is>
+          <t>Nav</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>nav.cta</t>
+        </is>
+      </c>
+      <c r="D285" s="3" t="inlineStr">
+        <is>
+          <t>Free call</t>
+        </is>
+      </c>
+      <c r="E285" s="3" t="inlineStr">
+        <is>
+          <t>უფასო ზარი</t>
+        </is>
+      </c>
+      <c r="F285" s="3" t="inlineStr">
+        <is>
+          <t>Бесплатный звонок</t>
+        </is>
+      </c>
+      <c r="G285" s="3" t="inlineStr"/>
+      <c r="H285" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H284"/>
+  <autoFilter ref="A1:H285"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H483" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H484" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -29500,7 +29614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:H167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -29971,17 +30085,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -33399,17 +33513,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -34411,17 +34525,17 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>დარეკვა</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Позвонить</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr"/>
@@ -35817,17 +35931,17 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr"/>
@@ -35879,10 +35993,48 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>Banks</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>Nav</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>nav.cta</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>Free call</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>უფასო ზარი</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>Бесплатный звонок</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="inlineStr"/>
+      <c r="H167" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H166"/>
+  <autoFilter ref="A1:H167"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H365" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H366" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -35896,7 +36048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H177"/>
+  <dimension ref="A1:H178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.630000000000001" customWidth="1" style="6" min="2" max="2"/>
@@ -36208,7 +36360,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>კვლევას და ძიებას</t>
+          <t>კვლევას</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -36363,17 +36515,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr"/>
@@ -39783,17 +39935,17 @@
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr"/>
@@ -40779,17 +40931,17 @@
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>დარეკვა</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Позвонить</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr"/>
@@ -42185,17 +42337,17 @@
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Request a free 20-minute call</t>
+          <t>Request a free call</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>მოითხოვე 20-წუთიანი უფასო ზარი</t>
+          <t>მოითხოვე უფასო ზარი</t>
         </is>
       </c>
       <c r="F165" s="3" t="inlineStr">
         <is>
-          <t>Запросить бесплатный 20-минутный звонок</t>
+          <t>Запросить бесплатный звонок</t>
         </is>
       </c>
       <c r="G165" s="3" t="inlineStr"/>
@@ -42255,34 +42407,30 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>Prod</t>
+          <t>Nav</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>prod.title</t>
-        </is>
-      </c>
-      <c r="D167" s="9" t="inlineStr">
-        <is>
-          <t>Our own products</t>
-        </is>
-      </c>
-      <c r="E167" s="9" t="inlineStr">
-        <is>
-          <t>ჩვენი პროდუქტები</t>
-        </is>
-      </c>
-      <c r="F167" s="9" t="inlineStr">
-        <is>
-          <t>Наши продукты</t>
-        </is>
-      </c>
-      <c r="G167" s="3" t="inlineStr">
-        <is>
-          <t>Only on this landing</t>
-        </is>
-      </c>
+          <t>nav.cta</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>Free call</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>უფასო ზარი</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>Бесплатный звонок</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="inlineStr"/>
       <c r="H167" s="3" t="inlineStr">
         <is>
           <t>New</t>
@@ -42302,22 +42450,22 @@
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>prod.sub</t>
+          <t>prod.title</t>
         </is>
       </c>
       <c r="D168" s="9" t="inlineStr">
         <is>
-          <t>Ready-made services we built ourselves, quick to plug into your system.</t>
+          <t>Our own products</t>
         </is>
       </c>
       <c r="E168" s="9" t="inlineStr">
         <is>
-          <t>ჩვენ მიერ შექმნილი მზა გადაწყვეტები, რომლებიც სწრაფად და მარტივად ინტეგრირდება შენს სისტემაში.</t>
+          <t>ჩვენი პროდუქტები</t>
         </is>
       </c>
       <c r="F168" s="9" t="inlineStr">
         <is>
-          <t>Готовые сервисы, которые мы создали сами и быстро подключаем к вашей системе.</t>
+          <t>Наши продукты</t>
         </is>
       </c>
       <c r="G168" s="3" t="inlineStr">
@@ -42344,22 +42492,22 @@
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>prod.cta</t>
+          <t>prod.sub</t>
         </is>
       </c>
       <c r="D169" s="9" t="inlineStr">
         <is>
-          <t>Request →</t>
+          <t>Ready-made services we built ourselves, quick to plug into your system.</t>
         </is>
       </c>
       <c r="E169" s="9" t="inlineStr">
         <is>
-          <t>მოითხოვე →</t>
+          <t>ჩვენ მიერ შექმნილი მზა გადაწყვეტები, რომლებიც სწრაფად და მარტივად ინტეგრირდება შენს სისტემაში.</t>
         </is>
       </c>
       <c r="F169" s="9" t="inlineStr">
         <is>
-          <t>Запросить →</t>
+          <t>Готовые сервисы, которые мы создали сами и быстро подключаем к вашей системе.</t>
         </is>
       </c>
       <c r="G169" s="3" t="inlineStr">
@@ -42386,22 +42534,22 @@
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>prod.1.desc</t>
+          <t>prod.cta</t>
         </is>
       </c>
       <c r="D170" s="9" t="inlineStr">
         <is>
-          <t>Bank transactions (TBC, Bank of Georgia) flow into your CRM automatically - with payment matching and in-house installment schedules.</t>
+          <t>Request →</t>
         </is>
       </c>
       <c r="E170" s="9" t="inlineStr">
         <is>
-          <t>საბანკო ტრანზაქციები (TBC, საქართველოს ბანკი) ავტომატურად ისახება CRM-ში — გადახდების შეჯერებითა და შიდა განვადების გრაფიკით.</t>
+          <t>მოითხოვე →</t>
         </is>
       </c>
       <c r="F170" s="9" t="inlineStr">
         <is>
-          <t>Транзакции банков (TBC, Банк Грузии) автоматически попадают в CRM - с привязкой платежей и графиком внутренней рассрочки.</t>
+          <t>Запросить →</t>
         </is>
       </c>
       <c r="G170" s="3" t="inlineStr">
@@ -42428,22 +42576,22 @@
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>prod.2.desc</t>
+          <t>prod.1.desc</t>
         </is>
       </c>
       <c r="D171" s="9" t="inlineStr">
         <is>
-          <t>An AI chat assistant on your website: answers questions 24/7 and writes leads straight into your CRM.</t>
+          <t>Bank transactions (TBC, Bank of Georgia) flow into your CRM automatically - with payment matching and in-house installment schedules.</t>
         </is>
       </c>
       <c r="E171" s="9" t="inlineStr">
         <is>
-          <t>AI ჩატ-ასისტენტი შენს საიტზე: 24/7 პასუხობს შეკითხვებს და ლიდებს პირდაპირ CRM-ში აღრიცხავს.</t>
+          <t>საბანკო ტრანზაქციები (TBC, საქართველოს ბანკი) ავტომატურად ისახება CRM-ში — გადახდების შეჯერებითა და შიდა განვადების გრაფიკით.</t>
         </is>
       </c>
       <c r="F171" s="9" t="inlineStr">
         <is>
-          <t>AI-чат-ассистент на вашем сайте: отвечает на вопросы 24/7 и записывает лиды прямо в CRM.</t>
+          <t>Транзакции банков (TBC, Банк Грузии) автоматически попадают в CRM - с привязкой платежей и графиком внутренней рассрочки.</t>
         </is>
       </c>
       <c r="G171" s="3" t="inlineStr">
@@ -42470,22 +42618,22 @@
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>prod.3.desc</t>
+          <t>prod.2.desc</t>
         </is>
       </c>
       <c r="D172" s="9" t="inlineStr">
         <is>
-          <t>Transcription of Georgian-language meetings, a short summary and next steps - automatically.</t>
+          <t>An AI chat assistant on your website: answers questions 24/7 and writes leads straight into your CRM.</t>
         </is>
       </c>
       <c r="E172" s="9" t="inlineStr">
         <is>
-          <t>ქართულენოვანი შეხვედრების ტრანსკრიფცია, მოკლე შეჯამება და სამოქმედო ნაბიჯები — სრულად ავტომატურად.</t>
+          <t>AI ჩატ-ასისტენტი შენს საიტზე: 24/7 პასუხობს შეკითხვებს და ლიდებს პირდაპირ CRM-ში აღრიცხავს.</t>
         </is>
       </c>
       <c r="F172" s="9" t="inlineStr">
         <is>
-          <t>Расшифровка встреч на грузинском, краткое резюме и следующие шаги - автоматически.</t>
+          <t>AI-чат-ассистент на вашем сайте: отвечает на вопросы 24/7 и записывает лиды прямо в CRM.</t>
         </is>
       </c>
       <c r="G172" s="3" t="inlineStr">
@@ -42512,22 +42660,22 @@
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>prod.4.desc</t>
+          <t>prod.3.desc</t>
         </is>
       </c>
       <c r="D173" s="9" t="inlineStr">
         <is>
-          <t>Claude connected to your data: ask in plain language and get answers in numbers.</t>
+          <t>Transcription of Georgian-language meetings, a short summary and next steps - automatically.</t>
         </is>
       </c>
       <c r="E173" s="9" t="inlineStr">
         <is>
-          <t>Claude დაკავშირებული შენს მონაცემებთან: დასვი კითხვა მარტივ ენაზე და მიიღე ზუსტი პასუხები ციფრებში.</t>
+          <t>ქართულენოვანი შეხვედრების ტრანსკრიფცია, მოკლე შეჯამება და სამოქმედო ნაბიჯები — სრულად ავტომატურად.</t>
         </is>
       </c>
       <c r="F173" s="9" t="inlineStr">
         <is>
-          <t>Claude, подключённый к вашим данным: спрашивайте обычным языком и получайте ответы в цифрах.</t>
+          <t>Расшифровка встреч на грузинском, краткое резюме и следующие шаги - автоматически.</t>
         </is>
       </c>
       <c r="G173" s="3" t="inlineStr">
@@ -42554,22 +42702,22 @@
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>prod.5.desc</t>
+          <t>prod.4.desc</t>
         </is>
       </c>
       <c r="D174" s="9" t="inlineStr">
         <is>
-          <t>Calls, recordings and click-to-call right inside your CRM - with routing to the right manager.</t>
+          <t>Claude connected to your data: ask in plain language and get answers in numbers.</t>
         </is>
       </c>
       <c r="E174" s="9" t="inlineStr">
         <is>
-          <t>ზარები, აუდიოჩანაწერები და click-to-call პირდაპირ CRM-ში — ზარის შესაბამის მენეჯერზე ჭკვიანი გადამისამართებით.</t>
+          <t>Claude დაკავშირებული შენს მონაცემებთან: დასვი კითხვა მარტივ ენაზე და მიიღე ზუსტი პასუხები ციფრებში.</t>
         </is>
       </c>
       <c r="F174" s="9" t="inlineStr">
         <is>
-          <t>Звонки, записи и click-to-call прямо в CRM - с маршрутизацией на нужного менеджера.</t>
+          <t>Claude, подключённый к вашим данным: спрашивайте обычным языком и получайте ответы в цифрах.</t>
         </is>
       </c>
       <c r="G174" s="3" t="inlineStr">
@@ -42596,22 +42744,22 @@
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>prod.6.desc</t>
+          <t>prod.5.desc</t>
         </is>
       </c>
       <c r="D175" s="9" t="inlineStr">
         <is>
-          <t>Every new lead is processed automatically: contact created, duplicates found, owner assigned.</t>
+          <t>Calls, recordings and click-to-call right inside your CRM - with routing to the right manager.</t>
         </is>
       </c>
       <c r="E175" s="9" t="inlineStr">
         <is>
-          <t>ყოველი ახალი ლიდი მუშავდება ავტომატურად: კონტაქტის შექმნა, დუბლიკატების პრევენცია და პასუხისმგებელი მენეჯერის მინიჭება.</t>
+          <t>ზარები, აუდიოჩანაწერები და click-to-call პირდაპირ CRM-ში — ზარის შესაბამის მენეჯერზე ჭკვიანი გადამისამართებით.</t>
         </is>
       </c>
       <c r="F175" s="9" t="inlineStr">
         <is>
-          <t>Каждый новый лид обрабатывается автоматически: создание контакта, поиск дублей, назначение менеджера.</t>
+          <t>Звонки, записи и click-to-call прямо в CRM - с маршрутизацией на нужного менеджера.</t>
         </is>
       </c>
       <c r="G175" s="3" t="inlineStr">
@@ -42638,22 +42786,22 @@
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>prod.7.desc</t>
+          <t>prod.6.desc</t>
         </is>
       </c>
       <c r="D176" s="9" t="inlineStr">
         <is>
-          <t>Partners submit leads in one place and see their status, while you get the full history of every referral.</t>
+          <t>Every new lead is processed automatically: contact created, duplicates found, owner assigned.</t>
         </is>
       </c>
       <c r="E176" s="9" t="inlineStr">
         <is>
-          <t>პარტნიორები ლიდებს ერთიან პორტალში აგზავნიან და ხედავენ სტატუსებს, შენ კი იღებ თითოეული რეკომენდაციის სრულ ისტორიას.</t>
+          <t>ყოველი ახალი ლიდი მუშავდება ავტომატურად: კონტაქტის შექმნა, დუბლიკატების პრევენცია და პასუხისმგებელი მენეჯერის მინიჭება.</t>
         </is>
       </c>
       <c r="F176" s="9" t="inlineStr">
         <is>
-          <t>Партнёры отправляют лиды в одном месте и видят их статус, а вы - полную историю каждой рекомендации.</t>
+          <t>Каждый новый лид обрабатывается автоматически: создание контакта, поиск дублей, назначение менеджера.</t>
         </is>
       </c>
       <c r="G176" s="3" t="inlineStr">
@@ -42680,39 +42828,81 @@
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
+          <t>prod.7.desc</t>
+        </is>
+      </c>
+      <c r="D177" s="9" t="inlineStr">
+        <is>
+          <t>Partners submit leads in one place and see their status, while you get the full history of every referral.</t>
+        </is>
+      </c>
+      <c r="E177" s="9" t="inlineStr">
+        <is>
+          <t>პარტნიორები ლიდებს ერთიან პორტალში აგზავნიან და ხედავენ სტატუსებს, შენ კი იღებ თითოეული რეკომენდაციის სრულ ისტორიას.</t>
+        </is>
+      </c>
+      <c r="F177" s="9" t="inlineStr">
+        <is>
+          <t>Партнёры отправляют лиды в одном месте и видят их статус, а вы - полную историю каждой рекомендации.</t>
+        </is>
+      </c>
+      <c r="G177" s="3" t="inlineStr">
+        <is>
+          <t>Only on this landing</t>
+        </is>
+      </c>
+      <c r="H177" s="3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>Solutions</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>Prod</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
           <t>prod.8.desc</t>
         </is>
       </c>
-      <c r="D177" s="9" t="inlineStr">
+      <c r="D178" s="9" t="inlineStr">
         <is>
           <t>Personalised SMS reminders and notifications straight from your CRM - for payments, meetings and bookings.</t>
         </is>
       </c>
-      <c r="E177" s="9" t="inlineStr">
+      <c r="E178" s="9" t="inlineStr">
         <is>
           <t>პერსონალიზებული SMS შეხსენებები და შეტყობინებები პირდაპირ CRM-იდან — გადახდებზე, შეხვედრებსა და ჯავშნებზე.</t>
         </is>
       </c>
-      <c r="F177" s="9" t="inlineStr">
+      <c r="F178" s="9" t="inlineStr">
         <is>
           <t>Персональные SMS-напоминания и уведомления прямо из CRM - о платежах, встречах и бронях.</t>
         </is>
       </c>
-      <c r="G177" s="3" t="inlineStr">
+      <c r="G178" s="3" t="inlineStr">
         <is>
           <t>Only on this landing</t>
         </is>
       </c>
-      <c r="H177" s="3" t="inlineStr">
+      <c r="H178" s="3" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H177"/>
+  <autoFilter ref="A1:H178"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H376" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H377" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Updated,New,Changed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -43793,17 +43983,17 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Call</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>დარეკვა</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Позвонить</t>
+          <t>+995 32 205 50 60</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">

</xml_diff>